<commit_message>
fix: normalizar bordes eliminando recuadro negro en Toluca y Morelos del reporte diario
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -200,7 +200,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -568,13 +568,14 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -800,8 +801,20 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3642,29 +3655,29 @@
           <t>AAA</t>
         </is>
       </c>
-      <c r="B26" s="74" t="n"/>
-      <c r="C26" s="75" t="inlineStr">
+      <c r="B26" s="49" t="n"/>
+      <c r="C26" s="48" t="inlineStr">
         <is>
           <t>VALLE-SAN JUAN</t>
         </is>
       </c>
-      <c r="D26" s="76" t="inlineStr">
+      <c r="D26" s="33" t="inlineStr">
         <is>
           <t>EULEN</t>
         </is>
       </c>
-      <c r="E26" s="77" t="n">
+      <c r="E26" s="13" t="n">
         <v>363</v>
       </c>
-      <c r="F26" s="77" t="n">
+      <c r="F26" s="13" t="n">
         <v>32</v>
       </c>
-      <c r="G26" s="77" t="n"/>
-      <c r="H26" s="77" t="n">
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="I26" s="77" t="n"/>
-      <c r="J26" s="77" t="n">
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n">
         <v>396</v>
       </c>
       <c r="L26" s="3" t="n"/>
@@ -3778,142 +3791,139 @@
           <t>AAA</t>
         </is>
       </c>
-      <c r="B27" s="81" t="inlineStr">
+      <c r="B27" s="49" t="inlineStr">
         <is>
           <t>MORELOS</t>
         </is>
       </c>
-      <c r="C27" s="82" t="inlineStr">
+      <c r="C27" s="48" t="inlineStr">
         <is>
           <t>MORELOS</t>
         </is>
       </c>
-      <c r="D27" s="72" t="inlineStr">
+      <c r="D27" s="33" t="inlineStr">
         <is>
           <t>IASA</t>
         </is>
       </c>
-      <c r="E27" s="83" t="n">
+      <c r="E27" s="13" t="n">
         <v>2353</v>
       </c>
-      <c r="F27" s="83" t="n">
+      <c r="F27" s="13" t="n">
         <v>312</v>
       </c>
-      <c r="G27" s="83" t="n"/>
-      <c r="H27" s="83" t="n"/>
-      <c r="I27" s="83" t="n"/>
-      <c r="J27" s="83" t="n">
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n">
         <v>2665</v>
       </c>
-      <c r="K27" s="67" t="n"/>
       <c r="L27" s="3" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
       <c r="O27" s="3" t="n"/>
       <c r="P27" s="3" t="n"/>
-      <c r="R27" s="84" t="n">
+      <c r="R27" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="S27" s="85" t="n"/>
-      <c r="T27" s="86" t="n">
+      <c r="S27" s="15" t="n"/>
+      <c r="T27" s="16" t="n">
         <v>126</v>
       </c>
-      <c r="U27" s="86" t="n">
+      <c r="U27" s="16" t="n">
         <v>756</v>
       </c>
-      <c r="V27" s="72" t="n"/>
-      <c r="W27" s="87" t="n"/>
-      <c r="X27" s="87" t="n"/>
-      <c r="Y27" s="87" t="n"/>
-      <c r="Z27" s="87" t="n"/>
-      <c r="AA27" s="87" t="n"/>
-      <c r="AB27" s="87" t="n"/>
-      <c r="AC27" s="87" t="n"/>
-      <c r="AD27" s="87" t="n">
+      <c r="W27" s="24" t="n"/>
+      <c r="X27" s="24" t="n"/>
+      <c r="Y27" s="24" t="n"/>
+      <c r="Z27" s="24" t="n"/>
+      <c r="AA27" s="24" t="n"/>
+      <c r="AB27" s="24" t="n"/>
+      <c r="AC27" s="24" t="n"/>
+      <c r="AD27" s="24" t="n">
         <v>31</v>
       </c>
-      <c r="AE27" s="87" t="n"/>
-      <c r="AF27" s="87" t="n"/>
-      <c r="AG27" s="87" t="n"/>
-      <c r="AH27" s="87" t="n"/>
-      <c r="AI27" s="87" t="n"/>
-      <c r="AJ27" s="87" t="n"/>
-      <c r="AK27" s="87" t="n"/>
-      <c r="AL27" s="87" t="n"/>
-      <c r="AM27" s="87" t="n"/>
-      <c r="AN27" s="87" t="n"/>
-      <c r="AO27" s="87" t="n"/>
-      <c r="AP27" s="87" t="n"/>
-      <c r="AQ27" s="87" t="n"/>
-      <c r="AR27" s="87" t="n"/>
-      <c r="AS27" s="87" t="n"/>
-      <c r="AT27" s="87" t="n"/>
-      <c r="AU27" s="87" t="n"/>
-      <c r="AV27" s="87" t="n"/>
-      <c r="AW27" s="87" t="n"/>
-      <c r="AX27" s="87" t="n"/>
-      <c r="AY27" s="87" t="n"/>
-      <c r="AZ27" s="87" t="n"/>
-      <c r="BA27" s="87" t="n"/>
-      <c r="BB27" s="87" t="n"/>
-      <c r="BC27" s="87" t="n"/>
-      <c r="BD27" s="87" t="n"/>
-      <c r="BE27" s="87" t="n"/>
-      <c r="BF27" s="87" t="n"/>
-      <c r="BG27" s="87" t="n"/>
-      <c r="BH27" s="87" t="n"/>
-      <c r="BI27" s="87" t="n"/>
-      <c r="BJ27" s="87" t="n"/>
-      <c r="BK27" s="87" t="n"/>
-      <c r="BL27" s="87" t="n"/>
-      <c r="BM27" s="87" t="n"/>
-      <c r="BN27" s="87" t="n"/>
-      <c r="BO27" s="87" t="n"/>
-      <c r="BP27" s="87" t="n"/>
-      <c r="BQ27" s="87" t="n"/>
-      <c r="BR27" s="87" t="n"/>
-      <c r="BS27" s="87" t="n"/>
-      <c r="BT27" s="87" t="n"/>
-      <c r="BU27" s="87" t="n"/>
-      <c r="BV27" s="87" t="n"/>
-      <c r="BW27" s="87" t="n"/>
-      <c r="BX27" s="87" t="n"/>
-      <c r="BY27" s="87" t="n"/>
-      <c r="BZ27" s="87" t="n"/>
-      <c r="CA27" s="87" t="n"/>
-      <c r="CB27" s="87" t="n"/>
-      <c r="CC27" s="87" t="n"/>
-      <c r="CD27" s="87" t="n"/>
-      <c r="CE27" s="87" t="n"/>
-      <c r="CF27" s="87" t="n"/>
-      <c r="CG27" s="87" t="n"/>
-      <c r="CH27" s="87" t="n"/>
-      <c r="CI27" s="87" t="n"/>
-      <c r="CJ27" s="87" t="n"/>
-      <c r="CK27" s="87" t="n"/>
-      <c r="CL27" s="87" t="n"/>
-      <c r="CM27" s="87" t="n"/>
-      <c r="CN27" s="88">
+      <c r="AE27" s="24" t="n"/>
+      <c r="AF27" s="24" t="n"/>
+      <c r="AG27" s="24" t="n"/>
+      <c r="AH27" s="24" t="n"/>
+      <c r="AI27" s="24" t="n"/>
+      <c r="AJ27" s="24" t="n"/>
+      <c r="AK27" s="24" t="n"/>
+      <c r="AL27" s="24" t="n"/>
+      <c r="AM27" s="24" t="n"/>
+      <c r="AN27" s="24" t="n"/>
+      <c r="AO27" s="24" t="n"/>
+      <c r="AP27" s="24" t="n"/>
+      <c r="AQ27" s="24" t="n"/>
+      <c r="AR27" s="24" t="n"/>
+      <c r="AS27" s="24" t="n"/>
+      <c r="AT27" s="24" t="n"/>
+      <c r="AU27" s="24" t="n"/>
+      <c r="AV27" s="24" t="n"/>
+      <c r="AW27" s="24" t="n"/>
+      <c r="AX27" s="24" t="n"/>
+      <c r="AY27" s="24" t="n"/>
+      <c r="AZ27" s="24" t="n"/>
+      <c r="BA27" s="24" t="n"/>
+      <c r="BB27" s="24" t="n"/>
+      <c r="BC27" s="24" t="n"/>
+      <c r="BD27" s="24" t="n"/>
+      <c r="BE27" s="24" t="n"/>
+      <c r="BF27" s="24" t="n"/>
+      <c r="BG27" s="24" t="n"/>
+      <c r="BH27" s="24" t="n"/>
+      <c r="BI27" s="24" t="n"/>
+      <c r="BJ27" s="24" t="n"/>
+      <c r="BK27" s="24" t="n"/>
+      <c r="BL27" s="24" t="n"/>
+      <c r="BM27" s="24" t="n"/>
+      <c r="BN27" s="24" t="n"/>
+      <c r="BO27" s="24" t="n"/>
+      <c r="BP27" s="24" t="n"/>
+      <c r="BQ27" s="24" t="n"/>
+      <c r="BR27" s="24" t="n"/>
+      <c r="BS27" s="24" t="n"/>
+      <c r="BT27" s="24" t="n"/>
+      <c r="BU27" s="24" t="n"/>
+      <c r="BV27" s="24" t="n"/>
+      <c r="BW27" s="24" t="n"/>
+      <c r="BX27" s="24" t="n"/>
+      <c r="BY27" s="24" t="n"/>
+      <c r="BZ27" s="24" t="n"/>
+      <c r="CA27" s="24" t="n"/>
+      <c r="CB27" s="24" t="n"/>
+      <c r="CC27" s="24" t="n"/>
+      <c r="CD27" s="24" t="n"/>
+      <c r="CE27" s="24" t="n"/>
+      <c r="CF27" s="24" t="n"/>
+      <c r="CG27" s="24" t="n"/>
+      <c r="CH27" s="24" t="n"/>
+      <c r="CI27" s="24" t="n"/>
+      <c r="CJ27" s="24" t="n"/>
+      <c r="CK27" s="24" t="n"/>
+      <c r="CL27" s="24" t="n"/>
+      <c r="CM27" s="24" t="n"/>
+      <c r="CN27" s="37">
         <f>+SUM(W27:CM27)</f>
         <v/>
       </c>
-      <c r="CO27" s="72" t="n"/>
-      <c r="CP27" s="89" t="n">
+      <c r="CP27" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="CQ27" s="90" t="n">
-        <v>0</v>
-      </c>
-      <c r="CR27" s="90" t="n">
+      <c r="CQ27" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR27" s="22" t="n">
         <v>31</v>
       </c>
-      <c r="CS27" s="91" t="n"/>
-      <c r="CT27" s="113" t="n"/>
-      <c r="CU27" s="93" t="n">
+      <c r="CS27" s="42" t="n"/>
+      <c r="CT27" s="111" t="n"/>
+      <c r="CU27" s="32" t="n">
         <v>618</v>
       </c>
-      <c r="CV27" s="83" t="n"/>
-      <c r="CW27" s="94" t="n"/>
+      <c r="CV27" s="14" t="n"/>
+      <c r="CW27" s="14" t="n"/>
       <c r="CX27" s="112" t="n"/>
       <c r="CY27" s="17" t="n"/>
     </row>
@@ -3923,33 +3933,33 @@
           <t>AAA</t>
         </is>
       </c>
-      <c r="B28" s="60" t="inlineStr">
+      <c r="B28" s="49" t="inlineStr">
         <is>
           <t>TOLUCA</t>
         </is>
       </c>
-      <c r="C28" s="78" t="inlineStr">
+      <c r="C28" s="48" t="inlineStr">
         <is>
           <t>TOLUCA</t>
         </is>
       </c>
-      <c r="D28" s="79" t="inlineStr">
+      <c r="D28" s="33" t="inlineStr">
         <is>
           <t>IASA</t>
         </is>
       </c>
-      <c r="E28" s="80" t="n">
+      <c r="E28" s="13" t="n">
         <v>1107</v>
       </c>
-      <c r="F28" s="80" t="n">
+      <c r="F28" s="13" t="n">
         <v>270</v>
       </c>
-      <c r="G28" s="80" t="n">
+      <c r="G28" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="80" t="n"/>
-      <c r="I28" s="80" t="n"/>
-      <c r="J28" s="80" t="n">
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n">
         <v>1378</v>
       </c>
       <c r="L28" s="3" t="n"/>
@@ -14879,56 +14889,56 @@
       <c r="CS26" s="17" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A27" s="76" t="inlineStr">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="B27" s="59" t="inlineStr">
+      <c r="B27" s="50" t="inlineStr">
         <is>
           <t>MORELOS</t>
         </is>
       </c>
-      <c r="C27" s="95" t="inlineStr">
+      <c r="C27" s="57" t="inlineStr">
         <is>
           <t>MORELOS</t>
         </is>
       </c>
-      <c r="D27" s="76" t="inlineStr">
+      <c r="D27" s="33" t="inlineStr">
         <is>
           <t>EULEN</t>
         </is>
       </c>
-      <c r="E27" s="77" t="n">
+      <c r="E27" s="13" t="n">
         <v>74</v>
       </c>
-      <c r="F27" s="77" t="n">
+      <c r="F27" s="13" t="n">
         <v>91</v>
       </c>
-      <c r="G27" s="77" t="n"/>
-      <c r="H27" s="77" t="n">
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="I27" s="77" t="n">
+      <c r="I27" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="J27" s="77" t="n">
+      <c r="J27" s="13" t="n">
         <v>581</v>
       </c>
-      <c r="K27" s="77" t="n">
+      <c r="K27" s="13" t="n">
         <v>816</v>
       </c>
-      <c r="L27" s="77" t="n">
+      <c r="L27" s="13" t="n">
         <v>53</v>
       </c>
-      <c r="M27" s="77" t="n">
+      <c r="M27" s="13" t="n">
         <v>35</v>
       </c>
-      <c r="N27" s="77" t="n">
+      <c r="N27" s="13" t="n">
         <v>219</v>
       </c>
-      <c r="O27" s="77" t="n"/>
-      <c r="P27" s="77" t="n">
+      <c r="O27" s="13" t="n"/>
+      <c r="P27" s="13" t="n">
         <v>1892</v>
       </c>
       <c r="R27" s="3" t="n"/>
@@ -15029,207 +15039,205 @@
       <c r="CS27" s="17" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" thickBot="1">
-      <c r="A28" s="97" t="inlineStr">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="B28" s="98" t="inlineStr">
+      <c r="B28" s="50" t="inlineStr">
         <is>
           <t>TOLUCA</t>
         </is>
       </c>
-      <c r="C28" s="99" t="inlineStr">
+      <c r="C28" s="57" t="inlineStr">
         <is>
           <t>TOLUCA</t>
         </is>
       </c>
-      <c r="D28" s="72" t="inlineStr">
+      <c r="D28" s="33" t="inlineStr">
         <is>
           <t>IASA</t>
         </is>
       </c>
-      <c r="E28" s="83" t="n">
+      <c r="E28" s="13" t="n">
         <v>67</v>
       </c>
-      <c r="F28" s="83" t="n">
+      <c r="F28" s="13" t="n">
         <v>38</v>
       </c>
-      <c r="G28" s="83" t="n"/>
-      <c r="H28" s="83" t="n">
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="I28" s="83" t="n">
+      <c r="I28" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="J28" s="83" t="n">
+      <c r="J28" s="13" t="n">
         <v>642</v>
       </c>
-      <c r="K28" s="83" t="n">
+      <c r="K28" s="13" t="n">
         <v>1135</v>
       </c>
-      <c r="L28" s="83" t="n">
+      <c r="L28" s="13" t="n">
         <v>17</v>
       </c>
-      <c r="M28" s="83" t="n">
+      <c r="M28" s="13" t="n">
         <v>27</v>
       </c>
-      <c r="N28" s="83" t="n">
+      <c r="N28" s="13" t="n">
         <v>97</v>
       </c>
-      <c r="O28" s="83" t="n"/>
-      <c r="P28" s="83" t="n">
+      <c r="O28" s="13" t="n"/>
+      <c r="P28" s="13" t="n">
         <v>2030</v>
       </c>
-      <c r="Q28" s="67" t="n"/>
       <c r="R28" s="3" t="n"/>
       <c r="S28" s="3" t="n"/>
       <c r="T28" s="3" t="n"/>
       <c r="U28" s="3" t="n"/>
       <c r="V28" s="3" t="n"/>
-      <c r="X28" s="84" t="n">
+      <c r="X28" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="Y28" s="85" t="n"/>
-      <c r="Z28" s="86" t="n">
+      <c r="Y28" s="15" t="n"/>
+      <c r="Z28" s="16" t="n">
         <v>90</v>
       </c>
-      <c r="AA28" s="86" t="n">
+      <c r="AA28" s="16" t="n">
         <v>540</v>
       </c>
-      <c r="AB28" s="70" t="n"/>
-      <c r="AC28" s="87" t="n"/>
-      <c r="AD28" s="87" t="n"/>
-      <c r="AE28" s="87" t="n"/>
-      <c r="AF28" s="87" t="n"/>
-      <c r="AG28" s="87" t="n"/>
-      <c r="AH28" s="87" t="n"/>
-      <c r="AI28" s="87" t="n"/>
-      <c r="AJ28" s="87" t="n">
+      <c r="AB28" s="6" t="n"/>
+      <c r="AC28" s="24" t="n"/>
+      <c r="AD28" s="24" t="n"/>
+      <c r="AE28" s="24" t="n"/>
+      <c r="AF28" s="24" t="n"/>
+      <c r="AG28" s="24" t="n"/>
+      <c r="AH28" s="24" t="n"/>
+      <c r="AI28" s="24" t="n"/>
+      <c r="AJ28" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="AK28" s="87" t="n"/>
-      <c r="AL28" s="87" t="n"/>
-      <c r="AM28" s="87" t="n"/>
-      <c r="AN28" s="87" t="n"/>
-      <c r="AO28" s="87" t="n"/>
-      <c r="AP28" s="87" t="n"/>
-      <c r="AQ28" s="87" t="n"/>
-      <c r="AR28" s="87" t="n"/>
-      <c r="AS28" s="87" t="n"/>
-      <c r="AT28" s="87" t="n"/>
-      <c r="AU28" s="87" t="n"/>
-      <c r="AV28" s="87" t="n"/>
-      <c r="AW28" s="87" t="n"/>
-      <c r="AX28" s="87" t="n"/>
-      <c r="AY28" s="87" t="n"/>
-      <c r="AZ28" s="87" t="n"/>
-      <c r="BA28" s="87" t="n"/>
-      <c r="BB28" s="87" t="n"/>
-      <c r="BC28" s="87" t="n"/>
-      <c r="BD28" s="87" t="n"/>
-      <c r="BE28" s="87" t="n"/>
-      <c r="BF28" s="87" t="n"/>
-      <c r="BG28" s="87" t="n"/>
-      <c r="BH28" s="87" t="n"/>
-      <c r="BI28" s="87" t="n"/>
-      <c r="BJ28" s="87" t="n"/>
-      <c r="BK28" s="87" t="n"/>
-      <c r="BL28" s="87" t="n"/>
-      <c r="BM28" s="87" t="n"/>
-      <c r="BN28" s="87" t="n"/>
-      <c r="BO28" s="87" t="n"/>
-      <c r="BP28" s="87" t="n"/>
-      <c r="BQ28" s="87" t="n"/>
-      <c r="BR28" s="87" t="n"/>
-      <c r="BS28" s="87" t="n"/>
-      <c r="BT28" s="87" t="n"/>
-      <c r="BU28" s="87" t="n"/>
-      <c r="BV28" s="87" t="n"/>
-      <c r="BW28" s="87" t="n"/>
-      <c r="BX28" s="87" t="n"/>
-      <c r="BY28" s="87" t="n"/>
-      <c r="BZ28" s="87" t="n"/>
-      <c r="CA28" s="87" t="n"/>
-      <c r="CB28" s="87" t="n"/>
-      <c r="CC28" s="87" t="n"/>
-      <c r="CD28" s="87" t="n"/>
-      <c r="CE28" s="87" t="n"/>
-      <c r="CF28" s="87" t="n"/>
-      <c r="CG28" s="87" t="n"/>
-      <c r="CH28" s="88">
+      <c r="AK28" s="24" t="n"/>
+      <c r="AL28" s="24" t="n"/>
+      <c r="AM28" s="24" t="n"/>
+      <c r="AN28" s="24" t="n"/>
+      <c r="AO28" s="24" t="n"/>
+      <c r="AP28" s="24" t="n"/>
+      <c r="AQ28" s="24" t="n"/>
+      <c r="AR28" s="24" t="n"/>
+      <c r="AS28" s="24" t="n"/>
+      <c r="AT28" s="24" t="n"/>
+      <c r="AU28" s="24" t="n"/>
+      <c r="AV28" s="24" t="n"/>
+      <c r="AW28" s="24" t="n"/>
+      <c r="AX28" s="24" t="n"/>
+      <c r="AY28" s="24" t="n"/>
+      <c r="AZ28" s="24" t="n"/>
+      <c r="BA28" s="24" t="n"/>
+      <c r="BB28" s="24" t="n"/>
+      <c r="BC28" s="24" t="n"/>
+      <c r="BD28" s="24" t="n"/>
+      <c r="BE28" s="24" t="n"/>
+      <c r="BF28" s="24" t="n"/>
+      <c r="BG28" s="24" t="n"/>
+      <c r="BH28" s="24" t="n"/>
+      <c r="BI28" s="24" t="n"/>
+      <c r="BJ28" s="24" t="n"/>
+      <c r="BK28" s="24" t="n"/>
+      <c r="BL28" s="24" t="n"/>
+      <c r="BM28" s="24" t="n"/>
+      <c r="BN28" s="24" t="n"/>
+      <c r="BO28" s="24" t="n"/>
+      <c r="BP28" s="24" t="n"/>
+      <c r="BQ28" s="24" t="n"/>
+      <c r="BR28" s="24" t="n"/>
+      <c r="BS28" s="24" t="n"/>
+      <c r="BT28" s="24" t="n"/>
+      <c r="BU28" s="24" t="n"/>
+      <c r="BV28" s="24" t="n"/>
+      <c r="BW28" s="24" t="n"/>
+      <c r="BX28" s="24" t="n"/>
+      <c r="BY28" s="24" t="n"/>
+      <c r="BZ28" s="24" t="n"/>
+      <c r="CA28" s="24" t="n"/>
+      <c r="CB28" s="24" t="n"/>
+      <c r="CC28" s="24" t="n"/>
+      <c r="CD28" s="24" t="n"/>
+      <c r="CE28" s="24" t="n"/>
+      <c r="CF28" s="24" t="n"/>
+      <c r="CG28" s="24" t="n"/>
+      <c r="CH28" s="37">
         <f>+SUM(AC28:CG28)</f>
         <v/>
       </c>
-      <c r="CI28" s="72" t="n"/>
-      <c r="CJ28" s="89" t="n">
+      <c r="CJ28" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="CK28" s="90" t="n"/>
-      <c r="CL28" s="90" t="n">
+      <c r="CK28" s="22" t="n"/>
+      <c r="CL28" s="22" t="n">
         <v>13</v>
       </c>
-      <c r="CM28" s="91" t="n"/>
-      <c r="CN28" s="113" t="n"/>
-      <c r="CO28" s="100" t="n">
+      <c r="CM28" s="42" t="n"/>
+      <c r="CN28" s="111" t="n"/>
+      <c r="CO28" s="32" t="n">
         <v>100</v>
       </c>
-      <c r="CP28" s="83" t="n"/>
-      <c r="CQ28" s="94" t="n"/>
+      <c r="CP28" s="14" t="n"/>
+      <c r="CQ28" s="14" t="n"/>
       <c r="CR28" s="112" t="n"/>
       <c r="CS28" s="17" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="79" t="n">
+      <c r="A29" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="B29" s="61" t="inlineStr">
+      <c r="B29" s="50" t="inlineStr">
         <is>
           <t>GUADALAJARA</t>
         </is>
       </c>
-      <c r="C29" s="96" t="inlineStr">
+      <c r="C29" s="57" t="inlineStr">
         <is>
           <t>GUADALAJARA CENTRO</t>
         </is>
       </c>
-      <c r="D29" s="79" t="inlineStr">
+      <c r="D29" s="33" t="inlineStr">
         <is>
           <t>IASA</t>
         </is>
       </c>
-      <c r="E29" s="80" t="n">
+      <c r="E29" s="13" t="n">
         <v>22</v>
       </c>
-      <c r="F29" s="80" t="n">
+      <c r="F29" s="13" t="n">
         <v>240</v>
       </c>
-      <c r="G29" s="80" t="n">
+      <c r="G29" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="H29" s="80" t="n">
+      <c r="H29" s="13" t="n">
         <v>92</v>
       </c>
-      <c r="I29" s="80" t="n">
+      <c r="I29" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="J29" s="80" t="n">
+      <c r="J29" s="13" t="n">
         <v>134</v>
       </c>
-      <c r="K29" s="80" t="n">
+      <c r="K29" s="13" t="n">
         <v>851</v>
       </c>
-      <c r="L29" s="80" t="n">
+      <c r="L29" s="13" t="n">
         <v>954</v>
       </c>
-      <c r="M29" s="80" t="n">
+      <c r="M29" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="N29" s="80" t="n">
+      <c r="N29" s="13" t="n">
         <v>116</v>
       </c>
-      <c r="O29" s="80" t="n"/>
-      <c r="P29" s="80" t="n">
+      <c r="O29" s="13" t="n"/>
+      <c r="P29" s="13" t="n">
         <v>2417</v>
       </c>
       <c r="R29" s="3" t="n"/>
@@ -22105,114 +22113,118 @@
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A78" s="31" t="n"/>
-      <c r="B78" s="64" t="inlineStr">
+      <c r="A78" s="113" t="n"/>
+      <c r="B78" s="113" t="inlineStr">
         <is>
           <t>MORELOS</t>
         </is>
       </c>
-      <c r="C78" s="65" t="inlineStr">
+      <c r="C78" s="113" t="inlineStr">
         <is>
           <t>MORELOS</t>
         </is>
       </c>
-      <c r="D78" s="65" t="inlineStr">
+      <c r="D78" s="113" t="inlineStr">
         <is>
           <t>IASA</t>
         </is>
       </c>
-      <c r="E78" s="66" t="n"/>
-      <c r="F78" s="66" t="n"/>
-      <c r="G78" s="66" t="n"/>
-      <c r="H78" s="66" t="n"/>
-      <c r="I78" s="66" t="n"/>
-      <c r="J78" s="66" t="n"/>
-      <c r="K78" s="66" t="n"/>
-      <c r="L78" s="66" t="n"/>
-      <c r="M78" s="66" t="n"/>
-      <c r="N78" s="66" t="n"/>
-      <c r="O78" s="66" t="n"/>
-      <c r="P78" s="66" t="n"/>
-      <c r="Q78" s="67" t="n"/>
-      <c r="R78" s="32" t="n"/>
-      <c r="S78" s="32" t="n"/>
-      <c r="T78" s="32" t="n"/>
-      <c r="U78" s="32" t="n"/>
-      <c r="V78" s="32" t="n"/>
-      <c r="X78" s="68" t="n"/>
-      <c r="Y78" s="69" t="n"/>
-      <c r="Z78" s="66" t="n"/>
-      <c r="AA78" s="66" t="n"/>
-      <c r="AB78" s="70" t="n"/>
-      <c r="AC78" s="71" t="n"/>
-      <c r="AD78" s="71" t="n"/>
-      <c r="AE78" s="71" t="n"/>
-      <c r="AF78" s="71" t="n"/>
-      <c r="AG78" s="71" t="n"/>
-      <c r="AH78" s="71" t="n"/>
-      <c r="AI78" s="71" t="n"/>
-      <c r="AJ78" s="71" t="n"/>
-      <c r="AK78" s="71" t="n"/>
-      <c r="AL78" s="71" t="n"/>
-      <c r="AM78" s="71" t="n"/>
-      <c r="AN78" s="71" t="n"/>
-      <c r="AO78" s="71" t="n"/>
-      <c r="AP78" s="71" t="n"/>
-      <c r="AQ78" s="71" t="n"/>
-      <c r="AR78" s="71" t="n"/>
-      <c r="AS78" s="71" t="n"/>
-      <c r="AT78" s="71" t="n"/>
-      <c r="AU78" s="71" t="n"/>
-      <c r="AV78" s="71" t="n"/>
-      <c r="AW78" s="71" t="n"/>
-      <c r="AX78" s="71" t="n"/>
-      <c r="AY78" s="71" t="n"/>
-      <c r="AZ78" s="71" t="n"/>
-      <c r="BA78" s="71" t="n"/>
-      <c r="BB78" s="71" t="n"/>
-      <c r="BC78" s="71" t="n"/>
-      <c r="BD78" s="71" t="n"/>
-      <c r="BE78" s="71" t="n"/>
-      <c r="BF78" s="71" t="n"/>
-      <c r="BG78" s="71" t="n"/>
-      <c r="BH78" s="71" t="n"/>
-      <c r="BI78" s="71" t="n"/>
-      <c r="BJ78" s="71" t="n"/>
-      <c r="BK78" s="71" t="n"/>
-      <c r="BL78" s="71" t="n"/>
-      <c r="BM78" s="71" t="n"/>
-      <c r="BN78" s="71" t="n"/>
-      <c r="BO78" s="71" t="n"/>
-      <c r="BP78" s="71" t="n"/>
-      <c r="BQ78" s="71" t="n"/>
-      <c r="BR78" s="71" t="n"/>
-      <c r="BS78" s="71" t="n"/>
-      <c r="BT78" s="71" t="n"/>
-      <c r="BU78" s="71" t="n"/>
-      <c r="BV78" s="71" t="n"/>
-      <c r="BW78" s="71" t="n"/>
-      <c r="BX78" s="71" t="n"/>
-      <c r="BY78" s="71" t="n"/>
-      <c r="BZ78" s="71" t="n"/>
-      <c r="CA78" s="71" t="n"/>
-      <c r="CB78" s="71" t="n"/>
-      <c r="CC78" s="71" t="n"/>
-      <c r="CD78" s="71" t="n"/>
-      <c r="CE78" s="71" t="n"/>
-      <c r="CF78" s="71" t="n"/>
-      <c r="CG78" s="71" t="n"/>
-      <c r="CH78" s="71" t="n"/>
-      <c r="CI78" s="72" t="n"/>
-      <c r="CJ78" s="71" t="n"/>
-      <c r="CK78" s="71" t="n"/>
-      <c r="CL78" s="71" t="n"/>
-      <c r="CM78" s="71" t="n"/>
-      <c r="CN78" s="71" t="n"/>
-      <c r="CO78" s="71" t="n"/>
-      <c r="CP78" s="71" t="n">
+      <c r="E78" s="114" t="n"/>
+      <c r="F78" s="114" t="n"/>
+      <c r="G78" s="114" t="n"/>
+      <c r="H78" s="114" t="n"/>
+      <c r="I78" s="114" t="n"/>
+      <c r="J78" s="114" t="n"/>
+      <c r="K78" s="114" t="n"/>
+      <c r="L78" s="114" t="n"/>
+      <c r="M78" s="114" t="n"/>
+      <c r="N78" s="114" t="n"/>
+      <c r="O78" s="114" t="n"/>
+      <c r="P78" s="114" t="n"/>
+      <c r="Q78" s="115" t="n"/>
+      <c r="R78" s="116" t="n"/>
+      <c r="S78" s="116" t="n"/>
+      <c r="T78" s="116" t="n"/>
+      <c r="U78" s="116" t="n"/>
+      <c r="V78" s="116" t="n"/>
+      <c r="W78" s="115" t="n"/>
+      <c r="X78" s="116" t="n"/>
+      <c r="Y78" s="117" t="n"/>
+      <c r="Z78" s="114" t="n"/>
+      <c r="AA78" s="114" t="n"/>
+      <c r="AB78" s="118" t="n"/>
+      <c r="AC78" s="119" t="n"/>
+      <c r="AD78" s="119" t="n"/>
+      <c r="AE78" s="119" t="n"/>
+      <c r="AF78" s="119" t="n"/>
+      <c r="AG78" s="119" t="n"/>
+      <c r="AH78" s="119" t="n"/>
+      <c r="AI78" s="119" t="n"/>
+      <c r="AJ78" s="119" t="n"/>
+      <c r="AK78" s="119" t="n"/>
+      <c r="AL78" s="119" t="n"/>
+      <c r="AM78" s="119" t="n"/>
+      <c r="AN78" s="119" t="n"/>
+      <c r="AO78" s="119" t="n"/>
+      <c r="AP78" s="119" t="n"/>
+      <c r="AQ78" s="119" t="n"/>
+      <c r="AR78" s="119" t="n"/>
+      <c r="AS78" s="119" t="n"/>
+      <c r="AT78" s="119" t="n"/>
+      <c r="AU78" s="119" t="n"/>
+      <c r="AV78" s="119" t="n"/>
+      <c r="AW78" s="119" t="n"/>
+      <c r="AX78" s="119" t="n"/>
+      <c r="AY78" s="119" t="n"/>
+      <c r="AZ78" s="119" t="n"/>
+      <c r="BA78" s="119" t="n"/>
+      <c r="BB78" s="119" t="n"/>
+      <c r="BC78" s="119" t="n"/>
+      <c r="BD78" s="119" t="n"/>
+      <c r="BE78" s="119" t="n"/>
+      <c r="BF78" s="119" t="n"/>
+      <c r="BG78" s="119" t="n"/>
+      <c r="BH78" s="119" t="n"/>
+      <c r="BI78" s="119" t="n"/>
+      <c r="BJ78" s="119" t="n"/>
+      <c r="BK78" s="119" t="n"/>
+      <c r="BL78" s="119" t="n"/>
+      <c r="BM78" s="119" t="n"/>
+      <c r="BN78" s="119" t="n"/>
+      <c r="BO78" s="119" t="n"/>
+      <c r="BP78" s="119" t="n"/>
+      <c r="BQ78" s="119" t="n"/>
+      <c r="BR78" s="119" t="n"/>
+      <c r="BS78" s="119" t="n"/>
+      <c r="BT78" s="119" t="n"/>
+      <c r="BU78" s="119" t="n"/>
+      <c r="BV78" s="119" t="n"/>
+      <c r="BW78" s="119" t="n"/>
+      <c r="BX78" s="119" t="n"/>
+      <c r="BY78" s="119" t="n"/>
+      <c r="BZ78" s="119" t="n"/>
+      <c r="CA78" s="119" t="n"/>
+      <c r="CB78" s="119" t="n"/>
+      <c r="CC78" s="119" t="n"/>
+      <c r="CD78" s="119" t="n"/>
+      <c r="CE78" s="119" t="n"/>
+      <c r="CF78" s="119" t="n"/>
+      <c r="CG78" s="119" t="n"/>
+      <c r="CH78" s="119" t="n"/>
+      <c r="CI78" s="115" t="n"/>
+      <c r="CJ78" s="119" t="n"/>
+      <c r="CK78" s="119" t="n"/>
+      <c r="CL78" s="119" t="n"/>
+      <c r="CM78" s="119" t="n"/>
+      <c r="CN78" s="119" t="n"/>
+      <c r="CO78" s="119" t="n"/>
+      <c r="CP78" s="119" t="n">
         <v>792</v>
       </c>
-      <c r="CQ78" s="73" t="n"/>
+      <c r="CQ78" s="119" t="n"/>
+      <c r="CR78" s="115" t="n"/>
+      <c r="CS78" s="115" t="n"/>
+      <c r="CT78" s="115" t="n"/>
     </row>
     <row r="79">
       <c r="E79" s="21" t="n"/>

</xml_diff>

<commit_message>
fix: quitar negrita en area de materiales (casetas y cajas) y vaciar fila 78 en cajas
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="dd/mm/yy;@"/>
     <numFmt numFmtId="168" formatCode="dd/mmm/yy"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,6 +131,12 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font/>
   </fonts>
   <fills count="12">
     <fill>
@@ -801,19 +807,21 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3919,7 +3927,7 @@
       </c>
       <c r="CS27" s="42" t="n"/>
       <c r="CT27" s="111" t="n"/>
-      <c r="CU27" s="32" t="n">
+      <c r="CU27" s="113" t="n">
         <v>618</v>
       </c>
       <c r="CV27" s="14" t="n"/>
@@ -15179,7 +15187,7 @@
       </c>
       <c r="CM28" s="42" t="n"/>
       <c r="CN28" s="111" t="n"/>
-      <c r="CO28" s="32" t="n">
+      <c r="CO28" s="113" t="n">
         <v>100</v>
       </c>
       <c r="CP28" s="14" t="n"/>
@@ -22113,45 +22121,33 @@
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A78" s="113" t="n"/>
-      <c r="B78" s="113" t="inlineStr">
-        <is>
-          <t>MORELOS</t>
-        </is>
-      </c>
-      <c r="C78" s="113" t="inlineStr">
-        <is>
-          <t>MORELOS</t>
-        </is>
-      </c>
-      <c r="D78" s="113" t="inlineStr">
-        <is>
-          <t>IASA</t>
-        </is>
-      </c>
-      <c r="E78" s="114" t="n"/>
-      <c r="F78" s="114" t="n"/>
-      <c r="G78" s="114" t="n"/>
-      <c r="H78" s="114" t="n"/>
-      <c r="I78" s="114" t="n"/>
-      <c r="J78" s="114" t="n"/>
-      <c r="K78" s="114" t="n"/>
-      <c r="L78" s="114" t="n"/>
-      <c r="M78" s="114" t="n"/>
-      <c r="N78" s="114" t="n"/>
-      <c r="O78" s="114" t="n"/>
-      <c r="P78" s="114" t="n"/>
-      <c r="Q78" s="115" t="n"/>
+      <c r="A78" s="114" t="n"/>
+      <c r="B78" s="114" t="n"/>
+      <c r="C78" s="114" t="n"/>
+      <c r="D78" s="114" t="n"/>
+      <c r="E78" s="115" t="n"/>
+      <c r="F78" s="115" t="n"/>
+      <c r="G78" s="115" t="n"/>
+      <c r="H78" s="115" t="n"/>
+      <c r="I78" s="115" t="n"/>
+      <c r="J78" s="115" t="n"/>
+      <c r="K78" s="115" t="n"/>
+      <c r="L78" s="115" t="n"/>
+      <c r="M78" s="115" t="n"/>
+      <c r="N78" s="115" t="n"/>
+      <c r="O78" s="115" t="n"/>
+      <c r="P78" s="115" t="n"/>
+      <c r="Q78" s="114" t="n"/>
       <c r="R78" s="116" t="n"/>
       <c r="S78" s="116" t="n"/>
       <c r="T78" s="116" t="n"/>
       <c r="U78" s="116" t="n"/>
       <c r="V78" s="116" t="n"/>
-      <c r="W78" s="115" t="n"/>
+      <c r="W78" s="114" t="n"/>
       <c r="X78" s="116" t="n"/>
       <c r="Y78" s="117" t="n"/>
-      <c r="Z78" s="114" t="n"/>
-      <c r="AA78" s="114" t="n"/>
+      <c r="Z78" s="115" t="n"/>
+      <c r="AA78" s="115" t="n"/>
       <c r="AB78" s="118" t="n"/>
       <c r="AC78" s="119" t="n"/>
       <c r="AD78" s="119" t="n"/>
@@ -22211,20 +22207,18 @@
       <c r="CF78" s="119" t="n"/>
       <c r="CG78" s="119" t="n"/>
       <c r="CH78" s="119" t="n"/>
-      <c r="CI78" s="115" t="n"/>
+      <c r="CI78" s="114" t="n"/>
       <c r="CJ78" s="119" t="n"/>
       <c r="CK78" s="119" t="n"/>
       <c r="CL78" s="119" t="n"/>
       <c r="CM78" s="119" t="n"/>
       <c r="CN78" s="119" t="n"/>
       <c r="CO78" s="119" t="n"/>
-      <c r="CP78" s="119" t="n">
-        <v>792</v>
-      </c>
+      <c r="CP78" s="119" t="n"/>
       <c r="CQ78" s="119" t="n"/>
-      <c r="CR78" s="115" t="n"/>
-      <c r="CS78" s="115" t="n"/>
-      <c r="CT78" s="115" t="n"/>
+      <c r="CR78" s="114" t="n"/>
+      <c r="CS78" s="114" t="n"/>
+      <c r="CT78" s="114" t="n"/>
     </row>
     <row r="79">
       <c r="E79" s="21" t="n"/>

</xml_diff>

<commit_message>
Actualizar datos y Reporte Diario Excel con 178 registros y 30 entregas de Linkaform
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -3849,9 +3849,11 @@
       <c r="AB27" s="24" t="n"/>
       <c r="AC27" s="24" t="n"/>
       <c r="AD27" s="24" t="n">
-        <v>31</v>
-      </c>
-      <c r="AE27" s="24" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="AE27" s="24" t="n">
+        <v>16</v>
+      </c>
       <c r="AF27" s="24" t="n"/>
       <c r="AG27" s="24" t="n"/>
       <c r="AH27" s="24" t="n"/>
@@ -3917,13 +3919,13 @@
         <v/>
       </c>
       <c r="CP27" s="27" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="CQ27" s="22" t="n">
         <v>0</v>
       </c>
       <c r="CR27" s="22" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="CS27" s="42" t="n"/>
       <c r="CT27" s="111" t="n"/>
@@ -10531,7 +10533,9 @@
       <c r="AB76" s="24" t="n"/>
       <c r="AC76" s="24" t="n"/>
       <c r="AD76" s="24" t="n"/>
-      <c r="AE76" s="24" t="n"/>
+      <c r="AE76" s="24" t="n">
+        <v>2</v>
+      </c>
       <c r="AF76" s="24" t="n"/>
       <c r="AG76" s="24" t="n"/>
       <c r="AH76" s="24" t="n"/>
@@ -10597,13 +10601,13 @@
         <v/>
       </c>
       <c r="CP76" s="27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CQ76" s="22" t="n">
         <v>0</v>
       </c>
       <c r="CR76" s="22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CS76" s="42" t="n"/>
       <c r="CT76" s="111" t="n"/>
@@ -14976,7 +14980,9 @@
       <c r="AJ27" s="24" t="n">
         <v>53</v>
       </c>
-      <c r="AK27" s="24" t="n"/>
+      <c r="AK27" s="24" t="n">
+        <v>19</v>
+      </c>
       <c r="AL27" s="24" t="n"/>
       <c r="AM27" s="24" t="n"/>
       <c r="AN27" s="24" t="n"/>
@@ -15030,11 +15036,11 @@
         <v/>
       </c>
       <c r="CJ27" s="27" t="n">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="CK27" s="22" t="n"/>
       <c r="CL27" s="22" t="n">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="CM27" s="42" t="n"/>
       <c r="CN27" s="111" t="n"/>
@@ -15125,7 +15131,9 @@
       <c r="AJ28" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="AK28" s="24" t="n"/>
+      <c r="AK28" s="24" t="n">
+        <v>15</v>
+      </c>
       <c r="AL28" s="24" t="n"/>
       <c r="AM28" s="24" t="n"/>
       <c r="AN28" s="24" t="n"/>
@@ -15179,16 +15187,16 @@
         <v/>
       </c>
       <c r="CJ28" s="27" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="CK28" s="22" t="n"/>
       <c r="CL28" s="22" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="CM28" s="42" t="n"/>
       <c r="CN28" s="111" t="n"/>
       <c r="CO28" s="113" t="n">
-        <v>100</v>
+        <v>234</v>
       </c>
       <c r="CP28" s="14" t="n"/>
       <c r="CQ28" s="14" t="n"/>
@@ -15271,7 +15279,9 @@
       <c r="AH29" s="24" t="n"/>
       <c r="AI29" s="24" t="n"/>
       <c r="AJ29" s="24" t="n"/>
-      <c r="AK29" s="24" t="n"/>
+      <c r="AK29" s="24" t="n">
+        <v>3</v>
+      </c>
       <c r="AL29" s="24" t="n"/>
       <c r="AM29" s="24" t="n"/>
       <c r="AN29" s="24" t="n"/>
@@ -15324,13 +15334,17 @@
         <f>+SUM(AC29:CG29)</f>
         <v/>
       </c>
-      <c r="CJ29" s="27" t="n"/>
+      <c r="CJ29" s="27" t="n">
+        <v>3</v>
+      </c>
       <c r="CK29" s="22" t="n"/>
-      <c r="CL29" s="22" t="n"/>
+      <c r="CL29" s="22" t="n">
+        <v>3</v>
+      </c>
       <c r="CM29" s="42" t="n"/>
       <c r="CN29" s="111" t="n"/>
       <c r="CO29" s="14" t="n">
-        <v>49</v>
+        <v>289</v>
       </c>
       <c r="CP29" s="14" t="n"/>
       <c r="CQ29" s="14" t="n"/>
@@ -15466,7 +15480,7 @@
       <c r="CM30" s="42" t="n"/>
       <c r="CN30" s="111" t="n"/>
       <c r="CO30" s="14" t="n">
-        <v>121</v>
+        <v>184</v>
       </c>
       <c r="CP30" s="14" t="n"/>
       <c r="CQ30" s="14" t="n"/>
@@ -15742,7 +15756,9 @@
       <c r="CL32" s="22" t="n"/>
       <c r="CM32" s="42" t="n"/>
       <c r="CN32" s="111" t="n"/>
-      <c r="CO32" s="14" t="n"/>
+      <c r="CO32" s="14" t="n">
+        <v>88</v>
+      </c>
       <c r="CP32" s="14" t="n"/>
       <c r="CQ32" s="14" t="n"/>
       <c r="CR32" s="112" t="n"/>
@@ -16151,7 +16167,9 @@
       <c r="CL35" s="22" t="n"/>
       <c r="CM35" s="42" t="n"/>
       <c r="CN35" s="111" t="n"/>
-      <c r="CO35" s="14" t="n"/>
+      <c r="CO35" s="14" t="n">
+        <v>78</v>
+      </c>
       <c r="CP35" s="14" t="n"/>
       <c r="CQ35" s="14" t="n"/>
       <c r="CR35" s="112" t="n"/>
@@ -16227,7 +16245,9 @@
       <c r="AH36" s="24" t="n"/>
       <c r="AI36" s="24" t="n"/>
       <c r="AJ36" s="24" t="n"/>
-      <c r="AK36" s="24" t="n"/>
+      <c r="AK36" s="24" t="n">
+        <v>11</v>
+      </c>
       <c r="AL36" s="24" t="n"/>
       <c r="AM36" s="24" t="n"/>
       <c r="AN36" s="24" t="n"/>
@@ -16280,9 +16300,13 @@
         <f>+SUM(AC36:CG36)</f>
         <v/>
       </c>
-      <c r="CJ36" s="27" t="n"/>
+      <c r="CJ36" s="27" t="n">
+        <v>11</v>
+      </c>
       <c r="CK36" s="22" t="n"/>
-      <c r="CL36" s="22" t="n"/>
+      <c r="CL36" s="22" t="n">
+        <v>11</v>
+      </c>
       <c r="CM36" s="42" t="n"/>
       <c r="CN36" s="111" t="n"/>
       <c r="CO36" s="14" t="n"/>
@@ -16966,7 +16990,9 @@
       <c r="CL41" s="22" t="n"/>
       <c r="CM41" s="42" t="n"/>
       <c r="CN41" s="111" t="n"/>
-      <c r="CO41" s="14" t="n"/>
+      <c r="CO41" s="14" t="n">
+        <v>2</v>
+      </c>
       <c r="CP41" s="14" t="n"/>
       <c r="CQ41" s="14" t="n"/>
       <c r="CR41" s="112" t="n"/>
@@ -17242,7 +17268,9 @@
       <c r="CL43" s="22" t="n"/>
       <c r="CM43" s="42" t="n"/>
       <c r="CN43" s="111" t="n"/>
-      <c r="CO43" s="14" t="n"/>
+      <c r="CO43" s="14" t="n">
+        <v>20</v>
+      </c>
       <c r="CP43" s="14" t="n"/>
       <c r="CQ43" s="14" t="n"/>
       <c r="CR43" s="112" t="n"/>
@@ -17599,7 +17627,9 @@
       <c r="AH46" s="24" t="n"/>
       <c r="AI46" s="24" t="n"/>
       <c r="AJ46" s="24" t="n"/>
-      <c r="AK46" s="24" t="n"/>
+      <c r="AK46" s="24" t="n">
+        <v>1</v>
+      </c>
       <c r="AL46" s="24" t="n"/>
       <c r="AM46" s="24" t="n"/>
       <c r="AN46" s="24" t="n"/>
@@ -17652,12 +17682,18 @@
         <f>+SUM(AC46:CG46)</f>
         <v/>
       </c>
-      <c r="CJ46" s="27" t="n"/>
+      <c r="CJ46" s="27" t="n">
+        <v>1</v>
+      </c>
       <c r="CK46" s="22" t="n"/>
-      <c r="CL46" s="22" t="n"/>
+      <c r="CL46" s="22" t="n">
+        <v>1</v>
+      </c>
       <c r="CM46" s="42" t="n"/>
       <c r="CN46" s="111" t="n"/>
-      <c r="CO46" s="14" t="n"/>
+      <c r="CO46" s="14" t="n">
+        <v>14</v>
+      </c>
       <c r="CP46" s="14" t="n"/>
       <c r="CQ46" s="14" t="n"/>
       <c r="CR46" s="112" t="n"/>
@@ -18204,7 +18240,9 @@
       <c r="CL50" s="22" t="n"/>
       <c r="CM50" s="42" t="n"/>
       <c r="CN50" s="111" t="n"/>
-      <c r="CO50" s="14" t="n"/>
+      <c r="CO50" s="14" t="n">
+        <v>11</v>
+      </c>
       <c r="CP50" s="14" t="n"/>
       <c r="CQ50" s="14" t="n"/>
       <c r="CR50" s="112" t="n"/>
@@ -19098,7 +19136,9 @@
       <c r="AH57" s="24" t="n"/>
       <c r="AI57" s="24" t="n"/>
       <c r="AJ57" s="24" t="n"/>
-      <c r="AK57" s="24" t="n"/>
+      <c r="AK57" s="24" t="n">
+        <v>4</v>
+      </c>
       <c r="AL57" s="24" t="n"/>
       <c r="AM57" s="24" t="n"/>
       <c r="AN57" s="24" t="n"/>
@@ -19151,12 +19191,18 @@
         <f>+SUM(AC57:CG57)</f>
         <v/>
       </c>
-      <c r="CJ57" s="27" t="n"/>
+      <c r="CJ57" s="27" t="n">
+        <v>4</v>
+      </c>
       <c r="CK57" s="22" t="n"/>
-      <c r="CL57" s="22" t="n"/>
+      <c r="CL57" s="22" t="n">
+        <v>4</v>
+      </c>
       <c r="CM57" s="42" t="n"/>
       <c r="CN57" s="111" t="n"/>
-      <c r="CO57" s="14" t="n"/>
+      <c r="CO57" s="14" t="n">
+        <v>14</v>
+      </c>
       <c r="CP57" s="14" t="n"/>
       <c r="CQ57" s="14" t="n"/>
       <c r="CR57" s="112" t="n"/>
@@ -19566,7 +19612,9 @@
       <c r="CL60" s="22" t="n"/>
       <c r="CM60" s="42" t="n"/>
       <c r="CN60" s="111" t="n"/>
-      <c r="CO60" s="14" t="n"/>
+      <c r="CO60" s="14" t="n">
+        <v>86</v>
+      </c>
       <c r="CP60" s="14" t="n"/>
       <c r="CQ60" s="14" t="n"/>
       <c r="CR60" s="112" t="n"/>

</xml_diff>

<commit_message>
Corregir desfase de huso horario en lectura de fechas ExcelJS para evitar duplicacion de datos en 22 de octubre
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -25379,147 +25379,53 @@
       <c r="AL83" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="AM83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BY83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BZ83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CA83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CC83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CD83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CE83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CF83" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CG83" s="25" t="n">
-        <v>0</v>
-      </c>
+      <c r="AM83" s="25" t="n"/>
+      <c r="AN83" s="25" t="n"/>
+      <c r="AO83" s="25" t="n"/>
+      <c r="AP83" s="25" t="n"/>
+      <c r="AQ83" s="25" t="n"/>
+      <c r="AR83" s="25" t="n"/>
+      <c r="AS83" s="25" t="n"/>
+      <c r="AT83" s="25" t="n"/>
+      <c r="AU83" s="25" t="n"/>
+      <c r="AV83" s="25" t="n"/>
+      <c r="AW83" s="25" t="n"/>
+      <c r="AX83" s="25" t="n"/>
+      <c r="AY83" s="25" t="n"/>
+      <c r="AZ83" s="25" t="n"/>
+      <c r="BA83" s="25" t="n"/>
+      <c r="BB83" s="25" t="n"/>
+      <c r="BC83" s="25" t="n"/>
+      <c r="BD83" s="25" t="n"/>
+      <c r="BE83" s="25" t="n"/>
+      <c r="BF83" s="25" t="n"/>
+      <c r="BG83" s="25" t="n"/>
+      <c r="BH83" s="25" t="n"/>
+      <c r="BI83" s="25" t="n"/>
+      <c r="BJ83" s="25" t="n"/>
+      <c r="BK83" s="25" t="n"/>
+      <c r="BL83" s="25" t="n"/>
+      <c r="BM83" s="25" t="n"/>
+      <c r="BN83" s="25" t="n"/>
+      <c r="BO83" s="25" t="n"/>
+      <c r="BP83" s="25" t="n"/>
+      <c r="BQ83" s="25" t="n"/>
+      <c r="BR83" s="25" t="n"/>
+      <c r="BS83" s="25" t="n"/>
+      <c r="BT83" s="25" t="n"/>
+      <c r="BU83" s="25" t="n"/>
+      <c r="BV83" s="25" t="n"/>
+      <c r="BW83" s="25" t="n"/>
+      <c r="BX83" s="25" t="n"/>
+      <c r="BY83" s="25" t="n"/>
+      <c r="BZ83" s="25" t="n"/>
+      <c r="CA83" s="25" t="n"/>
+      <c r="CB83" s="25" t="n"/>
+      <c r="CC83" s="25" t="n"/>
+      <c r="CD83" s="25" t="n"/>
+      <c r="CE83" s="25" t="n"/>
+      <c r="CF83" s="25" t="n"/>
+      <c r="CG83" s="25" t="n"/>
       <c r="CH83" s="25" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
data: actualizacion de dashboard con 428 registros limpios sin pruebas ni duplicados
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -3929,7 +3929,7 @@
         <v>11</v>
       </c>
       <c r="AG27" s="24" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AH27" s="24" t="n"/>
       <c r="AI27" s="24" t="n"/>
@@ -4249,7 +4249,9 @@
       <c r="AD29" s="24" t="n"/>
       <c r="AE29" s="24" t="n"/>
       <c r="AF29" s="24" t="n"/>
-      <c r="AG29" s="24" t="n"/>
+      <c r="AG29" s="24" t="n">
+        <v>18</v>
+      </c>
       <c r="AH29" s="24" t="n"/>
       <c r="AI29" s="24" t="n"/>
       <c r="AJ29" s="24" t="n"/>
@@ -16491,7 +16493,7 @@
         <v>22</v>
       </c>
       <c r="AM27" s="24" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AN27" s="24" t="n"/>
       <c r="AO27" s="24" t="n"/>
@@ -16857,7 +16859,7 @@
       </c>
       <c r="AL29" s="24" t="n"/>
       <c r="AM29" s="24" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="AN29" s="24" t="n"/>
       <c r="AO29" s="24" t="n"/>
@@ -19598,7 +19600,7 @@
         <v>20</v>
       </c>
       <c r="AM46" s="24" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="AN46" s="24" t="n"/>
       <c r="AO46" s="24" t="n"/>
@@ -21029,7 +21031,7 @@
       <c r="AK55" s="24" t="n"/>
       <c r="AL55" s="24" t="n"/>
       <c r="AM55" s="24" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AN55" s="24" t="n"/>
       <c r="AO55" s="24" t="n"/>

</xml_diff>

<commit_message>
data: actualizacion de reportes con deduplicacion automatica y sincronizacion Linkaform
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -3931,7 +3931,9 @@
       <c r="AG27" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="AH27" s="24" t="n"/>
+      <c r="AH27" s="24" t="n">
+        <v>1</v>
+      </c>
       <c r="AI27" s="24" t="n"/>
       <c r="AJ27" s="24" t="n"/>
       <c r="AK27" s="24" t="n"/>
@@ -4091,9 +4093,11 @@
       <c r="AE28" s="24" t="n"/>
       <c r="AF28" s="24" t="n"/>
       <c r="AG28" s="24" t="n">
-        <v>43</v>
-      </c>
-      <c r="AH28" s="24" t="n"/>
+        <v>29</v>
+      </c>
+      <c r="AH28" s="24" t="n">
+        <v>10</v>
+      </c>
       <c r="AI28" s="24" t="n"/>
       <c r="AJ28" s="24" t="n"/>
       <c r="AK28" s="24" t="n"/>
@@ -4249,10 +4253,10 @@
       <c r="AD29" s="24" t="n"/>
       <c r="AE29" s="24" t="n"/>
       <c r="AF29" s="24" t="n"/>
-      <c r="AG29" s="24" t="n">
+      <c r="AG29" s="24" t="n"/>
+      <c r="AH29" s="24" t="n">
         <v>18</v>
       </c>
-      <c r="AH29" s="24" t="n"/>
       <c r="AI29" s="24" t="n"/>
       <c r="AJ29" s="24" t="n"/>
       <c r="AK29" s="24" t="n"/>
@@ -7265,7 +7269,9 @@
       <c r="AE49" s="24" t="n"/>
       <c r="AF49" s="24" t="n"/>
       <c r="AG49" s="24" t="n"/>
-      <c r="AH49" s="24" t="n"/>
+      <c r="AH49" s="24" t="n">
+        <v>1</v>
+      </c>
       <c r="AI49" s="24" t="n"/>
       <c r="AJ49" s="24" t="n"/>
       <c r="AK49" s="24" t="n"/>
@@ -16495,7 +16501,9 @@
       <c r="AM27" s="24" t="n">
         <v>26</v>
       </c>
-      <c r="AN27" s="24" t="n"/>
+      <c r="AN27" s="24" t="n">
+        <v>1</v>
+      </c>
       <c r="AO27" s="24" t="n"/>
       <c r="AP27" s="24" t="n"/>
       <c r="AQ27" s="24" t="n"/>
@@ -16859,9 +16867,11 @@
       </c>
       <c r="AL29" s="24" t="n"/>
       <c r="AM29" s="24" t="n">
-        <v>17</v>
-      </c>
-      <c r="AN29" s="24" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="AN29" s="24" t="n">
+        <v>7</v>
+      </c>
       <c r="AO29" s="24" t="n"/>
       <c r="AP29" s="24" t="n"/>
       <c r="AQ29" s="24" t="n"/>
@@ -19600,9 +19610,11 @@
         <v>20</v>
       </c>
       <c r="AM46" s="24" t="n">
-        <v>19</v>
-      </c>
-      <c r="AN46" s="24" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="AN46" s="24" t="n">
+        <v>10</v>
+      </c>
       <c r="AO46" s="24" t="n"/>
       <c r="AP46" s="24" t="n"/>
       <c r="AQ46" s="24" t="n"/>
@@ -21356,7 +21368,9 @@
       <c r="AM57" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="AN57" s="24" t="n"/>
+      <c r="AN57" s="24" t="n">
+        <v>2</v>
+      </c>
       <c r="AO57" s="24" t="n"/>
       <c r="AP57" s="24" t="n"/>
       <c r="AQ57" s="24" t="n"/>

</xml_diff>

<commit_message>
feat: Implementar regla oficial de horario de corte 10 PM y ventana matutina 10 AM con banner de estado y soporte en reportes Excel
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -3926,13 +3926,13 @@
         <v>16</v>
       </c>
       <c r="AF27" s="24" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="AG27" s="24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AH27" s="24" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="AI27" s="24" t="n"/>
       <c r="AJ27" s="24" t="n"/>
@@ -4093,10 +4093,10 @@
       <c r="AE28" s="24" t="n"/>
       <c r="AF28" s="24" t="n"/>
       <c r="AG28" s="24" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="AH28" s="24" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="AI28" s="24" t="n"/>
       <c r="AJ28" s="24" t="n"/>
@@ -4253,9 +4253,11 @@
       <c r="AD29" s="24" t="n"/>
       <c r="AE29" s="24" t="n"/>
       <c r="AF29" s="24" t="n"/>
-      <c r="AG29" s="24" t="n"/>
+      <c r="AG29" s="24" t="n">
+        <v>3</v>
+      </c>
       <c r="AH29" s="24" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AI29" s="24" t="n"/>
       <c r="AJ29" s="24" t="n"/>
@@ -4799,7 +4801,7 @@
       </c>
       <c r="CX32" s="79" t="n"/>
       <c r="CY32" s="17" t="n">
-        <v>36</v>
+        <v>188</v>
       </c>
       <c r="DD32" s="14">
         <f>SUM(CY32:DC32)</f>
@@ -7269,9 +7271,7 @@
       <c r="AE49" s="24" t="n"/>
       <c r="AF49" s="24" t="n"/>
       <c r="AG49" s="24" t="n"/>
-      <c r="AH49" s="24" t="n">
-        <v>1</v>
-      </c>
+      <c r="AH49" s="24" t="n"/>
       <c r="AI49" s="24" t="n"/>
       <c r="AJ49" s="24" t="n"/>
       <c r="AK49" s="24" t="n"/>
@@ -11370,7 +11370,9 @@
       <c r="AE76" s="24" t="n"/>
       <c r="AF76" s="24" t="n"/>
       <c r="AG76" s="24" t="n"/>
-      <c r="AH76" s="24" t="n"/>
+      <c r="AH76" s="24" t="n">
+        <v>2</v>
+      </c>
       <c r="AI76" s="24" t="n"/>
       <c r="AJ76" s="24" t="n"/>
       <c r="AK76" s="24" t="n"/>
@@ -16496,13 +16498,13 @@
         <v>19</v>
       </c>
       <c r="AL27" s="24" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="AM27" s="24" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="AN27" s="24" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="AO27" s="24" t="n"/>
       <c r="AP27" s="24" t="n"/>
@@ -16684,7 +16686,9 @@
       <c r="AM28" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="AN28" s="24" t="n"/>
+      <c r="AN28" s="24" t="n">
+        <v>11</v>
+      </c>
       <c r="AO28" s="24" t="n"/>
       <c r="AP28" s="24" t="n"/>
       <c r="AQ28" s="24" t="n"/>
@@ -16867,10 +16871,10 @@
       </c>
       <c r="AL29" s="24" t="n"/>
       <c r="AM29" s="24" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="AN29" s="24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AO29" s="24" t="n"/>
       <c r="AP29" s="24" t="n"/>
@@ -17432,8 +17436,11 @@
       <c r="CT32" t="n">
         <v>12</v>
       </c>
+      <c r="DA32" t="n">
+        <v>2</v>
+      </c>
       <c r="DB32" t="n">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="DC32" s="14">
         <f>SUM(CS32:DB32)</f>
@@ -18003,7 +18010,9 @@
         <v>9</v>
       </c>
       <c r="AM36" s="24" t="n"/>
-      <c r="AN36" s="24" t="n"/>
+      <c r="AN36" s="24" t="n">
+        <v>2</v>
+      </c>
       <c r="AO36" s="24" t="n"/>
       <c r="AP36" s="24" t="n"/>
       <c r="AQ36" s="24" t="n"/>
@@ -18162,7 +18171,9 @@
       <c r="AK37" s="24" t="n"/>
       <c r="AL37" s="24" t="n"/>
       <c r="AM37" s="24" t="n"/>
-      <c r="AN37" s="24" t="n"/>
+      <c r="AN37" s="24" t="n">
+        <v>2</v>
+      </c>
       <c r="AO37" s="24" t="n"/>
       <c r="AP37" s="24" t="n"/>
       <c r="AQ37" s="24" t="n"/>
@@ -19129,7 +19140,9 @@
       <c r="AM43" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="AN43" s="24" t="n"/>
+      <c r="AN43" s="24" t="n">
+        <v>20</v>
+      </c>
       <c r="AO43" s="24" t="n"/>
       <c r="AP43" s="24" t="n"/>
       <c r="AQ43" s="24" t="n"/>
@@ -19610,10 +19623,10 @@
         <v>20</v>
       </c>
       <c r="AM46" s="24" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="AN46" s="24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AO46" s="24" t="n"/>
       <c r="AP46" s="24" t="n"/>
@@ -20411,7 +20424,9 @@
       <c r="AK51" s="24" t="n"/>
       <c r="AL51" s="24" t="n"/>
       <c r="AM51" s="24" t="n"/>
-      <c r="AN51" s="24" t="n"/>
+      <c r="AN51" s="24" t="n">
+        <v>1</v>
+      </c>
       <c r="AO51" s="24" t="n"/>
       <c r="AP51" s="24" t="n"/>
       <c r="AQ51" s="24" t="n"/>
@@ -20962,7 +20977,9 @@
         <v/>
       </c>
       <c r="CR54" s="79" t="n"/>
-      <c r="CS54" s="17" t="n"/>
+      <c r="CS54" s="17" t="n">
+        <v>26</v>
+      </c>
       <c r="DC54" s="14">
         <f>SUM(CS54:DB54)</f>
         <v/>
@@ -21043,9 +21060,11 @@
       <c r="AK55" s="24" t="n"/>
       <c r="AL55" s="24" t="n"/>
       <c r="AM55" s="24" t="n">
-        <v>14</v>
-      </c>
-      <c r="AN55" s="24" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="AN55" s="24" t="n">
+        <v>6</v>
+      </c>
       <c r="AO55" s="24" t="n"/>
       <c r="AP55" s="24" t="n"/>
       <c r="AQ55" s="24" t="n"/>
@@ -21446,7 +21465,9 @@
         <v/>
       </c>
       <c r="CR57" s="79" t="n"/>
-      <c r="CS57" s="17" t="n"/>
+      <c r="CS57" s="17" t="n">
+        <v>46</v>
+      </c>
       <c r="CV57" t="n">
         <v>45</v>
       </c>
@@ -22011,7 +22032,9 @@
       <c r="AM61" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="AN61" s="24" t="n"/>
+      <c r="AN61" s="24" t="n">
+        <v>3</v>
+      </c>
       <c r="AO61" s="24" t="n"/>
       <c r="AP61" s="24" t="n"/>
       <c r="AQ61" s="24" t="n"/>
@@ -22491,7 +22514,9 @@
       <c r="AK64" s="24" t="n"/>
       <c r="AL64" s="24" t="n"/>
       <c r="AM64" s="24" t="n"/>
-      <c r="AN64" s="24" t="n"/>
+      <c r="AN64" s="24" t="n">
+        <v>12</v>
+      </c>
       <c r="AO64" s="24" t="n"/>
       <c r="AP64" s="24" t="n"/>
       <c r="AQ64" s="24" t="n"/>
@@ -22568,6 +22593,12 @@
       </c>
       <c r="CR64" s="79" t="n"/>
       <c r="CS64" s="17" t="n"/>
+      <c r="CV64" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB64" t="n">
+        <v>9</v>
+      </c>
       <c r="DC64" s="14">
         <f>SUM(CS64:DB64)</f>
         <v/>
@@ -24256,7 +24287,9 @@
       <c r="AK75" s="24" t="n"/>
       <c r="AL75" s="24" t="n"/>
       <c r="AM75" s="24" t="n"/>
-      <c r="AN75" s="24" t="n"/>
+      <c r="AN75" s="24" t="n">
+        <v>4</v>
+      </c>
       <c r="AO75" s="24" t="n"/>
       <c r="AP75" s="24" t="n"/>
       <c r="AQ75" s="24" t="n"/>
@@ -24333,6 +24366,9 @@
       </c>
       <c r="CR75" s="79" t="n"/>
       <c r="CS75" s="17" t="n"/>
+      <c r="CV75" t="n">
+        <v>1</v>
+      </c>
       <c r="DC75" s="14">
         <f>SUM(CS75:DB75)</f>
         <v/>

</xml_diff>

<commit_message>
feat: congelar linea base oficial entregada al 25-Oct (947 activos) e iniciar acumulacion diaria normal desde 26-Oct (corte 7:00 AM)
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PCI\Documents\Antigravity\dashboard-imagen-telmex\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BBA8C42-44BD-42CA-A3C5-08734612B7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F88555D8-065B-4499-ADCB-5F4CD7651C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN GENERAL" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,6 @@
     <sheet name="Programa CAJAS REPORTE DIARIO" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Programa CAJAS REPORTE DIARIO'!$A$13:$CQ$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Programa CASETAS REPORTE DIARIO'!$A$13:$CW$79</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Programa CAJAS REPORTE DIARIO'!$B$1:$AA$84</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Programa CASETAS REPORTE DIARIO'!$B$1:$U$86</definedName>
   </definedNames>
@@ -28,133 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="171">
-  <si>
-    <t>REPORTE DIARIO DE CASETAS Y CAJAS CONTRATISTAS 2026 - IASA / TELMEX</t>
-  </si>
-  <si>
-    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Reporte matutino cerrado al 25/10/2026 (22:00 hrs). La jornada de hoy se liberará a las 10:00 AM.</t>
-  </si>
-  <si>
-    <t>TOTAL CASETAS AL MOMENTO</t>
-  </si>
-  <si>
-    <t>TOTAL CAJAS AL MOMENTO</t>
-  </si>
-  <si>
-    <t>SUMA TOTAL AL MOMENTO (CASETAS + CAJAS)</t>
-  </si>
-  <si>
-    <t>Casetas Instaladas Validadas</t>
-  </si>
-  <si>
-    <t>Cajas Instaladas Validadas</t>
-  </si>
-  <si>
-    <t>Gran Total Acumulado al Momento</t>
-  </si>
-  <si>
-    <t>DESGLOSE DE AVANCE DIARIO CONSOLIDADO (TELMEX)</t>
-  </si>
-  <si>
-    <t>FECHA</t>
-  </si>
-  <si>
-    <t>DÍA SEMANA</t>
-  </si>
-  <si>
-    <t>CASETAS</t>
-  </si>
-  <si>
-    <t>CAJAS</t>
-  </si>
-  <si>
-    <t>TOTAL DÍA (CASETAS + CAJAS)</t>
-  </si>
-  <si>
-    <t>ACUMULADO AL MOMENTO</t>
-  </si>
-  <si>
-    <t>ESTADO CORTE</t>
-  </si>
-  <si>
-    <t>2026-10-17</t>
-  </si>
-  <si>
-    <t>Sábado</t>
-  </si>
-  <si>
-    <t>Base Histórica</t>
-  </si>
-  <si>
-    <t>2026-10-18</t>
-  </si>
-  <si>
-    <t>Domingo</t>
-  </si>
-  <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>Lunes</t>
-  </si>
-  <si>
-    <t>2026-10-20</t>
-  </si>
-  <si>
-    <t>Martes</t>
-  </si>
-  <si>
-    <t>2026-10-21</t>
-  </si>
-  <si>
-    <t>Miércoles</t>
-  </si>
-  <si>
-    <t>Validado Oficial</t>
-  </si>
-  <si>
-    <t>2026-10-22</t>
-  </si>
-  <si>
-    <t>Jueves</t>
-  </si>
-  <si>
-    <t>2026-10-23</t>
-  </si>
-  <si>
-    <t>Viernes</t>
-  </si>
-  <si>
-    <t>2026-10-24</t>
-  </si>
-  <si>
-    <t>2026-10-25</t>
-  </si>
-  <si>
-    <t>Corte Fin de Semana</t>
-  </si>
-  <si>
-    <t>TOTAL GENERAL AL MOMENTO</t>
-  </si>
-  <si>
-    <t>100% CONCILIADO</t>
-  </si>
-  <si>
-    <t>NOTAS DE INTEGRIDAD Y REGLAS DE AUDITORÍA</t>
-  </si>
-  <si>
-    <t>1. La suma total al momento es de 921 intervenciones oficiales validadas (245 casetas + 676 cajas).</t>
-  </si>
-  <si>
-    <t>2. Cero Data Leakage y Deduplicación Estricta: Cada caseta o caja se contabiliza una sola vez por activo en orden cronológico.</t>
-  </si>
-  <si>
-    <t>3. Diferencia con Linkaform: Los folios registrados en Linkaform que corresponden a reintentos de captura o activos repetidos se deduplican para evitar duplicidades frente a Telmex.</t>
-  </si>
-  <si>
-    <t>4. Regla de Horario de Corte: Las capturas realizadas después de las 22:00 hrs se contabilizan oficialmente para el ciclo del día siguiente.</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="171">
   <si>
     <t>TOTAL CASETAS AL MOMENTO:</t>
   </si>
@@ -487,6 +359,132 @@
   </si>
   <si>
     <t>TIJUANA</t>
+  </si>
+  <si>
+    <t>REPORTE DIARIO DE CASETAS Y CAJAS CONTRATISTAS 2026 - IASA / TELMEX</t>
+  </si>
+  <si>
+    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (26/10/2026, 13:00 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
+  </si>
+  <si>
+    <t>TOTAL CASETAS AL MOMENTO</t>
+  </si>
+  <si>
+    <t>TOTAL CAJAS AL MOMENTO</t>
+  </si>
+  <si>
+    <t>SUMA TOTAL AL MOMENTO (CASETAS + CAJAS)</t>
+  </si>
+  <si>
+    <t>Casetas Instaladas Validadas</t>
+  </si>
+  <si>
+    <t>Cajas Instaladas Validadas</t>
+  </si>
+  <si>
+    <t>Gran Total Acumulado al Momento</t>
+  </si>
+  <si>
+    <t>DESGLOSE DE AVANCE DIARIO CONSOLIDADO (TELMEX)</t>
+  </si>
+  <si>
+    <t>FECHA</t>
+  </si>
+  <si>
+    <t>DÍA SEMANA</t>
+  </si>
+  <si>
+    <t>CASETAS</t>
+  </si>
+  <si>
+    <t>CAJAS</t>
+  </si>
+  <si>
+    <t>TOTAL DÍA (CASETAS + CAJAS)</t>
+  </si>
+  <si>
+    <t>ACUMULADO AL MOMENTO</t>
+  </si>
+  <si>
+    <t>ESTADO CORTE</t>
+  </si>
+  <si>
+    <t>2026-10-17</t>
+  </si>
+  <si>
+    <t>Sábado</t>
+  </si>
+  <si>
+    <t>Línea Base Entregada</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>Domingo</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>Lunes</t>
+  </si>
+  <si>
+    <t>2026-10-20</t>
+  </si>
+  <si>
+    <t>Martes</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
+  </si>
+  <si>
+    <t>Miércoles</t>
+  </si>
+  <si>
+    <t>2026-10-22</t>
+  </si>
+  <si>
+    <t>Jueves</t>
+  </si>
+  <si>
+    <t>2026-10-23</t>
+  </si>
+  <si>
+    <t>Viernes</t>
+  </si>
+  <si>
+    <t>2026-10-24</t>
+  </si>
+  <si>
+    <t>2026-10-25</t>
+  </si>
+  <si>
+    <t>2026-10-26</t>
+  </si>
+  <si>
+    <t>En Proceso (7:00 AM)</t>
+  </si>
+  <si>
+    <t>TOTAL GENERAL AL MOMENTO</t>
+  </si>
+  <si>
+    <t>100% CONCILIADO</t>
+  </si>
+  <si>
+    <t>NOTAS DE INTEGRIDAD Y REGLAS DE AUDITORÍA</t>
+  </si>
+  <si>
+    <t>1. Línea Base Oficial Entregada: Los datos del 17 al 25 de Octubre corresponden al reporte entregado hoy (263 casetas + 684 cajas = 947 intervenciones validadas), los cuales quedan 100% fijos e inmutables.</t>
+  </si>
+  <si>
+    <t>2. Actividad Diaria Normal: A partir del 26 de Octubre, las actividades de campo se suman diariamente en cada corte matutino (7:00 AM) sobre la línea base oficial.</t>
+  </si>
+  <si>
+    <t>3. Deduplicación Estricta: Cada activo físico se contabiliza una sola vez por orden cronológico, protegiendo las cifras frente a reintentos de captura en campo.</t>
+  </si>
+  <si>
+    <t>4. Regla de Horario de Corte: Las capturas realizadas después de las 22:00 hrs se contabilizan oficialmente para el ciclo del día siguiente.</t>
   </si>
   <si>
     <t>TOTAL CAJAS AL MOMENTO:</t>
@@ -1318,8 +1316,19 @@
     <xf numFmtId="0" fontId="19" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1327,10 +1336,12 @@
     <xf numFmtId="0" fontId="21" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1350,19 +1361,6 @@
     <xf numFmtId="0" fontId="25" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="3" builtinId="3"/>
@@ -1680,7 +1678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J26"/>
+  <dimension ref="B2:J27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1693,121 +1691,121 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
+      <c r="B2" s="100" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
     </row>
     <row r="3" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="85" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
+      <c r="B3" s="90" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" s="91"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
     </row>
     <row r="5" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="88" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="84"/>
-      <c r="E5" s="88" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="84"/>
-      <c r="H5" s="89" t="s">
-        <v>4</v>
-      </c>
-      <c r="I5" s="90"/>
-      <c r="J5" s="90"/>
+      <c r="B5" s="95" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="89"/>
+      <c r="E5" s="95" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" s="89"/>
+      <c r="H5" s="96" t="s">
+        <v>115</v>
+      </c>
+      <c r="I5" s="97"/>
+      <c r="J5" s="97"/>
     </row>
     <row r="6" spans="2:10" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="83">
+      <c r="B6" s="88">
         <f>'Programa CASETAS REPORTE DIARIO'!CN79</f>
-        <v>245</v>
-      </c>
-      <c r="C6" s="84"/>
-      <c r="E6" s="83">
+        <v>263</v>
+      </c>
+      <c r="C6" s="89"/>
+      <c r="E6" s="88">
         <f>'Programa CAJAS REPORTE DIARIO'!CH77</f>
-        <v>676</v>
-      </c>
-      <c r="F6" s="84"/>
-      <c r="H6" s="94">
+        <v>684</v>
+      </c>
+      <c r="F6" s="89"/>
+      <c r="H6" s="101">
         <f>B6+E6</f>
-        <v>921</v>
-      </c>
-      <c r="I6" s="90"/>
-      <c r="J6" s="90"/>
+        <v>947</v>
+      </c>
+      <c r="I6" s="97"/>
+      <c r="J6" s="97"/>
     </row>
     <row r="7" spans="2:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="87" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="84"/>
-      <c r="E7" s="87" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="84"/>
-      <c r="H7" s="92" t="s">
-        <v>7</v>
-      </c>
-      <c r="I7" s="90"/>
-      <c r="J7" s="90"/>
+      <c r="B7" s="93" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="89"/>
+      <c r="E7" s="93" t="s">
+        <v>117</v>
+      </c>
+      <c r="F7" s="89"/>
+      <c r="H7" s="99" t="s">
+        <v>118</v>
+      </c>
+      <c r="I7" s="97"/>
+      <c r="J7" s="97"/>
     </row>
     <row r="9" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="82"/>
-      <c r="D9" s="82"/>
-      <c r="E9" s="82"/>
-      <c r="F9" s="82"/>
-      <c r="G9" s="82"/>
-      <c r="H9" s="82"/>
-      <c r="I9" s="82"/>
-      <c r="J9" s="82"/>
+      <c r="B9" s="98" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="91"/>
+      <c r="D9" s="91"/>
+      <c r="E9" s="91"/>
+      <c r="F9" s="91"/>
+      <c r="G9" s="91"/>
+      <c r="H9" s="91"/>
+      <c r="I9" s="91"/>
+      <c r="J9" s="91"/>
     </row>
     <row r="10" spans="2:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="68" t="s">
-        <v>9</v>
+        <v>120</v>
       </c>
       <c r="C10" s="68" t="s">
-        <v>10</v>
+        <v>121</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>11</v>
+        <v>122</v>
       </c>
       <c r="E10" s="68" t="s">
-        <v>12</v>
+        <v>123</v>
       </c>
       <c r="F10" s="68" t="s">
-        <v>13</v>
+        <v>124</v>
       </c>
       <c r="G10" s="68" t="s">
-        <v>14</v>
+        <v>125</v>
       </c>
       <c r="H10" s="68" t="s">
-        <v>15</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="69" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
       <c r="C11" s="69" t="s">
-        <v>17</v>
+        <v>128</v>
       </c>
       <c r="D11" s="70">
         <f>'Programa CASETAS REPORTE DIARIO'!AB79</f>
@@ -1818,7 +1816,7 @@
         <v>52</v>
       </c>
       <c r="F11" s="70">
-        <f t="shared" ref="F11:F19" si="0">D11+E11</f>
+        <f t="shared" ref="F11:F20" si="0">D11+E11</f>
         <v>76</v>
       </c>
       <c r="G11" s="70">
@@ -1826,15 +1824,15 @@
         <v>76</v>
       </c>
       <c r="H11" s="69" t="s">
-        <v>18</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="71" t="s">
-        <v>19</v>
+        <v>130</v>
       </c>
       <c r="C12" s="71" t="s">
-        <v>20</v>
+        <v>131</v>
       </c>
       <c r="D12" s="72">
         <f>'Programa CASETAS REPORTE DIARIO'!AC79</f>
@@ -1849,19 +1847,19 @@
         <v>0</v>
       </c>
       <c r="G12" s="72">
-        <f t="shared" ref="G12:G19" si="1">G11+F12</f>
+        <f t="shared" ref="G12:G20" si="1">G11+F12</f>
         <v>76</v>
       </c>
       <c r="H12" s="71" t="s">
-        <v>18</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="69" t="s">
-        <v>21</v>
+        <v>132</v>
       </c>
       <c r="C13" s="69" t="s">
-        <v>22</v>
+        <v>133</v>
       </c>
       <c r="D13" s="70">
         <f>'Programa CASETAS REPORTE DIARIO'!AD79</f>
@@ -1880,15 +1878,15 @@
         <v>107</v>
       </c>
       <c r="H13" s="69" t="s">
-        <v>18</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="71" t="s">
-        <v>23</v>
+        <v>134</v>
       </c>
       <c r="C14" s="71" t="s">
-        <v>24</v>
+        <v>135</v>
       </c>
       <c r="D14" s="72">
         <f>'Programa CASETAS REPORTE DIARIO'!AE79</f>
@@ -1907,15 +1905,15 @@
         <v>177</v>
       </c>
       <c r="H14" s="71" t="s">
-        <v>18</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="69" t="s">
-        <v>25</v>
+        <v>136</v>
       </c>
       <c r="C15" s="69" t="s">
-        <v>26</v>
+        <v>137</v>
       </c>
       <c r="D15" s="70">
         <f>'Programa CASETAS REPORTE DIARIO'!AF79</f>
@@ -1934,15 +1932,15 @@
         <v>251</v>
       </c>
       <c r="H15" s="69" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="71" t="s">
-        <v>28</v>
+        <v>138</v>
       </c>
       <c r="C16" s="71" t="s">
-        <v>29</v>
+        <v>139</v>
       </c>
       <c r="D16" s="72">
         <f>'Programa CASETAS REPORTE DIARIO'!AG79</f>
@@ -1961,15 +1959,15 @@
         <v>408</v>
       </c>
       <c r="H16" s="71" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="69" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="C17" s="69" t="s">
-        <v>31</v>
+        <v>141</v>
       </c>
       <c r="D17" s="70">
         <f>'Programa CASETAS REPORTE DIARIO'!AH79</f>
@@ -1988,142 +1986,169 @@
         <v>650</v>
       </c>
       <c r="H17" s="69" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="71" t="s">
-        <v>32</v>
+        <v>142</v>
       </c>
       <c r="C18" s="71" t="s">
-        <v>17</v>
+        <v>128</v>
       </c>
       <c r="D18" s="72">
         <f>'Programa CASETAS REPORTE DIARIO'!AI79</f>
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E18" s="72">
         <f>'Programa CAJAS REPORTE DIARIO'!AO77</f>
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="F18" s="72">
         <f t="shared" si="0"/>
-        <v>208</v>
+        <v>181</v>
       </c>
       <c r="G18" s="72">
         <f t="shared" si="1"/>
-        <v>858</v>
+        <v>831</v>
       </c>
       <c r="H18" s="71" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="69" t="s">
-        <v>33</v>
+        <v>143</v>
       </c>
       <c r="C19" s="69" t="s">
-        <v>20</v>
+        <v>131</v>
       </c>
       <c r="D19" s="70">
         <f>'Programa CASETAS REPORTE DIARIO'!AJ79</f>
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="E19" s="70">
         <f>'Programa CAJAS REPORTE DIARIO'!AP77</f>
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="F19" s="70">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="G19" s="70">
         <f t="shared" si="1"/>
-        <v>921</v>
+        <v>947</v>
       </c>
       <c r="H19" s="69" t="s">
-        <v>34</v>
+        <v>129</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="73" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="74"/>
-      <c r="D20" s="75">
-        <f>SUM(D11:D19)</f>
-        <v>245</v>
-      </c>
-      <c r="E20" s="75">
-        <f>SUM(E11:E19)</f>
-        <v>676</v>
-      </c>
-      <c r="F20" s="75">
-        <f>SUM(F11:F19)</f>
-        <v>921</v>
-      </c>
-      <c r="G20" s="75">
-        <f>F20</f>
-        <v>921</v>
-      </c>
-      <c r="H20" s="76" t="s">
-        <v>36</v>
+    <row r="20" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="71" t="s">
+        <v>144</v>
+      </c>
+      <c r="C20" s="71" t="s">
+        <v>133</v>
+      </c>
+      <c r="D20" s="72">
+        <f>'Programa CASETAS REPORTE DIARIO'!AK79</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="72">
+        <f>'Programa CAJAS REPORTE DIARIO'!AQ77</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="72">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="72">
+        <f t="shared" si="1"/>
+        <v>947</v>
+      </c>
+      <c r="H20" s="71" t="s">
+        <v>145</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="81" t="s">
-        <v>37</v>
-      </c>
-      <c r="C22" s="82"/>
-      <c r="D22" s="82"/>
-      <c r="E22" s="82"/>
-      <c r="F22" s="82"/>
-      <c r="G22" s="82"/>
-      <c r="H22" s="82"/>
+    <row r="21" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="73" t="s">
+        <v>146</v>
+      </c>
+      <c r="C21" s="74"/>
+      <c r="D21" s="75">
+        <f>SUM(D11:D20)</f>
+        <v>263</v>
+      </c>
+      <c r="E21" s="75">
+        <f>SUM(E11:E20)</f>
+        <v>684</v>
+      </c>
+      <c r="F21" s="75">
+        <f>SUM(F11:F20)</f>
+        <v>947</v>
+      </c>
+      <c r="G21" s="75">
+        <f>F21</f>
+        <v>947</v>
+      </c>
+      <c r="H21" s="76" t="s">
+        <v>147</v>
+      </c>
     </row>
-    <row r="23" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="86" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="82"/>
-      <c r="D23" s="82"/>
-      <c r="E23" s="82"/>
-      <c r="F23" s="82"/>
-      <c r="G23" s="82"/>
-      <c r="H23" s="82"/>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B23" s="92" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" s="91"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="91"/>
+      <c r="H23" s="91"/>
     </row>
     <row r="24" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="86" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" s="82"/>
-      <c r="D24" s="82"/>
-      <c r="E24" s="82"/>
-      <c r="F24" s="82"/>
-      <c r="G24" s="82"/>
-      <c r="H24" s="82"/>
+      <c r="B24" s="94" t="s">
+        <v>149</v>
+      </c>
+      <c r="C24" s="91"/>
+      <c r="D24" s="91"/>
+      <c r="E24" s="91"/>
+      <c r="F24" s="91"/>
+      <c r="G24" s="91"/>
+      <c r="H24" s="91"/>
     </row>
     <row r="25" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="86" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" s="82"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
-      <c r="F25" s="82"/>
-      <c r="G25" s="82"/>
-      <c r="H25" s="82"/>
+      <c r="B25" s="94" t="s">
+        <v>150</v>
+      </c>
+      <c r="C25" s="91"/>
+      <c r="D25" s="91"/>
+      <c r="E25" s="91"/>
+      <c r="F25" s="91"/>
+      <c r="G25" s="91"/>
+      <c r="H25" s="91"/>
     </row>
     <row r="26" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="86" t="s">
-        <v>41</v>
-      </c>
-      <c r="C26" s="82"/>
-      <c r="D26" s="82"/>
-      <c r="E26" s="82"/>
-      <c r="F26" s="82"/>
-      <c r="G26" s="82"/>
-      <c r="H26" s="82"/>
+      <c r="B26" s="94" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26" s="91"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="91"/>
+      <c r="F26" s="91"/>
+      <c r="G26" s="91"/>
+      <c r="H26" s="91"/>
+    </row>
+    <row r="27" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="94" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" s="91"/>
+      <c r="D27" s="91"/>
+      <c r="E27" s="91"/>
+      <c r="F27" s="91"/>
+      <c r="G27" s="91"/>
+      <c r="H27" s="91"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -2131,6 +2156,7 @@
     <mergeCell ref="H6:J6"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="B27:H27"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="E5:F5"/>
@@ -2138,7 +2164,6 @@
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="H7:J7"/>
-    <mergeCell ref="B22:H22"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="E6:F6"/>
@@ -2194,28 +2219,28 @@
   <sheetData>
     <row r="3" spans="1:108" ht="21" x14ac:dyDescent="0.3">
       <c r="B3" s="77" t="s">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="D3" s="78">
         <f>+CN79</f>
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="F3" s="79" t="s">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="I3" s="80">
         <f>'Programa CAJAS REPORTE DIARIO'!CH77+CN79</f>
-        <v>921</v>
+        <v>947</v>
       </c>
     </row>
     <row r="10" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A10" s="31"/>
-      <c r="E10" s="95" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="96"/>
-      <c r="G10" s="96"/>
-      <c r="H10" s="96"/>
+      <c r="E10" s="81" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" s="82"/>
+      <c r="G10" s="82"/>
+      <c r="H10" s="82"/>
       <c r="I10" s="1"/>
       <c r="J10" s="14"/>
       <c r="R10" s="2"/>
@@ -2238,78 +2263,78 @@
         <v>18</v>
       </c>
       <c r="U11" s="6"/>
-      <c r="W11" s="97" t="s">
-        <v>45</v>
-      </c>
-      <c r="X11" s="98"/>
-      <c r="Y11" s="98"/>
-      <c r="Z11" s="98"/>
-      <c r="AA11" s="98"/>
-      <c r="AB11" s="98"/>
-      <c r="AC11" s="98"/>
-      <c r="AD11" s="98"/>
-      <c r="AE11" s="98"/>
-      <c r="AF11" s="98"/>
-      <c r="AG11" s="98"/>
-      <c r="AH11" s="98"/>
-      <c r="AI11" s="98"/>
-      <c r="AJ11" s="98"/>
-      <c r="AK11" s="98"/>
-      <c r="AL11" s="98"/>
-      <c r="AM11" s="98"/>
-      <c r="AN11" s="98"/>
-      <c r="AO11" s="98"/>
-      <c r="AP11" s="98"/>
-      <c r="AQ11" s="98"/>
-      <c r="AR11" s="98"/>
-      <c r="AS11" s="98"/>
-      <c r="AT11" s="98"/>
-      <c r="AU11" s="98"/>
-      <c r="AV11" s="98"/>
-      <c r="AW11" s="98"/>
-      <c r="AX11" s="98"/>
-      <c r="AY11" s="98"/>
-      <c r="AZ11" s="98"/>
-      <c r="BA11" s="98"/>
-      <c r="BB11" s="98"/>
-      <c r="BC11" s="98"/>
-      <c r="BD11" s="98"/>
-      <c r="BE11" s="98"/>
-      <c r="BF11" s="98"/>
-      <c r="BG11" s="98"/>
-      <c r="BH11" s="98"/>
-      <c r="BI11" s="98"/>
-      <c r="BJ11" s="98"/>
-      <c r="BK11" s="98"/>
-      <c r="BL11" s="98"/>
-      <c r="BM11" s="98"/>
-      <c r="BN11" s="98"/>
-      <c r="BO11" s="98"/>
-      <c r="BP11" s="98"/>
-      <c r="BQ11" s="98"/>
-      <c r="BR11" s="98"/>
-      <c r="BS11" s="98"/>
-      <c r="BT11" s="98"/>
-      <c r="BU11" s="98"/>
-      <c r="BV11" s="98"/>
-      <c r="BW11" s="98"/>
-      <c r="BX11" s="98"/>
-      <c r="BY11" s="98"/>
-      <c r="BZ11" s="98"/>
-      <c r="CA11" s="98"/>
-      <c r="CB11" s="98"/>
-      <c r="CC11" s="98"/>
-      <c r="CD11" s="98"/>
-      <c r="CE11" s="98"/>
-      <c r="CF11" s="98"/>
-      <c r="CG11" s="98"/>
-      <c r="CH11" s="98"/>
-      <c r="CI11" s="98"/>
-      <c r="CJ11" s="98"/>
-      <c r="CK11" s="98"/>
-      <c r="CL11" s="98"/>
-      <c r="CM11" s="98"/>
-      <c r="CN11" s="99"/>
+      <c r="W11" s="83" t="s">
+        <v>3</v>
+      </c>
+      <c r="X11" s="84"/>
+      <c r="Y11" s="84"/>
+      <c r="Z11" s="84"/>
+      <c r="AA11" s="84"/>
+      <c r="AB11" s="84"/>
+      <c r="AC11" s="84"/>
+      <c r="AD11" s="84"/>
+      <c r="AE11" s="84"/>
+      <c r="AF11" s="84"/>
+      <c r="AG11" s="84"/>
+      <c r="AH11" s="84"/>
+      <c r="AI11" s="84"/>
+      <c r="AJ11" s="84"/>
+      <c r="AK11" s="84"/>
+      <c r="AL11" s="84"/>
+      <c r="AM11" s="84"/>
+      <c r="AN11" s="84"/>
+      <c r="AO11" s="84"/>
+      <c r="AP11" s="84"/>
+      <c r="AQ11" s="84"/>
+      <c r="AR11" s="84"/>
+      <c r="AS11" s="84"/>
+      <c r="AT11" s="84"/>
+      <c r="AU11" s="84"/>
+      <c r="AV11" s="84"/>
+      <c r="AW11" s="84"/>
+      <c r="AX11" s="84"/>
+      <c r="AY11" s="84"/>
+      <c r="AZ11" s="84"/>
+      <c r="BA11" s="84"/>
+      <c r="BB11" s="84"/>
+      <c r="BC11" s="84"/>
+      <c r="BD11" s="84"/>
+      <c r="BE11" s="84"/>
+      <c r="BF11" s="84"/>
+      <c r="BG11" s="84"/>
+      <c r="BH11" s="84"/>
+      <c r="BI11" s="84"/>
+      <c r="BJ11" s="84"/>
+      <c r="BK11" s="84"/>
+      <c r="BL11" s="84"/>
+      <c r="BM11" s="84"/>
+      <c r="BN11" s="84"/>
+      <c r="BO11" s="84"/>
+      <c r="BP11" s="84"/>
+      <c r="BQ11" s="84"/>
+      <c r="BR11" s="84"/>
+      <c r="BS11" s="84"/>
+      <c r="BT11" s="84"/>
+      <c r="BU11" s="84"/>
+      <c r="BV11" s="84"/>
+      <c r="BW11" s="84"/>
+      <c r="BX11" s="84"/>
+      <c r="BY11" s="84"/>
+      <c r="BZ11" s="84"/>
+      <c r="CA11" s="84"/>
+      <c r="CB11" s="84"/>
+      <c r="CC11" s="84"/>
+      <c r="CD11" s="84"/>
+      <c r="CE11" s="84"/>
+      <c r="CF11" s="84"/>
+      <c r="CG11" s="84"/>
+      <c r="CH11" s="84"/>
+      <c r="CI11" s="84"/>
+      <c r="CJ11" s="84"/>
+      <c r="CK11" s="84"/>
+      <c r="CL11" s="84"/>
+      <c r="CM11" s="84"/>
+      <c r="CN11" s="85"/>
       <c r="CP11" s="29"/>
       <c r="CQ11" s="29"/>
       <c r="CR11" s="29"/>
@@ -2324,38 +2349,38 @@
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="61"/>
-      <c r="E12" s="100" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" s="101"/>
-      <c r="G12" s="101"/>
-      <c r="H12" s="101"/>
-      <c r="I12" s="101"/>
-      <c r="J12" s="101"/>
+      <c r="E12" s="86" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="87"/>
+      <c r="G12" s="87"/>
+      <c r="H12" s="87"/>
+      <c r="I12" s="87"/>
+      <c r="J12" s="87"/>
       <c r="L12" s="36" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="N12" s="36" t="s">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="O12" s="36" t="s">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="P12" s="36" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="R12" s="8" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="S12" s="9"/>
       <c r="T12" s="8" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="U12" s="8" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="W12" s="26">
         <v>46307</v>
@@ -2565,63 +2590,63 @@
         <v>46375</v>
       </c>
       <c r="CN12" s="28" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="CP12" s="29" t="s">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="CQ12" s="29" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="CR12" s="29" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="CS12" s="29" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="CT12" s="29" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="CU12" s="29" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="CV12" s="29" t="s">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="CW12" s="29" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:108" s="12" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="B13" s="45" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="E13" s="62" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="F13" s="62" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="G13" s="62" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="H13" s="62" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="I13" s="62" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="J13" s="62" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="L13" s="11">
         <v>0</v>
@@ -2698,11 +2723,11 @@
       </c>
       <c r="AI13" s="23">
         <f t="shared" si="0"/>
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="AJ13" s="23">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="AK13" s="23">
         <f t="shared" si="0"/>
@@ -2926,7 +2951,7 @@
       </c>
       <c r="CN13" s="37">
         <f t="shared" si="2"/>
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="CP13" s="39"/>
       <c r="CQ13" s="40"/>
@@ -2937,36 +2962,36 @@
       <c r="CV13" s="29"/>
       <c r="CW13" s="29"/>
       <c r="CY13" s="65" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="CZ13" s="65" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="DA13" s="65" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="DB13" s="65" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="DC13" s="65" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="DD13" s="65" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B14" s="46" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="C14" s="47" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E14" s="13">
         <v>322</v>
@@ -3102,14 +3127,14 @@
     </row>
     <row r="15" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B15" s="48"/>
       <c r="C15" s="47" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E15" s="13">
         <v>756</v>
@@ -3245,14 +3270,14 @@
     </row>
     <row r="16" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A16" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B16" s="48"/>
       <c r="C16" s="47" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E16" s="13">
         <v>572</v>
@@ -3390,14 +3415,14 @@
     </row>
     <row r="17" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B17" s="48"/>
       <c r="C17" s="47" t="s">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E17" s="13">
         <v>192</v>
@@ -3533,14 +3558,14 @@
     </row>
     <row r="18" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A18" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B18" s="48"/>
       <c r="C18" s="47" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E18" s="13">
         <v>636</v>
@@ -3678,14 +3703,14 @@
     </row>
     <row r="19" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B19" s="48"/>
       <c r="C19" s="47" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E19" s="13">
         <v>1392</v>
@@ -3823,14 +3848,14 @@
     </row>
     <row r="20" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A20" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B20" s="48"/>
       <c r="C20" s="47" t="s">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="D20" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E20" s="13">
         <v>308</v>
@@ -3968,14 +3993,14 @@
     </row>
     <row r="21" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A21" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B21" s="48"/>
       <c r="C21" s="47" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="D21" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E21" s="13">
         <v>2132</v>
@@ -4113,14 +4138,14 @@
     </row>
     <row r="22" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A22" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B22" s="48"/>
       <c r="C22" s="47" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="D22" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E22" s="13">
         <v>437</v>
@@ -4256,14 +4281,14 @@
     </row>
     <row r="23" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A23" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B23" s="48"/>
       <c r="C23" s="47" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="D23" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E23" s="13">
         <v>79</v>
@@ -4399,14 +4424,14 @@
     </row>
     <row r="24" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A24" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B24" s="48"/>
       <c r="C24" s="47" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="D24" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E24" s="13">
         <v>374</v>
@@ -4542,14 +4567,14 @@
     </row>
     <row r="25" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A25" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B25" s="48"/>
       <c r="C25" s="47" t="s">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="D25" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E25" s="13">
         <v>418</v>
@@ -4687,14 +4712,14 @@
     </row>
     <row r="26" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B26" s="49"/>
       <c r="C26" s="47" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="D26" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E26" s="13">
         <v>363</v>
@@ -4832,16 +4857,16 @@
     </row>
     <row r="27" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A27" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B27" s="50" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="C27" s="47" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="D27" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E27" s="13">
         <v>2353</v>
@@ -4996,16 +5021,16 @@
     </row>
     <row r="28" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A28" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B28" s="50" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="C28" s="47" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="D28" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E28" s="13">
         <v>1107</v>
@@ -5157,13 +5182,13 @@
         <v>1</v>
       </c>
       <c r="B29" s="58" t="s">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E29" s="13">
         <v>686</v>
@@ -5209,11 +5234,9 @@
       <c r="AH29" s="24">
         <v>15</v>
       </c>
-      <c r="AI29" s="24">
-        <v>9</v>
-      </c>
+      <c r="AI29" s="24"/>
       <c r="AJ29" s="24">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AK29" s="24"/>
       <c r="AL29" s="24"/>
@@ -5272,43 +5295,43 @@
       <c r="CM29" s="24"/>
       <c r="CN29" s="37">
         <f t="shared" si="3"/>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="CP29" s="27">
         <f t="shared" si="4"/>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="CQ29" s="22">
         <v>0</v>
       </c>
       <c r="CR29" s="22">
         <f t="shared" si="5"/>
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="CS29" s="42"/>
       <c r="CT29" s="44"/>
       <c r="CU29" s="14">
         <f t="shared" si="6"/>
-        <v>1228</v>
+        <v>812</v>
       </c>
       <c r="CV29" s="14">
         <f t="shared" si="7"/>
-        <v>614</v>
+        <v>406</v>
       </c>
       <c r="CW29" s="14">
         <f t="shared" si="8"/>
-        <v>574</v>
+        <v>383</v>
       </c>
       <c r="CX29" s="43"/>
       <c r="CY29" s="17">
-        <v>1156</v>
+        <v>740</v>
       </c>
       <c r="CZ29">
         <v>72</v>
       </c>
       <c r="DD29" s="14">
         <f t="shared" si="9"/>
-        <v>1228</v>
+        <v>812</v>
       </c>
     </row>
     <row r="30" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -5317,10 +5340,10 @@
       </c>
       <c r="B30" s="60"/>
       <c r="C30" s="47" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="D30" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E30" s="13">
         <v>74</v>
@@ -5364,7 +5387,9 @@
       <c r="AG30" s="24"/>
       <c r="AH30" s="24"/>
       <c r="AI30" s="24"/>
-      <c r="AJ30" s="24"/>
+      <c r="AJ30" s="24">
+        <v>35</v>
+      </c>
       <c r="AK30" s="24"/>
       <c r="AL30" s="24"/>
       <c r="AM30" s="24"/>
@@ -5422,18 +5447,18 @@
       <c r="CM30" s="24"/>
       <c r="CN30" s="37">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="CP30" s="27">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="CQ30" s="22">
         <v>0</v>
       </c>
       <c r="CR30" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="CS30" s="42"/>
       <c r="CT30" s="44"/>
@@ -5447,7 +5472,7 @@
       </c>
       <c r="CW30" s="14">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>-33</v>
       </c>
       <c r="CX30" s="43"/>
       <c r="CY30" s="17"/>
@@ -5465,10 +5490,10 @@
       </c>
       <c r="B31" s="59"/>
       <c r="C31" s="47" t="s">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="D31" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E31" s="13">
         <v>321</v>
@@ -5609,13 +5634,13 @@
         <v>2</v>
       </c>
       <c r="B32" s="58" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="C32" s="47" t="s">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="D32" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E32" s="13">
         <v>2</v>
@@ -5729,23 +5754,23 @@
       <c r="CT32" s="44"/>
       <c r="CU32" s="14">
         <f t="shared" si="6"/>
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="CV32" s="14">
         <f t="shared" si="7"/>
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="CW32" s="14">
         <f t="shared" si="8"/>
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="CX32" s="43"/>
       <c r="CY32" s="17">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="DD32" s="14">
         <f t="shared" si="9"/>
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33" spans="1:108" x14ac:dyDescent="0.3">
@@ -5754,10 +5779,10 @@
       </c>
       <c r="B33" s="60"/>
       <c r="C33" s="47" t="s">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E33" s="13">
         <v>862</v>
@@ -5897,10 +5922,10 @@
       </c>
       <c r="B34" s="59"/>
       <c r="C34" s="47" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="D34" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E34" s="13">
         <v>661</v>
@@ -6040,13 +6065,13 @@
         <v>4</v>
       </c>
       <c r="B35" s="50" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="C35" s="47" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="D35" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E35" s="13">
         <v>123</v>
@@ -6185,13 +6210,13 @@
         <v>5</v>
       </c>
       <c r="B36" s="50" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C36" s="47" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="D36" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E36" s="13">
         <v>144</v>
@@ -6330,13 +6355,13 @@
         <v>6</v>
       </c>
       <c r="B37" s="50" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="C37" s="47" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="D37" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E37" s="13">
         <v>2632</v>
@@ -6475,13 +6500,13 @@
         <v>8</v>
       </c>
       <c r="B38" s="50" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="C38" s="47" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="D38" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E38" s="13">
         <v>978</v>
@@ -6620,13 +6645,13 @@
         <v>9</v>
       </c>
       <c r="B39" s="50" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="C39" s="47" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E39" s="13">
         <v>276</v>
@@ -6765,13 +6790,13 @@
         <v>10</v>
       </c>
       <c r="B40" s="50" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="C40" s="47" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="D40" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E40" s="13">
         <v>107</v>
@@ -6909,13 +6934,13 @@
         <v>12</v>
       </c>
       <c r="B41" s="50" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C41" s="47" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E41" s="13">
         <v>1267</v>
@@ -7054,13 +7079,13 @@
         <v>13</v>
       </c>
       <c r="B42" s="50" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="C42" s="47" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E42" s="13">
         <v>1218</v>
@@ -7199,13 +7224,13 @@
         <v>14</v>
       </c>
       <c r="B43" s="50" t="s">
-        <v>108</v>
+        <v>66</v>
       </c>
       <c r="C43" s="47" t="s">
-        <v>108</v>
+        <v>66</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E43" s="13">
         <v>1734</v>
@@ -7344,13 +7369,13 @@
         <v>15</v>
       </c>
       <c r="B44" s="50" t="s">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="C44" s="47" t="s">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="D44" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E44" s="13">
         <v>1716</v>
@@ -7489,13 +7514,13 @@
         <v>18</v>
       </c>
       <c r="B45" s="50" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="C45" s="47" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="D45" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E45" s="13">
         <v>222</v>
@@ -7634,13 +7659,13 @@
         <v>19</v>
       </c>
       <c r="B46" s="50" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="C46" s="47" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="D46" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E46" s="13">
         <v>938</v>
@@ -7781,13 +7806,13 @@
         <v>20</v>
       </c>
       <c r="B47" s="58" t="s">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="C47" s="47" t="s">
-        <v>113</v>
+        <v>71</v>
       </c>
       <c r="D47" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E47" s="13">
         <v>749</v>
@@ -7927,10 +7952,10 @@
       </c>
       <c r="B48" s="59"/>
       <c r="C48" s="47" t="s">
-        <v>114</v>
+        <v>72</v>
       </c>
       <c r="D48" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E48" s="13">
         <v>2252</v>
@@ -8047,24 +8072,21 @@
       <c r="CT48" s="44"/>
       <c r="CU48" s="14">
         <f t="shared" si="13"/>
-        <v>154</v>
+        <v>0</v>
       </c>
       <c r="CV48" s="14">
         <f t="shared" si="14"/>
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="CW48" s="14">
         <f t="shared" si="15"/>
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="CX48" s="43"/>
       <c r="CY48" s="17"/>
-      <c r="CZ48">
-        <v>154</v>
-      </c>
       <c r="DD48" s="14">
         <f t="shared" si="16"/>
-        <v>154</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:108" x14ac:dyDescent="0.3">
@@ -8072,13 +8094,13 @@
         <v>21</v>
       </c>
       <c r="B49" s="50" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="C49" s="47" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D49" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E49" s="13">
         <v>587</v>
@@ -8217,13 +8239,13 @@
         <v>22</v>
       </c>
       <c r="B50" s="50" t="s">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="C50" s="47" t="s">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="D50" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E50" s="13">
         <v>1932</v>
@@ -8361,13 +8383,13 @@
         <v>23</v>
       </c>
       <c r="B51" s="50" t="s">
-        <v>117</v>
+        <v>75</v>
       </c>
       <c r="C51" s="47" t="s">
-        <v>117</v>
+        <v>75</v>
       </c>
       <c r="D51" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E51" s="13">
         <v>2498</v>
@@ -8508,13 +8530,13 @@
         <v>24</v>
       </c>
       <c r="B52" s="50" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="C52" s="47" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="D52" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E52" s="13">
         <v>566</v>
@@ -8653,13 +8675,13 @@
         <v>26</v>
       </c>
       <c r="B53" s="50" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="C53" s="47" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="D53" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E53" s="13">
         <v>852</v>
@@ -8798,13 +8820,13 @@
         <v>27</v>
       </c>
       <c r="B54" s="50" t="s">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="C54" s="47" t="s">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="D54" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E54" s="13">
         <v>96</v>
@@ -8943,13 +8965,13 @@
         <v>28</v>
       </c>
       <c r="B55" s="50" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="C55" s="47" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D55" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E55" s="13">
         <v>496</v>
@@ -9088,13 +9110,13 @@
         <v>29</v>
       </c>
       <c r="B56" s="50" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="C56" s="47" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="D56" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E56" s="13">
         <v>1435</v>
@@ -9233,13 +9255,13 @@
         <v>30</v>
       </c>
       <c r="B57" s="46" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="C57" s="51" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="D57" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E57" s="13">
         <v>320</v>
@@ -9378,13 +9400,13 @@
         <v>31</v>
       </c>
       <c r="B58" s="49" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="C58" s="51" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="D58" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E58" s="13">
         <v>1021</v>
@@ -9525,13 +9547,13 @@
         <v>31</v>
       </c>
       <c r="B59" s="50" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C59" s="47" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="D59" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E59" s="13">
         <v>474</v>
@@ -9672,13 +9694,13 @@
         <v>32</v>
       </c>
       <c r="B60" s="50" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="C60" s="47" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="D60" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E60" s="13">
         <v>338</v>
@@ -9819,13 +9841,13 @@
         <v>33</v>
       </c>
       <c r="B61" s="50" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="C61" s="47" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="D61" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E61" s="13">
         <v>361</v>
@@ -9964,13 +9986,13 @@
         <v>34</v>
       </c>
       <c r="B62" s="50" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="C62" s="47" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="D62" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E62" s="13">
         <v>724</v>
@@ -10111,13 +10133,13 @@
         <v>35</v>
       </c>
       <c r="B63" s="50" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="C63" s="47" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="D63" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E63" s="13">
         <v>565</v>
@@ -10256,13 +10278,13 @@
         <v>36</v>
       </c>
       <c r="B64" s="50" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="C64" s="47" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="D64" s="33" t="s">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="E64" s="13">
         <v>583</v>
@@ -10403,13 +10425,13 @@
         <v>37</v>
       </c>
       <c r="B65" s="50" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="C65" s="47" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="D65" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E65" s="13">
         <v>907</v>
@@ -10547,13 +10569,13 @@
         <v>38</v>
       </c>
       <c r="B66" s="50" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="C66" s="47" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="D66" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E66" s="13">
         <v>857</v>
@@ -10694,13 +10716,13 @@
         <v>39</v>
       </c>
       <c r="B67" s="50" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="C67" s="47" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="D67" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E67" s="13">
         <v>719</v>
@@ -10839,13 +10861,13 @@
         <v>44</v>
       </c>
       <c r="B68" s="50" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="C68" s="47" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="D68" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E68" s="13">
         <v>53</v>
@@ -10982,13 +11004,13 @@
         <v>45</v>
       </c>
       <c r="B69" s="50" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="C69" s="47" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="D69" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E69" s="13">
         <v>419</v>
@@ -11129,13 +11151,13 @@
         <v>47</v>
       </c>
       <c r="B70" s="50" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
       <c r="C70" s="47" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
       <c r="D70" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E70" s="13">
         <v>441</v>
@@ -11274,13 +11296,13 @@
         <v>48</v>
       </c>
       <c r="B71" s="50" t="s">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="C71" s="47" t="s">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="D71" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E71" s="13">
         <v>1179</v>
@@ -11416,16 +11438,16 @@
     </row>
     <row r="72" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B72" s="50" t="s">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="C72" s="47" t="s">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="D72" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E72" s="13">
         <v>947</v>
@@ -11561,16 +11583,16 @@
     </row>
     <row r="73" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A73" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B73" s="50" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="C73" s="47" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="D73" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E73" s="13">
         <v>48</v>
@@ -11706,16 +11728,16 @@
     </row>
     <row r="74" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B74" s="50" t="s">
-        <v>142</v>
+        <v>100</v>
       </c>
       <c r="C74" s="47" t="s">
-        <v>142</v>
+        <v>100</v>
       </c>
       <c r="D74" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E74" s="13">
         <v>1152</v>
@@ -11851,16 +11873,16 @@
     </row>
     <row r="75" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A75" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B75" s="50" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="C75" s="47" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="D75" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E75" s="13">
         <v>1418</v>
@@ -11998,16 +12020,16 @@
     </row>
     <row r="76" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B76" s="50" t="s">
-        <v>144</v>
+        <v>102</v>
       </c>
       <c r="C76" s="47" t="s">
-        <v>144</v>
+        <v>102</v>
       </c>
       <c r="D76" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E76" s="13">
         <v>1066</v>
@@ -12143,16 +12165,16 @@
     </row>
     <row r="77" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B77" s="50" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="C77" s="47" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="D77" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E77" s="13">
         <v>825</v>
@@ -12288,16 +12310,16 @@
     </row>
     <row r="78" spans="1:108" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A78" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B78" s="50" t="s">
-        <v>146</v>
+        <v>104</v>
       </c>
       <c r="C78" s="47" t="s">
-        <v>146</v>
+        <v>104</v>
       </c>
       <c r="D78" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E78" s="13">
         <v>82</v>
@@ -12432,7 +12454,7 @@
     <row r="79" spans="1:108" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A79" s="18"/>
       <c r="B79" s="18" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="C79" s="18"/>
       <c r="D79" s="18"/>
@@ -12528,11 +12550,11 @@
       </c>
       <c r="AI79" s="25">
         <f t="shared" si="22"/>
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="AJ79" s="25">
         <f t="shared" si="22"/>
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="AK79" s="25">
         <f t="shared" si="22"/>
@@ -12756,11 +12778,11 @@
       </c>
       <c r="CN79" s="25">
         <f t="shared" si="24"/>
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="CP79" s="25">
         <f>+SUM(CP14:CP78)</f>
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="CQ79" s="25">
         <f>+SUM(CQ14:CQ78)</f>
@@ -12768,21 +12790,21 @@
       </c>
       <c r="CR79" s="25">
         <f>+SUM(CR14:CR78)</f>
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="CS79" s="25"/>
       <c r="CT79" s="25"/>
       <c r="CU79" s="25">
         <f>+SUM(CU14:CU78)</f>
-        <v>5077</v>
+        <v>4499</v>
       </c>
       <c r="CV79" s="25">
         <f>+SUM(CV14:CV78)</f>
-        <v>2538.5</v>
+        <v>2249.5</v>
       </c>
       <c r="CW79" s="25">
         <f>+SUM(CW14:CW78)</f>
-        <v>2293.5</v>
+        <v>1986.5</v>
       </c>
     </row>
     <row r="80" spans="1:108" hidden="1" x14ac:dyDescent="0.3">
@@ -12864,7 +12886,7 @@
     </row>
     <row r="81" spans="1:101" hidden="1" x14ac:dyDescent="0.3">
       <c r="B81" s="53" t="s">
-        <v>147</v>
+        <v>105</v>
       </c>
       <c r="C81" s="54"/>
       <c r="D81" s="54"/>
@@ -12952,7 +12974,7 @@
       <c r="CL81" s="30"/>
       <c r="CM81" s="30"/>
       <c r="CN81" s="53" t="s">
-        <v>147</v>
+        <v>105</v>
       </c>
       <c r="CP81" s="53"/>
       <c r="CQ81" s="53"/>
@@ -12961,13 +12983,13 @@
     <row r="82" spans="1:101" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="33"/>
       <c r="B82" s="50" t="s">
-        <v>148</v>
+        <v>106</v>
       </c>
       <c r="C82" s="47" t="s">
-        <v>148</v>
+        <v>106</v>
       </c>
       <c r="D82" s="33" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="E82" s="13"/>
       <c r="F82" s="13"/>
@@ -13082,13 +13104,13 @@
     <row r="83" spans="1:101" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="33"/>
       <c r="B83" s="50" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="C83" s="47" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="D83" s="33" t="s">
-        <v>151</v>
+        <v>109</v>
       </c>
       <c r="E83" s="13"/>
       <c r="F83" s="13"/>
@@ -13204,13 +13226,13 @@
     <row r="84" spans="1:101" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="33"/>
       <c r="B84" s="50" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="C84" s="47" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="D84" s="33" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="E84" s="13"/>
       <c r="F84" s="13"/>
@@ -13326,7 +13348,7 @@
     <row r="85" spans="1:101" ht="15.75" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A85" s="18"/>
       <c r="B85" s="18" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="C85" s="18"/>
       <c r="D85" s="18"/>
@@ -13776,7 +13798,7 @@
     </row>
     <row r="89" spans="1:101" x14ac:dyDescent="0.3">
       <c r="B89" s="53" t="s">
-        <v>147</v>
+        <v>105</v>
       </c>
       <c r="C89" s="54"/>
       <c r="D89" s="54"/>
@@ -13872,13 +13894,13 @@
         <v>17</v>
       </c>
       <c r="B90" s="50" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="C90" s="47" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="D90" s="33" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="E90" s="13"/>
       <c r="F90" s="13"/>
@@ -13909,13 +13931,13 @@
         <v>25</v>
       </c>
       <c r="B91" s="50" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="C91" s="47" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="D91" s="33" t="s">
-        <v>151</v>
+        <v>109</v>
       </c>
       <c r="E91" s="13"/>
       <c r="F91" s="13"/>
@@ -13946,13 +13968,13 @@
         <v>43</v>
       </c>
       <c r="B92" s="50" t="s">
-        <v>148</v>
+        <v>106</v>
       </c>
       <c r="C92" s="47" t="s">
-        <v>148</v>
+        <v>106</v>
       </c>
       <c r="D92" s="33" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="E92" s="13"/>
       <c r="F92" s="13"/>
@@ -13980,7 +14002,7 @@
     <row r="93" spans="1:101" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A93" s="18"/>
       <c r="B93" s="18" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="C93" s="18"/>
       <c r="D93" s="18"/>
@@ -14040,7 +14062,6 @@
       <c r="V93" s="20"/>
     </row>
   </sheetData>
-  <autoFilter ref="A13:CW79" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="3">
     <mergeCell ref="E10:H10"/>
     <mergeCell ref="W11:CN11"/>
@@ -14117,24 +14138,24 @@
       </c>
       <c r="D3" s="78">
         <f>+CH77</f>
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="F3" s="79" t="s">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="I3" s="80">
         <f>'Programa CASETAS REPORTE DIARIO'!CN79+CH77</f>
-        <v>921</v>
+        <v>947</v>
       </c>
     </row>
     <row r="10" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A10" s="31"/>
-      <c r="E10" s="95" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="96"/>
-      <c r="G10" s="96"/>
-      <c r="H10" s="96"/>
+      <c r="E10" s="81" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" s="82"/>
+      <c r="G10" s="82"/>
+      <c r="H10" s="82"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -14170,66 +14191,66 @@
         <v>15</v>
       </c>
       <c r="AA11" s="6"/>
-      <c r="AC11" s="97" t="s">
+      <c r="AC11" s="83" t="s">
         <v>154</v>
       </c>
-      <c r="AD11" s="98"/>
-      <c r="AE11" s="98"/>
-      <c r="AF11" s="98"/>
-      <c r="AG11" s="98"/>
-      <c r="AH11" s="98"/>
-      <c r="AI11" s="98"/>
-      <c r="AJ11" s="98"/>
-      <c r="AK11" s="98"/>
-      <c r="AL11" s="98"/>
-      <c r="AM11" s="98"/>
-      <c r="AN11" s="98"/>
-      <c r="AO11" s="98"/>
-      <c r="AP11" s="98"/>
-      <c r="AQ11" s="98"/>
-      <c r="AR11" s="98"/>
-      <c r="AS11" s="98"/>
-      <c r="AT11" s="98"/>
-      <c r="AU11" s="98"/>
-      <c r="AV11" s="98"/>
-      <c r="AW11" s="98"/>
-      <c r="AX11" s="98"/>
-      <c r="AY11" s="98"/>
-      <c r="AZ11" s="98"/>
-      <c r="BA11" s="98"/>
-      <c r="BB11" s="98"/>
-      <c r="BC11" s="98"/>
-      <c r="BD11" s="98"/>
-      <c r="BE11" s="98"/>
-      <c r="BF11" s="98"/>
-      <c r="BG11" s="98"/>
-      <c r="BH11" s="98"/>
-      <c r="BI11" s="98"/>
-      <c r="BJ11" s="98"/>
-      <c r="BK11" s="98"/>
-      <c r="BL11" s="98"/>
-      <c r="BM11" s="98"/>
-      <c r="BN11" s="98"/>
-      <c r="BO11" s="98"/>
-      <c r="BP11" s="98"/>
-      <c r="BQ11" s="98"/>
-      <c r="BR11" s="98"/>
-      <c r="BS11" s="98"/>
-      <c r="BT11" s="98"/>
-      <c r="BU11" s="98"/>
-      <c r="BV11" s="98"/>
-      <c r="BW11" s="98"/>
-      <c r="BX11" s="98"/>
-      <c r="BY11" s="98"/>
-      <c r="BZ11" s="98"/>
-      <c r="CA11" s="98"/>
-      <c r="CB11" s="98"/>
-      <c r="CC11" s="98"/>
-      <c r="CD11" s="98"/>
-      <c r="CE11" s="98"/>
-      <c r="CF11" s="98"/>
-      <c r="CG11" s="98"/>
-      <c r="CH11" s="99"/>
+      <c r="AD11" s="84"/>
+      <c r="AE11" s="84"/>
+      <c r="AF11" s="84"/>
+      <c r="AG11" s="84"/>
+      <c r="AH11" s="84"/>
+      <c r="AI11" s="84"/>
+      <c r="AJ11" s="84"/>
+      <c r="AK11" s="84"/>
+      <c r="AL11" s="84"/>
+      <c r="AM11" s="84"/>
+      <c r="AN11" s="84"/>
+      <c r="AO11" s="84"/>
+      <c r="AP11" s="84"/>
+      <c r="AQ11" s="84"/>
+      <c r="AR11" s="84"/>
+      <c r="AS11" s="84"/>
+      <c r="AT11" s="84"/>
+      <c r="AU11" s="84"/>
+      <c r="AV11" s="84"/>
+      <c r="AW11" s="84"/>
+      <c r="AX11" s="84"/>
+      <c r="AY11" s="84"/>
+      <c r="AZ11" s="84"/>
+      <c r="BA11" s="84"/>
+      <c r="BB11" s="84"/>
+      <c r="BC11" s="84"/>
+      <c r="BD11" s="84"/>
+      <c r="BE11" s="84"/>
+      <c r="BF11" s="84"/>
+      <c r="BG11" s="84"/>
+      <c r="BH11" s="84"/>
+      <c r="BI11" s="84"/>
+      <c r="BJ11" s="84"/>
+      <c r="BK11" s="84"/>
+      <c r="BL11" s="84"/>
+      <c r="BM11" s="84"/>
+      <c r="BN11" s="84"/>
+      <c r="BO11" s="84"/>
+      <c r="BP11" s="84"/>
+      <c r="BQ11" s="84"/>
+      <c r="BR11" s="84"/>
+      <c r="BS11" s="84"/>
+      <c r="BT11" s="84"/>
+      <c r="BU11" s="84"/>
+      <c r="BV11" s="84"/>
+      <c r="BW11" s="84"/>
+      <c r="BX11" s="84"/>
+      <c r="BY11" s="84"/>
+      <c r="BZ11" s="84"/>
+      <c r="CA11" s="84"/>
+      <c r="CB11" s="84"/>
+      <c r="CC11" s="84"/>
+      <c r="CD11" s="84"/>
+      <c r="CE11" s="84"/>
+      <c r="CF11" s="84"/>
+      <c r="CG11" s="84"/>
+      <c r="CH11" s="85"/>
       <c r="CJ11" s="29"/>
       <c r="CK11" s="29"/>
       <c r="CL11" s="29"/>
@@ -14244,44 +14265,44 @@
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
-      <c r="E12" s="100" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="101"/>
-      <c r="G12" s="101"/>
-      <c r="H12" s="101"/>
-      <c r="I12" s="101"/>
-      <c r="J12" s="101"/>
-      <c r="K12" s="101"/>
-      <c r="L12" s="101"/>
-      <c r="M12" s="101"/>
-      <c r="N12" s="101"/>
-      <c r="O12" s="101"/>
-      <c r="P12" s="101"/>
+      <c r="E12" s="86" t="s">
+        <v>123</v>
+      </c>
+      <c r="F12" s="87"/>
+      <c r="G12" s="87"/>
+      <c r="H12" s="87"/>
+      <c r="I12" s="87"/>
+      <c r="J12" s="87"/>
+      <c r="K12" s="87"/>
+      <c r="L12" s="87"/>
+      <c r="M12" s="87"/>
+      <c r="N12" s="87"/>
+      <c r="O12" s="87"/>
+      <c r="P12" s="87"/>
       <c r="R12" s="36" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="S12" s="36" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="T12" s="36" t="s">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="U12" s="36" t="s">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="V12" s="36" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="X12" s="8" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="Y12" s="9"/>
       <c r="Z12" s="8" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="AA12" s="8" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="AC12" s="26">
         <v>46307</v>
@@ -14455,31 +14476,31 @@
         <v>46363</v>
       </c>
       <c r="CH12" s="28" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="CJ12" s="29" t="s">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="CK12" s="29" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="CL12" s="29" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="CM12" s="29" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="CN12" s="29" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="CO12" s="29" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="CP12" s="29" t="s">
         <v>155</v>
       </c>
       <c r="CQ12" s="29" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="CS12" s="29" t="s">
         <v>156</v>
@@ -14514,16 +14535,16 @@
     </row>
     <row r="13" spans="1:107" s="12" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>158</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="D13" s="57" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="E13" s="57" t="s">
         <v>159</v>
@@ -14559,7 +14580,7 @@
         <v>169</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="R13" s="11">
         <v>0</v>
@@ -14637,11 +14658,11 @@
       </c>
       <c r="AO13" s="38">
         <f t="shared" si="0"/>
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="AP13" s="38">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="AQ13" s="38">
         <f t="shared" si="0"/>
@@ -14817,7 +14838,7 @@
       </c>
       <c r="CH13" s="38">
         <f t="shared" si="1"/>
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="CJ13" s="39"/>
       <c r="CK13" s="40"/>
@@ -14858,21 +14879,21 @@
         <v>168</v>
       </c>
       <c r="DC13" s="66" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B14" s="46" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="C14" s="56" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E14" s="13">
         <v>71</v>
@@ -15016,14 +15037,14 @@
     </row>
     <row r="15" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B15" s="48"/>
       <c r="C15" s="56" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E15" s="13">
         <v>84</v>
@@ -15169,14 +15190,14 @@
     </row>
     <row r="16" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A16" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B16" s="48"/>
       <c r="C16" s="56" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E16" s="13">
         <v>92</v>
@@ -15322,14 +15343,14 @@
     </row>
     <row r="17" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B17" s="48"/>
       <c r="C17" s="56" t="s">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E17" s="13">
         <v>188</v>
@@ -15475,14 +15496,14 @@
     </row>
     <row r="18" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A18" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B18" s="48"/>
       <c r="C18" s="56" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E18" s="13">
         <v>81</v>
@@ -15628,14 +15649,14 @@
     </row>
     <row r="19" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B19" s="48"/>
       <c r="C19" s="56" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E19" s="13">
         <v>23</v>
@@ -15781,14 +15802,14 @@
     </row>
     <row r="20" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A20" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B20" s="48"/>
       <c r="C20" s="56" t="s">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="D20" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E20" s="13">
         <v>16</v>
@@ -15934,14 +15955,14 @@
     </row>
     <row r="21" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A21" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B21" s="48"/>
       <c r="C21" s="56" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="D21" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E21" s="13">
         <v>91</v>
@@ -16085,14 +16106,14 @@
     </row>
     <row r="22" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A22" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B22" s="48"/>
       <c r="C22" s="56" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="D22" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E22" s="13">
         <v>56</v>
@@ -16238,14 +16259,14 @@
     </row>
     <row r="23" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A23" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B23" s="48"/>
       <c r="C23" s="56" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="D23" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E23" s="13">
         <v>60</v>
@@ -16389,14 +16410,14 @@
     </row>
     <row r="24" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A24" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B24" s="48"/>
       <c r="C24" s="56" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="D24" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E24" s="13">
         <v>80</v>
@@ -16540,14 +16561,14 @@
     </row>
     <row r="25" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B25" s="48"/>
       <c r="C25" s="56" t="s">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="D25" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E25" s="13">
         <v>35</v>
@@ -16693,14 +16714,14 @@
     </row>
     <row r="26" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A26" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B26" s="49"/>
       <c r="C26" s="56" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="D26" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E26" s="13">
         <v>31</v>
@@ -16845,16 +16866,16 @@
     </row>
     <row r="27" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A27" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B27" s="50" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="C27" s="56" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="D27" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E27" s="13">
         <v>74</v>
@@ -17024,16 +17045,16 @@
     </row>
     <row r="28" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="33" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="B28" s="50" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="C28" s="56" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="D28" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E28" s="13">
         <v>67</v>
@@ -17105,7 +17126,7 @@
         <v>29</v>
       </c>
       <c r="AO28" s="24">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AP28" s="24"/>
       <c r="AQ28" s="24"/>
@@ -17153,32 +17174,32 @@
       <c r="CG28" s="24"/>
       <c r="CH28" s="37">
         <f t="shared" si="2"/>
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="CJ28" s="27">
         <f t="shared" si="3"/>
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="CK28" s="22">
         <v>0</v>
       </c>
       <c r="CL28" s="22">
         <f t="shared" si="4"/>
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="CM28" s="42"/>
       <c r="CN28" s="44"/>
       <c r="CO28" s="14">
         <f t="shared" si="5"/>
-        <v>1931</v>
+        <v>178</v>
       </c>
       <c r="CP28" s="14">
         <f t="shared" si="6"/>
-        <v>1931</v>
+        <v>178</v>
       </c>
       <c r="CQ28" s="14">
         <f t="shared" si="7"/>
-        <v>1826</v>
+        <v>77</v>
       </c>
       <c r="CR28" s="43"/>
       <c r="CS28" s="17">
@@ -17191,10 +17212,10 @@
         <v>5</v>
       </c>
       <c r="CX28">
-        <v>642</v>
+        <v>8</v>
       </c>
       <c r="CY28">
-        <v>1135</v>
+        <v>16</v>
       </c>
       <c r="CZ28">
         <v>17</v>
@@ -17204,7 +17225,7 @@
       </c>
       <c r="DC28" s="14">
         <f t="shared" si="8"/>
-        <v>1931</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -17212,13 +17233,13 @@
         <v>1</v>
       </c>
       <c r="B29" s="58" t="s">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="C29" s="56" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E29" s="13">
         <v>22</v>
@@ -17287,10 +17308,10 @@
       <c r="AN29" s="24">
         <v>3</v>
       </c>
-      <c r="AO29" s="24">
-        <v>9</v>
-      </c>
-      <c r="AP29" s="24"/>
+      <c r="AO29" s="24"/>
+      <c r="AP29" s="24">
+        <v>15</v>
+      </c>
       <c r="AQ29" s="24"/>
       <c r="AR29" s="24"/>
       <c r="AS29" s="24"/>
@@ -17336,47 +17357,44 @@
       <c r="CG29" s="24"/>
       <c r="CH29" s="37">
         <f t="shared" si="2"/>
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="CJ29" s="27">
         <f t="shared" si="3"/>
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="CK29" s="22">
         <v>0</v>
       </c>
       <c r="CL29" s="22">
         <f t="shared" si="4"/>
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="CM29" s="42"/>
       <c r="CN29" s="44"/>
       <c r="CO29" s="14">
         <f t="shared" si="5"/>
-        <v>197</v>
+        <v>86</v>
       </c>
       <c r="CP29" s="14">
         <f t="shared" si="6"/>
-        <v>197</v>
+        <v>86</v>
       </c>
       <c r="CQ29" s="14">
         <f t="shared" si="7"/>
-        <v>167</v>
+        <v>50</v>
       </c>
       <c r="CR29" s="43"/>
       <c r="CS29" s="17"/>
       <c r="CT29">
         <v>80</v>
       </c>
-      <c r="DA29">
-        <v>1</v>
-      </c>
       <c r="DB29">
-        <v>116</v>
+        <v>6</v>
       </c>
       <c r="DC29" s="14">
         <f t="shared" si="8"/>
-        <v>197</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -17385,10 +17403,10 @@
       </c>
       <c r="B30" s="60"/>
       <c r="C30" s="56" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="D30" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E30" s="13">
         <v>38</v>
@@ -17513,27 +17531,24 @@
       <c r="CN30" s="44"/>
       <c r="CO30" s="14">
         <f t="shared" si="5"/>
-        <v>420</v>
+        <v>40</v>
       </c>
       <c r="CP30" s="14">
         <f t="shared" si="6"/>
-        <v>420</v>
+        <v>40</v>
       </c>
       <c r="CQ30" s="14">
         <f t="shared" si="7"/>
-        <v>420</v>
+        <v>40</v>
       </c>
       <c r="CR30" s="43"/>
       <c r="CS30" s="17"/>
-      <c r="CZ30">
-        <v>380</v>
-      </c>
       <c r="DB30">
         <v>40</v>
       </c>
       <c r="DC30" s="14">
         <f t="shared" si="8"/>
-        <v>420</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:107" x14ac:dyDescent="0.3">
@@ -17542,10 +17557,10 @@
       </c>
       <c r="B31" s="59"/>
       <c r="C31" s="56" t="s">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="D31" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E31" s="13">
         <v>65</v>
@@ -17693,13 +17708,13 @@
         <v>2</v>
       </c>
       <c r="B32" s="58" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="C32" s="56" t="s">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="D32" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E32" s="13">
         <v>25</v>
@@ -17858,10 +17873,10 @@
       </c>
       <c r="B33" s="60"/>
       <c r="C33" s="56" t="s">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E33" s="13">
         <v>11</v>
@@ -18010,10 +18025,10 @@
       </c>
       <c r="B34" s="59"/>
       <c r="C34" s="56" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="D34" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E34" s="13">
         <v>3</v>
@@ -18160,13 +18175,13 @@
         <v>3</v>
       </c>
       <c r="B35" s="50" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="D35" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E35" s="13">
         <v>71</v>
@@ -18329,13 +18344,13 @@
         <v>5</v>
       </c>
       <c r="B36" s="50" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C36" s="56" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="D36" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E36" s="13">
         <v>2</v>
@@ -18482,13 +18497,13 @@
         <v>6</v>
       </c>
       <c r="B37" s="50" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="C37" s="56" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="D37" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E37" s="13">
         <v>163</v>
@@ -18551,9 +18566,7 @@
       <c r="AN37" s="24">
         <v>2</v>
       </c>
-      <c r="AO37" s="24">
-        <v>5</v>
-      </c>
+      <c r="AO37" s="24"/>
       <c r="AP37" s="24"/>
       <c r="AQ37" s="24"/>
       <c r="AR37" s="24"/>
@@ -18600,18 +18613,18 @@
       <c r="CG37" s="24"/>
       <c r="CH37" s="37">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="CJ37" s="27">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="CK37" s="22">
         <v>0</v>
       </c>
       <c r="CL37" s="22">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="CM37" s="42"/>
       <c r="CN37" s="44"/>
@@ -18625,7 +18638,7 @@
       </c>
       <c r="CQ37" s="14">
         <f t="shared" si="7"/>
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="CR37" s="43"/>
       <c r="CS37" s="17"/>
@@ -18648,13 +18661,13 @@
         <v>8</v>
       </c>
       <c r="B38" s="50" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="C38" s="56" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="D38" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E38" s="13">
         <v>68</v>
@@ -18799,13 +18812,13 @@
         <v>9</v>
       </c>
       <c r="B39" s="50" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="C39" s="56" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E39" s="13">
         <v>1</v>
@@ -18944,13 +18957,13 @@
         <v>12</v>
       </c>
       <c r="B40" s="50" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C40" s="56" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D40" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E40" s="13">
         <v>41</v>
@@ -19099,13 +19112,13 @@
         <v>13</v>
       </c>
       <c r="B41" s="50" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="C41" s="56" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E41" s="13">
         <v>2</v>
@@ -19262,13 +19275,13 @@
         <v>14</v>
       </c>
       <c r="B42" s="50" t="s">
-        <v>108</v>
+        <v>66</v>
       </c>
       <c r="C42" s="56" t="s">
-        <v>108</v>
+        <v>66</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E42" s="13">
         <v>32</v>
@@ -19415,13 +19428,13 @@
         <v>15</v>
       </c>
       <c r="B43" s="50" t="s">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="C43" s="56" t="s">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E43" s="13">
         <v>54</v>
@@ -19571,13 +19584,13 @@
         <v>18</v>
       </c>
       <c r="B44" s="50" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="C44" s="56" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="D44" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E44" s="13">
         <v>4</v>
@@ -19722,13 +19735,13 @@
         <v>19</v>
       </c>
       <c r="B45" s="50" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="C45" s="56" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="D45" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E45" s="13">
         <v>45</v>
@@ -19881,10 +19894,10 @@
         <v>170</v>
       </c>
       <c r="C46" s="56" t="s">
-        <v>114</v>
+        <v>72</v>
       </c>
       <c r="D46" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E46" s="13">
         <v>47</v>
@@ -20023,33 +20036,27 @@
       <c r="CN46" s="44"/>
       <c r="CO46" s="14">
         <f t="shared" si="9"/>
-        <v>603</v>
+        <v>331</v>
       </c>
       <c r="CP46" s="14">
         <f t="shared" ref="CP46:CP77" si="13">CO46</f>
-        <v>603</v>
+        <v>331</v>
       </c>
       <c r="CQ46" s="14">
         <f t="shared" ref="CQ46:CQ77" si="14">CP46-CJ46</f>
-        <v>499</v>
+        <v>227</v>
       </c>
       <c r="CR46" s="43"/>
       <c r="CS46" s="17"/>
       <c r="CT46">
-        <v>421</v>
+        <v>289</v>
       </c>
       <c r="CV46">
         <v>42</v>
       </c>
-      <c r="DA46">
-        <v>2</v>
-      </c>
-      <c r="DB46">
-        <v>138</v>
-      </c>
       <c r="DC46" s="14">
         <f t="shared" ref="DC46:DC77" si="15">SUM(CS46:DB46)</f>
-        <v>603</v>
+        <v>331</v>
       </c>
     </row>
     <row r="47" spans="1:107" x14ac:dyDescent="0.3">
@@ -20058,10 +20065,10 @@
       </c>
       <c r="B47" s="59"/>
       <c r="C47" s="56" t="s">
-        <v>113</v>
+        <v>71</v>
       </c>
       <c r="D47" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E47" s="13">
         <v>43</v>
@@ -20206,13 +20213,13 @@
         <v>21</v>
       </c>
       <c r="B48" s="50" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="C48" s="56" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D48" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E48" s="13">
         <v>55</v>
@@ -20358,13 +20365,13 @@
         <v>22</v>
       </c>
       <c r="B49" s="50" t="s">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="C49" s="56" t="s">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="D49" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E49" s="13">
         <v>50</v>
@@ -20513,13 +20520,13 @@
         <v>23</v>
       </c>
       <c r="B50" s="50" t="s">
-        <v>117</v>
+        <v>75</v>
       </c>
       <c r="C50" s="56" t="s">
-        <v>117</v>
+        <v>75</v>
       </c>
       <c r="D50" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E50" s="13">
         <v>56</v>
@@ -20586,7 +20593,7 @@
         <v>13</v>
       </c>
       <c r="AP50" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AQ50" s="24"/>
       <c r="AR50" s="24"/>
@@ -20633,18 +20640,18 @@
       <c r="CG50" s="24"/>
       <c r="CH50" s="37">
         <f t="shared" si="10"/>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="CJ50" s="27">
         <f t="shared" si="11"/>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="CK50" s="22">
         <v>0</v>
       </c>
       <c r="CL50" s="22">
         <f t="shared" si="12"/>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="CM50" s="42"/>
       <c r="CN50" s="44"/>
@@ -20657,7 +20664,7 @@
       </c>
       <c r="CQ50" s="14">
         <f t="shared" si="14"/>
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="CR50" s="43"/>
       <c r="CS50" s="17"/>
@@ -20671,13 +20678,13 @@
         <v>24</v>
       </c>
       <c r="B51" s="50" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="C51" s="56" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="D51" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E51" s="13">
         <v>83</v>
@@ -20826,13 +20833,13 @@
         <v>26</v>
       </c>
       <c r="B52" s="50" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="C52" s="56" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="D52" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E52" s="13">
         <v>52</v>
@@ -20985,13 +20992,13 @@
         <v>27</v>
       </c>
       <c r="B53" s="50" t="s">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="C53" s="56" t="s">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="D53" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E53" s="13">
         <v>93</v>
@@ -21114,26 +21121,21 @@
       <c r="CN53" s="44"/>
       <c r="CO53" s="14">
         <f t="shared" si="16"/>
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="CP53" s="14">
         <f t="shared" si="13"/>
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="CQ53" s="14">
         <f t="shared" si="14"/>
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="CR53" s="43"/>
-      <c r="CS53" s="17">
-        <v>93</v>
-      </c>
-      <c r="CT53">
-        <v>5</v>
-      </c>
+      <c r="CS53" s="17"/>
       <c r="DC53" s="14">
         <f t="shared" si="15"/>
-        <v>98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:107" x14ac:dyDescent="0.3">
@@ -21141,13 +21143,13 @@
         <v>28</v>
       </c>
       <c r="B54" s="50" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="C54" s="56" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="D54" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E54" s="13">
         <v>44</v>
@@ -21292,13 +21294,13 @@
         <v>29</v>
       </c>
       <c r="B55" s="50" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="C55" s="56" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="D55" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E55" s="13">
         <v>33</v>
@@ -21452,13 +21454,13 @@
         <v>30</v>
       </c>
       <c r="B56" s="50" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="C56" s="56" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="D56" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E56" s="13">
         <v>27</v>
@@ -21601,13 +21603,13 @@
         <v>31</v>
       </c>
       <c r="B57" s="46" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="C57" s="56" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="D57" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E57" s="13">
         <v>43</v>
@@ -21772,13 +21774,13 @@
         <v>31</v>
       </c>
       <c r="B58" s="49" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C58" s="56" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="D58" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E58" s="13">
         <v>46</v>
@@ -21925,13 +21927,13 @@
         <v>32</v>
       </c>
       <c r="B59" s="50" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="C59" s="56" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="D59" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E59" s="13">
         <v>22</v>
@@ -22078,13 +22080,13 @@
         <v>33</v>
       </c>
       <c r="B60" s="50" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="C60" s="56" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="D60" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E60" s="13">
         <v>4</v>
@@ -22226,13 +22228,13 @@
         <v>34</v>
       </c>
       <c r="B61" s="50" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="C61" s="56" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="D61" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E61" s="13">
         <v>44</v>
@@ -22393,13 +22395,13 @@
         <v>35</v>
       </c>
       <c r="B62" s="50" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="C62" s="56" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="D62" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E62" s="13">
         <v>40</v>
@@ -22548,13 +22550,13 @@
         <v>36</v>
       </c>
       <c r="B63" s="50" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="C63" s="56" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="D63" s="33" t="s">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="E63" s="13">
         <v>14</v>
@@ -22699,13 +22701,13 @@
         <v>37</v>
       </c>
       <c r="B64" s="50" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="C64" s="56" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="D64" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E64" s="13">
         <v>26</v>
@@ -22767,7 +22769,7 @@
       </c>
       <c r="AO64" s="24"/>
       <c r="AP64" s="24">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="AQ64" s="24"/>
       <c r="AR64" s="24"/>
@@ -22814,18 +22816,18 @@
       <c r="CG64" s="24"/>
       <c r="CH64" s="37">
         <f t="shared" si="10"/>
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="CJ64" s="27">
         <f t="shared" si="11"/>
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="CK64" s="22">
         <v>0</v>
       </c>
       <c r="CL64" s="22">
         <f t="shared" si="12"/>
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="CM64" s="42"/>
       <c r="CN64" s="44"/>
@@ -22839,7 +22841,7 @@
       </c>
       <c r="CQ64" s="14">
         <f t="shared" si="14"/>
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="CR64" s="43"/>
       <c r="CS64" s="17"/>
@@ -22859,13 +22861,13 @@
         <v>38</v>
       </c>
       <c r="B65" s="50" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="C65" s="56" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="D65" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E65" s="13">
         <v>16</v>
@@ -23012,13 +23014,13 @@
         <v>39</v>
       </c>
       <c r="B66" s="50" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="C66" s="56" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="D66" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E66" s="13">
         <v>11</v>
@@ -23167,13 +23169,13 @@
         <v>44</v>
       </c>
       <c r="B67" s="50" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="C67" s="56" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="D67" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E67" s="13">
         <v>3</v>
@@ -23316,13 +23318,13 @@
         <v>45</v>
       </c>
       <c r="B68" s="46" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="C68" s="56" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="D68" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E68" s="13">
         <v>35</v>
@@ -23471,13 +23473,13 @@
         <v>47</v>
       </c>
       <c r="B69" s="49" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
       <c r="C69" s="56" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
       <c r="D69" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E69" s="13">
         <v>6</v>
@@ -23624,13 +23626,13 @@
         <v>48</v>
       </c>
       <c r="B70" s="50" t="s">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="C70" s="56" t="s">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="D70" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E70" s="13">
         <v>26</v>
@@ -23779,16 +23781,16 @@
     </row>
     <row r="71" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B71" s="50" t="s">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="C71" s="56" t="s">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="D71" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E71" s="13">
         <v>63</v>
@@ -23933,16 +23935,16 @@
     </row>
     <row r="72" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A72" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B72" s="50" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="C72" s="56" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="D72" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E72" s="13">
         <v>25</v>
@@ -24084,16 +24086,16 @@
     </row>
     <row r="73" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B73" s="50" t="s">
-        <v>142</v>
+        <v>100</v>
       </c>
       <c r="C73" s="56" t="s">
-        <v>142</v>
+        <v>100</v>
       </c>
       <c r="D73" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E73" s="13">
         <v>20</v>
@@ -24239,16 +24241,16 @@
     </row>
     <row r="74" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A74" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B74" s="50" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="C74" s="56" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="D74" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E74" s="13">
         <v>14</v>
@@ -24392,16 +24394,16 @@
     </row>
     <row r="75" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B75" s="50" t="s">
-        <v>144</v>
+        <v>102</v>
       </c>
       <c r="C75" s="56" t="s">
-        <v>144</v>
+        <v>102</v>
       </c>
       <c r="D75" s="33" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E75" s="13">
         <v>18</v>
@@ -24550,16 +24552,16 @@
     </row>
     <row r="76" spans="1:107" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="33" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B76" s="50" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="C76" s="56" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="D76" s="33" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="E76" s="13">
         <v>51</v>
@@ -24704,7 +24706,7 @@
     <row r="77" spans="1:107" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A77" s="18"/>
       <c r="B77" s="18" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="C77" s="18"/>
       <c r="D77" s="18"/>
@@ -24818,11 +24820,11 @@
       </c>
       <c r="AO77" s="25">
         <f t="shared" si="18"/>
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="AP77" s="25">
         <f t="shared" si="18"/>
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="AQ77" s="25">
         <f t="shared" si="18"/>
@@ -24998,11 +25000,11 @@
       </c>
       <c r="CH77" s="25">
         <f t="shared" si="19"/>
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="CJ77" s="25">
         <f>+SUM(CJ14:CJ76)</f>
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="CK77" s="25">
         <f>+SUM(CK14:CK76)</f>
@@ -25010,21 +25012,21 @@
       </c>
       <c r="CL77" s="25">
         <f>+SUM(CL14:CL76)</f>
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="CM77" s="25"/>
       <c r="CN77" s="25"/>
       <c r="CO77" s="25">
         <f>+SUM(CO14:CO76)</f>
-        <v>4712</v>
+        <v>2098</v>
       </c>
       <c r="CP77" s="25">
         <f>+SUM(CP14:CP76)</f>
-        <v>4712</v>
+        <v>2098</v>
       </c>
       <c r="CQ77" s="25">
         <f>+SUM(CQ14:CQ76)</f>
-        <v>4036</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="78" spans="1:107" x14ac:dyDescent="0.3">
@@ -25100,7 +25102,7 @@
     </row>
     <row r="79" spans="1:107" x14ac:dyDescent="0.3">
       <c r="B79" s="53" t="s">
-        <v>147</v>
+        <v>105</v>
       </c>
       <c r="C79" s="54"/>
       <c r="D79" s="54"/>
@@ -25182,7 +25184,7 @@
       <c r="CF79" s="30"/>
       <c r="CG79" s="30"/>
       <c r="CH79" s="53" t="s">
-        <v>147</v>
+        <v>105</v>
       </c>
       <c r="CJ79" s="53"/>
       <c r="CK79" s="53"/>
@@ -25191,13 +25193,13 @@
     <row r="80" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A80" s="33"/>
       <c r="B80" s="50" t="s">
-        <v>148</v>
+        <v>106</v>
       </c>
       <c r="C80" s="47" t="s">
-        <v>148</v>
+        <v>106</v>
       </c>
       <c r="D80" s="33" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="E80" s="13">
         <v>4</v>
@@ -25328,13 +25330,13 @@
     <row r="81" spans="1:95" x14ac:dyDescent="0.3">
       <c r="A81" s="33"/>
       <c r="B81" s="50" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="C81" s="47" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="D81" s="33" t="s">
-        <v>151</v>
+        <v>109</v>
       </c>
       <c r="E81" s="13"/>
       <c r="F81" s="13">
@@ -25462,13 +25464,13 @@
     <row r="82" spans="1:95" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A82" s="33"/>
       <c r="B82" s="50" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="C82" s="47" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="D82" s="33" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="E82" s="13">
         <v>1</v>
@@ -25598,7 +25600,7 @@
     <row r="83" spans="1:95" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A83" s="18"/>
       <c r="B83" s="18" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="C83" s="18"/>
       <c r="D83" s="18"/>
@@ -26132,7 +26134,6 @@
       <c r="O98" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A13:CQ77" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="3">
     <mergeCell ref="AC11:CH11"/>
     <mergeCell ref="E10:H10"/>

</xml_diff>

<commit_message>
feat: integracion en tiempo real con Supabase Cloud (PostgreSQL)
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PCI\Documents\Antigravity\dashboard-imagen-telmex\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D108063-7E17-4B83-925F-4CF1D7F0BE3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187305DB-E4EE-40D3-A68B-D993C3F38755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7725" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -364,7 +364,7 @@
     <t>REPORTE DIARIO DE CASETAS Y CAJAS CONTRATISTAS 2026 - IASA / TELMEX</t>
   </si>
   <si>
-    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (26/10/2026, 20:06 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
+    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (26/10/2026, 21:11 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
   </si>
   <si>
     <t>TOTAL CASETAS AL MOMENTO</t>
@@ -1734,17 +1734,17 @@
     <row r="6" spans="2:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="88">
         <f>'Programa CASETAS REPORTE DIARIO'!CN79</f>
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="C6" s="89"/>
       <c r="E6" s="88">
         <f>'Programa CAJAS REPORTE DIARIO'!CH77</f>
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="F6" s="89"/>
       <c r="H6" s="101">
         <f>B6+E6</f>
-        <v>1194</v>
+        <v>1199</v>
       </c>
       <c r="I6" s="97"/>
       <c r="J6" s="97"/>
@@ -2052,19 +2052,19 @@
       </c>
       <c r="D20" s="72">
         <f>'Programa CASETAS REPORTE DIARIO'!AK79</f>
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="E20" s="72">
         <f>'Programa CAJAS REPORTE DIARIO'!AQ77</f>
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="F20" s="72">
         <f t="shared" si="0"/>
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="G20" s="72">
         <f t="shared" si="1"/>
-        <v>1194</v>
+        <v>1199</v>
       </c>
       <c r="H20" s="71" t="s">
         <v>145</v>
@@ -2077,19 +2077,19 @@
       <c r="C21" s="74"/>
       <c r="D21" s="75">
         <f>SUM(D11:D20)</f>
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="E21" s="75">
         <f>SUM(E11:E20)</f>
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="F21" s="75">
         <f>SUM(F11:F20)</f>
-        <v>1194</v>
+        <v>1199</v>
       </c>
       <c r="G21" s="75">
         <f>F21</f>
-        <v>1194</v>
+        <v>1199</v>
       </c>
       <c r="H21" s="76" t="s">
         <v>147</v>
@@ -2223,14 +2223,14 @@
       </c>
       <c r="D3" s="78">
         <f>+CN79</f>
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="F3" s="79" t="s">
         <v>1</v>
       </c>
       <c r="I3" s="80">
         <f>'Programa CAJAS REPORTE DIARIO'!CH77+CN79</f>
-        <v>1194</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="10" spans="1:108" x14ac:dyDescent="0.25">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="AK13" s="23">
         <f t="shared" si="0"/>
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="AL13" s="23">
         <f t="shared" si="0"/>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="CN13" s="37">
         <f t="shared" si="2"/>
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="CP13" s="39"/>
       <c r="CQ13" s="40"/>
@@ -5243,7 +5243,7 @@
         <v>5</v>
       </c>
       <c r="AK29" s="24">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="AL29" s="24"/>
       <c r="AM29" s="24"/>
@@ -5301,18 +5301,18 @@
       <c r="CM29" s="24"/>
       <c r="CN29" s="37">
         <f t="shared" si="3"/>
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="CP29" s="27">
         <f t="shared" si="4"/>
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="CQ29" s="22">
         <v>0</v>
       </c>
       <c r="CR29" s="22">
         <f t="shared" si="5"/>
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="CS29" s="42"/>
       <c r="CT29" s="44"/>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="CW29" s="14">
         <f t="shared" si="8"/>
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="CX29" s="43"/>
       <c r="CY29" s="17">
@@ -7138,7 +7138,9 @@
       <c r="AH42" s="24"/>
       <c r="AI42" s="24"/>
       <c r="AJ42" s="24"/>
-      <c r="AK42" s="24"/>
+      <c r="AK42" s="24">
+        <v>5</v>
+      </c>
       <c r="AL42" s="24"/>
       <c r="AM42" s="24"/>
       <c r="AN42" s="24"/>
@@ -7195,18 +7197,18 @@
       <c r="CM42" s="24"/>
       <c r="CN42" s="37">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CP42" s="27">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CQ42" s="22">
         <v>0</v>
       </c>
       <c r="CR42" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CS42" s="42"/>
       <c r="CT42" s="44"/>
@@ -7220,7 +7222,7 @@
       </c>
       <c r="CW42" s="14">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="CX42" s="43"/>
       <c r="CY42" s="17"/>
@@ -12578,7 +12580,7 @@
       </c>
       <c r="AK79" s="25">
         <f t="shared" si="22"/>
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="AL79" s="25">
         <f t="shared" si="22"/>
@@ -12798,11 +12800,11 @@
       </c>
       <c r="CN79" s="25">
         <f t="shared" si="24"/>
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="CP79" s="25">
         <f>+SUM(CP14:CP78)</f>
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="CQ79" s="25">
         <f>+SUM(CQ14:CQ78)</f>
@@ -12810,7 +12812,7 @@
       </c>
       <c r="CR79" s="25">
         <f>+SUM(CR14:CR78)</f>
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="CS79" s="25"/>
       <c r="CT79" s="25"/>
@@ -12824,7 +12826,7 @@
       </c>
       <c r="CW79" s="25">
         <f>+SUM(CW14:CW78)</f>
-        <v>2804.5</v>
+        <v>2792.5</v>
       </c>
     </row>
     <row r="80" spans="1:108" hidden="1" x14ac:dyDescent="0.25">
@@ -14158,14 +14160,14 @@
       </c>
       <c r="D3" s="78">
         <f>+CH77</f>
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="F3" s="79" t="s">
         <v>1</v>
       </c>
       <c r="I3" s="80">
         <f>'Programa CASETAS REPORTE DIARIO'!CN79+CH77</f>
-        <v>1194</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="10" spans="1:107" x14ac:dyDescent="0.25">
@@ -14686,7 +14688,7 @@
       </c>
       <c r="AQ13" s="38">
         <f t="shared" si="0"/>
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="AR13" s="38">
         <f t="shared" si="0"/>
@@ -14858,7 +14860,7 @@
       </c>
       <c r="CH13" s="38">
         <f t="shared" si="1"/>
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="CJ13" s="39"/>
       <c r="CK13" s="40"/>
@@ -16973,7 +16975,7 @@
       </c>
       <c r="AP27" s="24"/>
       <c r="AQ27" s="24">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AR27" s="24"/>
       <c r="AS27" s="24"/>
@@ -17019,18 +17021,18 @@
       <c r="CG27" s="24"/>
       <c r="CH27" s="37">
         <f t="shared" si="2"/>
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="CJ27" s="27">
         <f t="shared" si="3"/>
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="CK27" s="22">
         <v>0</v>
       </c>
       <c r="CL27" s="22">
         <f t="shared" si="4"/>
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="CM27" s="42"/>
       <c r="CN27" s="44"/>
@@ -17044,7 +17046,7 @@
       </c>
       <c r="CQ27" s="14">
         <f t="shared" si="7"/>
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="CR27" s="43"/>
       <c r="CS27" s="17"/>
@@ -17806,7 +17808,7 @@
       <c r="AO32" s="24"/>
       <c r="AP32" s="24"/>
       <c r="AQ32" s="24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR32" s="24"/>
       <c r="AS32" s="24"/>
@@ -17852,18 +17854,18 @@
       <c r="CG32" s="24"/>
       <c r="CH32" s="37">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CJ32" s="27">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CK32" s="22">
         <v>0</v>
       </c>
       <c r="CL32" s="22">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CM32" s="42"/>
       <c r="CN32" s="44"/>
@@ -17877,7 +17879,7 @@
       </c>
       <c r="CQ32" s="14">
         <f t="shared" si="7"/>
-        <v>4330</v>
+        <v>4331</v>
       </c>
       <c r="CR32" s="43"/>
       <c r="CS32" s="17"/>
@@ -24534,7 +24536,7 @@
       <c r="AO75" s="24"/>
       <c r="AP75" s="24"/>
       <c r="AQ75" s="24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR75" s="24"/>
       <c r="AS75" s="24"/>
@@ -24580,18 +24582,18 @@
       <c r="CG75" s="24"/>
       <c r="CH75" s="37">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CJ75" s="27">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CK75" s="22">
         <v>0</v>
       </c>
       <c r="CL75" s="22">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CM75" s="42"/>
       <c r="CN75" s="44"/>
@@ -24605,7 +24607,7 @@
       </c>
       <c r="CQ75" s="14">
         <f t="shared" si="14"/>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="CR75" s="43"/>
       <c r="CS75" s="17"/>
@@ -24895,7 +24897,7 @@
       </c>
       <c r="AQ77" s="25">
         <f t="shared" si="17"/>
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="AR77" s="25">
         <f t="shared" si="17"/>
@@ -25067,11 +25069,11 @@
       </c>
       <c r="CH77" s="25">
         <f t="shared" si="18"/>
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="CJ77" s="25">
         <f>+SUM(CJ14:CJ76)</f>
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="CK77" s="25">
         <f>+SUM(CK14:CK76)</f>
@@ -25079,7 +25081,7 @@
       </c>
       <c r="CL77" s="25">
         <f>+SUM(CL14:CL76)</f>
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="CM77" s="25"/>
       <c r="CN77" s="25"/>
@@ -25093,7 +25095,7 @@
       </c>
       <c r="CQ77" s="25">
         <f>+SUM(CQ14:CQ76)</f>
-        <v>6121</v>
+        <v>6128</v>
       </c>
     </row>
     <row r="78" spans="1:107" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
sync: actualizar datos en vivo a 1946 registros y reporte diario
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PCI\Documents\Antigravity\dashboard-imagen-telmex\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7684FE3-69FC-447E-9521-982023AEA364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FC4B55-C66E-4ACD-8BA2-D4EBE43D5F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="7725" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="5400" windowHeight="10910" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN GENERAL" sheetId="1" r:id="rId1"/>
@@ -364,7 +364,7 @@
     <t>REPORTE DIARIO DE CASETAS Y CAJAS CONTRATISTAS 2026 - IASA / TELMEX</t>
   </si>
   <si>
-    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (26/10/2026, 21:30 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
+    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (27/10/2026, 18:04 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
   </si>
   <si>
     <t>TOTAL CASETAS AL MOMENTO</t>
@@ -1679,7 +1679,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:J27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -1690,7 +1690,7 @@
     <col min="9" max="10" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="100" t="s">
         <v>111</v>
       </c>
@@ -1703,7 +1703,7 @@
       <c r="I2" s="91"/>
       <c r="J2" s="91"/>
     </row>
-    <row r="3" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="90" t="s">
         <v>112</v>
       </c>
@@ -1716,7 +1716,7 @@
       <c r="I3" s="91"/>
       <c r="J3" s="91"/>
     </row>
-    <row r="5" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="95" t="s">
         <v>113</v>
       </c>
@@ -1731,25 +1731,25 @@
       <c r="I5" s="97"/>
       <c r="J5" s="97"/>
     </row>
-    <row r="6" spans="2:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="88">
         <f>'Programa CASETAS REPORTE DIARIO'!CN79</f>
-        <v>343</v>
+        <v>454</v>
       </c>
       <c r="C6" s="89"/>
       <c r="E6" s="88">
         <f>'Programa CAJAS REPORTE DIARIO'!CH77</f>
-        <v>859</v>
+        <v>1240</v>
       </c>
       <c r="F6" s="89"/>
       <c r="H6" s="101">
         <f>B6+E6</f>
-        <v>1202</v>
+        <v>1694</v>
       </c>
       <c r="I6" s="97"/>
       <c r="J6" s="97"/>
     </row>
-    <row r="7" spans="2:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="93" t="s">
         <v>116</v>
       </c>
@@ -1764,7 +1764,7 @@
       <c r="I7" s="97"/>
       <c r="J7" s="97"/>
     </row>
-    <row r="9" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B9" s="98" t="s">
         <v>119</v>
       </c>
@@ -1777,7 +1777,7 @@
       <c r="I9" s="91"/>
       <c r="J9" s="91"/>
     </row>
-    <row r="10" spans="2:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="68" t="s">
         <v>120</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="69" t="s">
         <v>127</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="12" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="71" t="s">
         <v>130</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="69" t="s">
         <v>132</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="14" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="71" t="s">
         <v>134</v>
       </c>
@@ -1908,7 +1908,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="15" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="69" t="s">
         <v>136</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="71" t="s">
         <v>138</v>
       </c>
@@ -1962,7 +1962,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="69" t="s">
         <v>140</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="71" t="s">
         <v>142</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="69" t="s">
         <v>143</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="71" t="s">
         <v>144</v>
       </c>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D20" s="72">
         <f>'Programa CASETAS REPORTE DIARIO'!AK79</f>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E20" s="72">
         <f>'Programa CAJAS REPORTE DIARIO'!AQ77</f>
@@ -2060,24 +2060,24 @@
       </c>
       <c r="F20" s="72">
         <f t="shared" si="0"/>
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G20" s="72">
         <f t="shared" si="1"/>
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="H20" s="71" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="73" t="s">
         <v>146</v>
       </c>
       <c r="C21" s="74"/>
       <c r="D21" s="75">
         <f>SUM(D11:D20)</f>
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E21" s="75">
         <f>SUM(E11:E20)</f>
@@ -2085,17 +2085,17 @@
       </c>
       <c r="F21" s="75">
         <f>SUM(F11:F20)</f>
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="G21" s="75">
         <f>F21</f>
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="H21" s="76" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B23" s="92" t="s">
         <v>148</v>
       </c>
@@ -2106,7 +2106,7 @@
       <c r="G23" s="91"/>
       <c r="H23" s="91"/>
     </row>
-    <row r="24" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="94" t="s">
         <v>149</v>
       </c>
@@ -2117,7 +2117,7 @@
       <c r="G24" s="91"/>
       <c r="H24" s="91"/>
     </row>
-    <row r="25" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="94" t="s">
         <v>150</v>
       </c>
@@ -2128,7 +2128,7 @@
       <c r="G25" s="91"/>
       <c r="H25" s="91"/>
     </row>
-    <row r="26" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="94" t="s">
         <v>151</v>
       </c>
@@ -2139,7 +2139,7 @@
       <c r="G26" s="91"/>
       <c r="H26" s="91"/>
     </row>
-    <row r="27" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="94" t="s">
         <v>152</v>
       </c>
@@ -2177,63 +2177,63 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A3:DD93"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" customWidth="1"/>
-    <col min="11" max="11" width="2.7109375" customWidth="1"/>
-    <col min="12" max="12" width="7.5703125" hidden="1" customWidth="1"/>
-    <col min="13" max="15" width="7.140625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="29.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" customWidth="1"/>
+    <col min="7" max="7" width="18.7265625" customWidth="1"/>
+    <col min="8" max="8" width="16.453125" customWidth="1"/>
+    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="10" max="10" width="15.453125" customWidth="1"/>
+    <col min="11" max="11" width="2.7265625" customWidth="1"/>
+    <col min="12" max="12" width="7.54296875" hidden="1" customWidth="1"/>
+    <col min="13" max="15" width="7.1796875" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="9" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="1.85546875" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="13.5703125" style="3" customWidth="1"/>
-    <col min="19" max="19" width="1.5703125" style="3" customWidth="1"/>
-    <col min="20" max="21" width="12.85546875" customWidth="1"/>
-    <col min="22" max="22" width="3.5703125" customWidth="1"/>
-    <col min="23" max="26" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="27" width="13.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="28" max="35" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="36" width="13.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="37" max="37" width="13.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="13.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="39" max="39" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="40" max="40" width="13.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="41" max="42" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="43" max="91" width="13.5703125" customWidth="1" outlineLevel="1"/>
+    <col min="17" max="17" width="1.81640625" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="13.54296875" style="3" customWidth="1"/>
+    <col min="19" max="19" width="1.54296875" style="3" customWidth="1"/>
+    <col min="20" max="21" width="12.81640625" customWidth="1"/>
+    <col min="22" max="22" width="3.54296875" customWidth="1"/>
+    <col min="23" max="26" width="13.7265625" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="13.54296875" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="35" width="13.7265625" customWidth="1" outlineLevel="1"/>
+    <col min="36" max="36" width="13.54296875" customWidth="1" outlineLevel="1"/>
+    <col min="37" max="37" width="13.453125" customWidth="1" outlineLevel="1"/>
+    <col min="38" max="38" width="13.54296875" customWidth="1" outlineLevel="1"/>
+    <col min="39" max="39" width="13.7265625" customWidth="1" outlineLevel="1"/>
+    <col min="40" max="40" width="13.54296875" customWidth="1" outlineLevel="1"/>
+    <col min="41" max="42" width="13.7265625" customWidth="1" outlineLevel="1"/>
+    <col min="43" max="91" width="13.54296875" customWidth="1" outlineLevel="1"/>
     <col min="92" max="92" width="14" customWidth="1"/>
-    <col min="93" max="93" width="2.42578125" customWidth="1"/>
-    <col min="94" max="95" width="13.85546875" customWidth="1"/>
+    <col min="93" max="93" width="2.453125" customWidth="1"/>
+    <col min="94" max="95" width="13.81640625" customWidth="1"/>
     <col min="96" max="96" width="14" customWidth="1"/>
-    <col min="97" max="97" width="15.7109375" customWidth="1"/>
-    <col min="98" max="100" width="11.42578125" customWidth="1"/>
-    <col min="101" max="101" width="11.85546875" customWidth="1"/>
-    <col min="102" max="103" width="11.42578125" customWidth="1"/>
+    <col min="97" max="97" width="15.7265625" customWidth="1"/>
+    <col min="98" max="100" width="11.453125" customWidth="1"/>
+    <col min="101" max="101" width="11.81640625" customWidth="1"/>
+    <col min="102" max="103" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:108" ht="21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:108" ht="21" x14ac:dyDescent="0.35">
       <c r="B3" s="77" t="s">
         <v>0</v>
       </c>
       <c r="D3" s="78">
         <f>+CN79</f>
-        <v>343</v>
+        <v>454</v>
       </c>
       <c r="F3" s="79" t="s">
         <v>1</v>
       </c>
       <c r="I3" s="80">
         <f>'Programa CAJAS REPORTE DIARIO'!CH77+CN79</f>
-        <v>1202</v>
+        <v>1694</v>
       </c>
     </row>
-    <row r="10" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A10" s="31"/>
       <c r="E10" s="81" t="s">
         <v>2</v>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="U10" s="2"/>
     </row>
-    <row r="11" spans="1:108" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:108" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -2344,7 +2344,7 @@
       <c r="CV11" s="29"/>
       <c r="CW11" s="29"/>
     </row>
-    <row r="12" spans="1:108" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:108" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -2617,7 +2617,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:108" s="12" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:108" s="12" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>22</v>
       </c>
@@ -2731,11 +2731,11 @@
       </c>
       <c r="AK13" s="23">
         <f t="shared" si="0"/>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AL13" s="23">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="AM13" s="23">
         <f t="shared" si="0"/>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="CN13" s="37">
         <f t="shared" si="2"/>
-        <v>343</v>
+        <v>454</v>
       </c>
       <c r="CP13" s="39"/>
       <c r="CQ13" s="40"/>
@@ -2980,7 +2980,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="33" t="s">
         <v>33</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A15" s="33" t="s">
         <v>33</v>
       </c>
@@ -3268,7 +3268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A16" s="33" t="s">
         <v>33</v>
       </c>
@@ -3413,7 +3413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="33" t="s">
         <v>33</v>
       </c>
@@ -3556,7 +3556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A18" s="33" t="s">
         <v>33</v>
       </c>
@@ -3701,7 +3701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="33" t="s">
         <v>33</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A20" s="33" t="s">
         <v>33</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A22" s="33" t="s">
         <v>33</v>
       </c>
@@ -4279,7 +4279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A23" s="33" t="s">
         <v>33</v>
       </c>
@@ -4422,7 +4422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A24" s="33" t="s">
         <v>33</v>
       </c>
@@ -4565,7 +4565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A25" s="33" t="s">
         <v>33</v>
       </c>
@@ -4710,7 +4710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="33" t="s">
         <v>33</v>
       </c>
@@ -4855,7 +4855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A27" s="33" t="s">
         <v>33</v>
       </c>
@@ -4926,7 +4926,9 @@
       <c r="AK27" s="24">
         <v>19</v>
       </c>
-      <c r="AL27" s="24"/>
+      <c r="AL27" s="24">
+        <v>25</v>
+      </c>
       <c r="AM27" s="24"/>
       <c r="AN27" s="24"/>
       <c r="AO27" s="24"/>
@@ -4982,18 +4984,18 @@
       <c r="CM27" s="24"/>
       <c r="CN27" s="37">
         <f t="shared" si="3"/>
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="CP27" s="27">
         <f t="shared" si="4"/>
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="CQ27" s="22">
         <v>0</v>
       </c>
       <c r="CR27" s="22">
         <f t="shared" si="5"/>
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="CS27" s="42"/>
       <c r="CT27" s="44"/>
@@ -5007,7 +5009,7 @@
       </c>
       <c r="CW27" s="14">
         <f t="shared" si="8"/>
-        <v>245.5</v>
+        <v>220.5</v>
       </c>
       <c r="CX27" s="43"/>
       <c r="CY27" s="17">
@@ -5021,7 +5023,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="28" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A28" s="33" t="s">
         <v>33</v>
       </c>
@@ -5086,7 +5088,9 @@
       <c r="AK28" s="24">
         <v>2</v>
       </c>
-      <c r="AL28" s="24"/>
+      <c r="AL28" s="24">
+        <v>15</v>
+      </c>
       <c r="AM28" s="24"/>
       <c r="AN28" s="24"/>
       <c r="AO28" s="24"/>
@@ -5142,18 +5146,18 @@
       <c r="CM28" s="24"/>
       <c r="CN28" s="37">
         <f t="shared" si="3"/>
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="CP28" s="27">
         <f t="shared" si="4"/>
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="CQ28" s="22">
         <v>0</v>
       </c>
       <c r="CR28" s="22">
         <f t="shared" si="5"/>
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="CS28" s="42"/>
       <c r="CT28" s="44"/>
@@ -5167,7 +5171,7 @@
       </c>
       <c r="CW28" s="14">
         <f t="shared" si="8"/>
-        <v>1277</v>
+        <v>1262</v>
       </c>
       <c r="CX28" s="43"/>
       <c r="CY28" s="17">
@@ -5181,7 +5185,7 @@
         <v>2754</v>
       </c>
     </row>
-    <row r="29" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="33">
         <v>1</v>
       </c>
@@ -5340,7 +5344,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="30" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="33">
         <v>1</v>
       </c>
@@ -5490,7 +5494,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="33">
         <v>1</v>
       </c>
@@ -5635,7 +5639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A32" s="33">
         <v>2</v>
       </c>
@@ -5687,7 +5691,9 @@
       <c r="AI32" s="24"/>
       <c r="AJ32" s="24"/>
       <c r="AK32" s="24"/>
-      <c r="AL32" s="24"/>
+      <c r="AL32" s="24">
+        <v>11</v>
+      </c>
       <c r="AM32" s="24"/>
       <c r="AN32" s="24"/>
       <c r="AO32" s="24"/>
@@ -5743,18 +5749,18 @@
       <c r="CM32" s="24"/>
       <c r="CN32" s="37">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="CP32" s="27">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="CQ32" s="22">
         <v>0</v>
       </c>
       <c r="CR32" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="CS32" s="42"/>
       <c r="CT32" s="44"/>
@@ -5768,7 +5774,7 @@
       </c>
       <c r="CW32" s="14">
         <f t="shared" si="8"/>
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="CX32" s="43"/>
       <c r="CY32" s="17">
@@ -5779,7 +5785,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="33" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A33" s="33">
         <v>2</v>
       </c>
@@ -5922,7 +5928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A34" s="33">
         <v>2</v>
       </c>
@@ -6066,7 +6072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A35" s="33">
         <v>4</v>
       </c>
@@ -6123,7 +6129,9 @@
       <c r="AK35" s="24">
         <v>2</v>
       </c>
-      <c r="AL35" s="24"/>
+      <c r="AL35" s="24">
+        <v>13</v>
+      </c>
       <c r="AM35" s="24"/>
       <c r="AN35" s="24"/>
       <c r="AO35" s="24"/>
@@ -6179,18 +6187,18 @@
       <c r="CM35" s="24"/>
       <c r="CN35" s="37">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="CP35" s="27">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="CQ35" s="22">
         <v>0</v>
       </c>
       <c r="CR35" s="22">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="CS35" s="42"/>
       <c r="CT35" s="44"/>
@@ -6204,7 +6212,7 @@
       </c>
       <c r="CW35" s="14">
         <f t="shared" si="8"/>
-        <v>-2</v>
+        <v>-15</v>
       </c>
       <c r="CX35" s="43"/>
       <c r="CY35" s="17"/>
@@ -6213,7 +6221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A36" s="33">
         <v>5</v>
       </c>
@@ -6270,7 +6278,9 @@
       <c r="AK36" s="24">
         <v>8</v>
       </c>
-      <c r="AL36" s="24"/>
+      <c r="AL36" s="24">
+        <v>6</v>
+      </c>
       <c r="AM36" s="24"/>
       <c r="AN36" s="24"/>
       <c r="AO36" s="24"/>
@@ -6326,18 +6336,18 @@
       <c r="CM36" s="24"/>
       <c r="CN36" s="37">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="CP36" s="27">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="CQ36" s="22">
         <v>0</v>
       </c>
       <c r="CR36" s="22">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="CS36" s="42"/>
       <c r="CT36" s="44"/>
@@ -6351,7 +6361,7 @@
       </c>
       <c r="CW36" s="14">
         <f t="shared" si="8"/>
-        <v>-8</v>
+        <v>-14</v>
       </c>
       <c r="CX36" s="43"/>
       <c r="CY36" s="17"/>
@@ -6360,7 +6370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:108" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:108" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="33">
         <v>6</v>
       </c>
@@ -6505,7 +6515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A38" s="33">
         <v>8</v>
       </c>
@@ -6650,7 +6660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="33">
         <v>9</v>
       </c>
@@ -6795,7 +6805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A40" s="33">
         <v>10</v>
       </c>
@@ -6849,7 +6859,9 @@
       <c r="AI40" s="24"/>
       <c r="AJ40" s="24"/>
       <c r="AK40" s="24"/>
-      <c r="AL40" s="24"/>
+      <c r="AL40" s="24">
+        <v>7</v>
+      </c>
       <c r="AM40" s="24"/>
       <c r="AN40" s="24"/>
       <c r="AO40" s="24"/>
@@ -6905,18 +6917,18 @@
       <c r="CM40" s="24"/>
       <c r="CN40" s="37">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="CP40" s="27">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="CQ40" s="22">
         <v>0</v>
       </c>
       <c r="CR40" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="CS40" s="42"/>
       <c r="CT40" s="44"/>
@@ -6930,7 +6942,7 @@
       </c>
       <c r="CW40" s="14">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>-7</v>
       </c>
       <c r="CX40" s="43"/>
       <c r="CY40" s="17"/>
@@ -6939,7 +6951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A41" s="33">
         <v>12</v>
       </c>
@@ -7084,7 +7096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="33">
         <v>13</v>
       </c>
@@ -7139,9 +7151,11 @@
       <c r="AI42" s="24"/>
       <c r="AJ42" s="24"/>
       <c r="AK42" s="24">
-        <v>8</v>
-      </c>
-      <c r="AL42" s="24"/>
+        <v>9</v>
+      </c>
+      <c r="AL42" s="24">
+        <v>20</v>
+      </c>
       <c r="AM42" s="24"/>
       <c r="AN42" s="24"/>
       <c r="AO42" s="24"/>
@@ -7197,18 +7211,18 @@
       <c r="CM42" s="24"/>
       <c r="CN42" s="37">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="CP42" s="27">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="CQ42" s="22">
         <v>0</v>
       </c>
       <c r="CR42" s="22">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="CS42" s="42"/>
       <c r="CT42" s="44"/>
@@ -7222,7 +7236,7 @@
       </c>
       <c r="CW42" s="14">
         <f t="shared" si="8"/>
-        <v>-8</v>
+        <v>-29</v>
       </c>
       <c r="CX42" s="43"/>
       <c r="CY42" s="17"/>
@@ -7231,7 +7245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A43" s="33">
         <v>14</v>
       </c>
@@ -7376,7 +7390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A44" s="33">
         <v>15</v>
       </c>
@@ -7521,7 +7535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A45" s="33">
         <v>18</v>
       </c>
@@ -7666,7 +7680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A46" s="33">
         <v>19</v>
       </c>
@@ -7813,7 +7827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A47" s="33">
         <v>20</v>
       </c>
@@ -7958,7 +7972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A48" s="33">
         <v>20</v>
       </c>
@@ -8104,7 +8118,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="49" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A49" s="33">
         <v>21</v>
       </c>
@@ -8159,7 +8173,9 @@
       <c r="AI49" s="24"/>
       <c r="AJ49" s="24"/>
       <c r="AK49" s="24"/>
-      <c r="AL49" s="24"/>
+      <c r="AL49" s="24">
+        <v>1</v>
+      </c>
       <c r="AM49" s="24"/>
       <c r="AN49" s="24"/>
       <c r="AO49" s="24"/>
@@ -8215,18 +8231,18 @@
       <c r="CM49" s="24"/>
       <c r="CN49" s="37">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CP49" s="27">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CQ49" s="22">
         <v>0</v>
       </c>
       <c r="CR49" s="22">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CS49" s="42"/>
       <c r="CT49" s="44"/>
@@ -8240,7 +8256,7 @@
       </c>
       <c r="CW49" s="14">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="CX49" s="43"/>
       <c r="CY49" s="17"/>
@@ -8249,7 +8265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A50" s="33">
         <v>22</v>
       </c>
@@ -8393,7 +8409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A51" s="33">
         <v>23</v>
       </c>
@@ -8450,7 +8466,9 @@
       </c>
       <c r="AJ51" s="24"/>
       <c r="AK51" s="24"/>
-      <c r="AL51" s="24"/>
+      <c r="AL51" s="24">
+        <v>10</v>
+      </c>
       <c r="AM51" s="24"/>
       <c r="AN51" s="24"/>
       <c r="AO51" s="24"/>
@@ -8506,18 +8524,18 @@
       <c r="CM51" s="24"/>
       <c r="CN51" s="37">
         <f t="shared" si="10"/>
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="CP51" s="27">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="CQ51" s="22">
         <v>0</v>
       </c>
       <c r="CR51" s="22">
         <f t="shared" si="12"/>
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="CS51" s="42"/>
       <c r="CT51" s="44"/>
@@ -8531,7 +8549,7 @@
       </c>
       <c r="CW51" s="14">
         <f t="shared" si="15"/>
-        <v>749</v>
+        <v>739</v>
       </c>
       <c r="CX51" s="43"/>
       <c r="CY51" s="17"/>
@@ -8543,7 +8561,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="52" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A52" s="33">
         <v>24</v>
       </c>
@@ -8690,7 +8708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A53" s="33">
         <v>26</v>
       </c>
@@ -8835,7 +8853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A54" s="33">
         <v>27</v>
       </c>
@@ -8980,7 +8998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A55" s="33">
         <v>28</v>
       </c>
@@ -9125,7 +9143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A56" s="33">
         <v>29</v>
       </c>
@@ -9270,7 +9288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A57" s="33">
         <v>30</v>
       </c>
@@ -9415,7 +9433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A58" s="33">
         <v>31</v>
       </c>
@@ -9472,7 +9490,9 @@
       <c r="AI58" s="24"/>
       <c r="AJ58" s="24"/>
       <c r="AK58" s="24"/>
-      <c r="AL58" s="24"/>
+      <c r="AL58" s="24">
+        <v>2</v>
+      </c>
       <c r="AM58" s="24"/>
       <c r="AN58" s="24"/>
       <c r="AO58" s="24"/>
@@ -9528,18 +9548,18 @@
       <c r="CM58" s="24"/>
       <c r="CN58" s="37">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CP58" s="27">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CQ58" s="22">
         <v>0</v>
       </c>
       <c r="CR58" s="22">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CS58" s="42"/>
       <c r="CT58" s="44"/>
@@ -9553,7 +9573,7 @@
       </c>
       <c r="CW58" s="14">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="CX58" s="43"/>
       <c r="CY58" s="17"/>
@@ -9562,7 +9582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A59" s="33">
         <v>31</v>
       </c>
@@ -9709,7 +9729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A60" s="33">
         <v>32</v>
       </c>
@@ -9856,7 +9876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A61" s="33">
         <v>33</v>
       </c>
@@ -10001,7 +10021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A62" s="33">
         <v>34</v>
       </c>
@@ -10148,7 +10168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A63" s="33">
         <v>35</v>
       </c>
@@ -10293,7 +10313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A64" s="33">
         <v>36</v>
       </c>
@@ -10440,7 +10460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A65" s="33">
         <v>37</v>
       </c>
@@ -10586,7 +10606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A66" s="33">
         <v>38</v>
       </c>
@@ -10733,7 +10753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A67" s="33">
         <v>39</v>
       </c>
@@ -10878,7 +10898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A68" s="33">
         <v>44</v>
       </c>
@@ -11021,7 +11041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A69" s="33">
         <v>45</v>
       </c>
@@ -11168,7 +11188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="33">
         <v>47</v>
       </c>
@@ -11313,7 +11333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="33">
         <v>48</v>
       </c>
@@ -11458,7 +11478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="33" t="s">
         <v>97</v>
       </c>
@@ -11603,7 +11623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A73" s="33" t="s">
         <v>97</v>
       </c>
@@ -11748,7 +11768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="33" t="s">
         <v>97</v>
       </c>
@@ -11893,7 +11913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:108" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:108" x14ac:dyDescent="0.35">
       <c r="A75" s="33" t="s">
         <v>97</v>
       </c>
@@ -12040,7 +12060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="33" t="s">
         <v>97</v>
       </c>
@@ -12185,7 +12205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="33" t="s">
         <v>97</v>
       </c>
@@ -12330,7 +12350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:108" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:108" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="33" t="s">
         <v>97</v>
       </c>
@@ -12473,7 +12493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:108" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:108" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A79" s="18"/>
       <c r="B79" s="18" t="s">
         <v>31</v>
@@ -12580,11 +12600,11 @@
       </c>
       <c r="AK79" s="25">
         <f t="shared" si="22"/>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AL79" s="25">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="AM79" s="25">
         <f t="shared" si="22"/>
@@ -12800,11 +12820,11 @@
       </c>
       <c r="CN79" s="25">
         <f t="shared" si="24"/>
-        <v>343</v>
+        <v>454</v>
       </c>
       <c r="CP79" s="25">
         <f>+SUM(CP14:CP78)</f>
-        <v>343</v>
+        <v>454</v>
       </c>
       <c r="CQ79" s="25">
         <f>+SUM(CQ14:CQ78)</f>
@@ -12812,7 +12832,7 @@
       </c>
       <c r="CR79" s="25">
         <f>+SUM(CR14:CR78)</f>
-        <v>343</v>
+        <v>454</v>
       </c>
       <c r="CS79" s="25"/>
       <c r="CT79" s="25"/>
@@ -12826,10 +12846,10 @@
       </c>
       <c r="CW79" s="25">
         <f>+SUM(CW14:CW78)</f>
-        <v>2789.5</v>
+        <v>2678.5</v>
       </c>
     </row>
-    <row r="80" spans="1:108" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:108" hidden="1" x14ac:dyDescent="0.35">
       <c r="E80" s="21"/>
       <c r="F80" s="21"/>
       <c r="G80" s="21"/>
@@ -12906,7 +12926,7 @@
       <c r="CL80" s="17"/>
       <c r="CM80" s="17"/>
     </row>
-    <row r="81" spans="1:101" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:101" hidden="1" x14ac:dyDescent="0.35">
       <c r="B81" s="53" t="s">
         <v>105</v>
       </c>
@@ -13002,7 +13022,7 @@
       <c r="CQ81" s="53"/>
       <c r="CR81" s="53"/>
     </row>
-    <row r="82" spans="1:101" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:101" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="33"/>
       <c r="B82" s="50" t="s">
         <v>106</v>
@@ -13123,7 +13143,7 @@
       <c r="CV82" s="14"/>
       <c r="CW82" s="14"/>
     </row>
-    <row r="83" spans="1:101" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:101" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="33"/>
       <c r="B83" s="50" t="s">
         <v>108</v>
@@ -13245,7 +13265,7 @@
       <c r="CV83" s="14"/>
       <c r="CW83" s="14"/>
     </row>
-    <row r="84" spans="1:101" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:101" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="33"/>
       <c r="B84" s="50" t="s">
         <v>110</v>
@@ -13367,7 +13387,7 @@
       <c r="CV84" s="14"/>
       <c r="CW84" s="14"/>
     </row>
-    <row r="85" spans="1:101" ht="15.75" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:101" ht="15.75" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A85" s="18"/>
       <c r="B85" s="18" t="s">
         <v>31</v>
@@ -13723,7 +13743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:101" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:101" hidden="1" x14ac:dyDescent="0.35">
       <c r="E86" s="14"/>
       <c r="F86" s="14"/>
       <c r="G86" s="14"/>
@@ -13802,7 +13822,7 @@
       <c r="CP86" s="14"/>
       <c r="CQ86" s="35"/>
     </row>
-    <row r="87" spans="1:101" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:101" x14ac:dyDescent="0.35">
       <c r="B87" s="32"/>
       <c r="C87" s="32"/>
       <c r="D87" s="32"/>
@@ -13810,7 +13830,7 @@
       <c r="H87" s="14"/>
       <c r="I87" s="14"/>
     </row>
-    <row r="88" spans="1:101" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:101" x14ac:dyDescent="0.35">
       <c r="B88" s="32"/>
       <c r="C88" s="32"/>
       <c r="D88" s="32"/>
@@ -13818,7 +13838,7 @@
       <c r="H88" s="14"/>
       <c r="I88" s="14"/>
     </row>
-    <row r="89" spans="1:101" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:101" x14ac:dyDescent="0.35">
       <c r="B89" s="53" t="s">
         <v>105</v>
       </c>
@@ -13911,7 +13931,7 @@
       <c r="CV89" s="64"/>
       <c r="CW89" s="64"/>
     </row>
-    <row r="90" spans="1:101" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:101" x14ac:dyDescent="0.35">
       <c r="A90" s="33">
         <v>17</v>
       </c>
@@ -13948,7 +13968,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="91" spans="1:101" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:101" x14ac:dyDescent="0.35">
       <c r="A91" s="33">
         <v>25</v>
       </c>
@@ -13985,7 +14005,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="92" spans="1:101" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:101" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="33">
         <v>43</v>
       </c>
@@ -14021,7 +14041,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="93" spans="1:101" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:101" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A93" s="18"/>
       <c r="B93" s="18" t="s">
         <v>31</v>
@@ -14115,62 +14135,62 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:DC98"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" customWidth="1"/>
-    <col min="9" max="15" width="13.42578125" customWidth="1"/>
-    <col min="16" max="16" width="15.42578125" customWidth="1"/>
-    <col min="17" max="17" width="2.7109375" customWidth="1"/>
-    <col min="18" max="18" width="7.5703125" hidden="1" customWidth="1"/>
-    <col min="19" max="21" width="7.140625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="22.54296875" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" customWidth="1"/>
+    <col min="7" max="7" width="18.7265625" customWidth="1"/>
+    <col min="8" max="8" width="16.453125" customWidth="1"/>
+    <col min="9" max="15" width="13.453125" customWidth="1"/>
+    <col min="16" max="16" width="15.453125" customWidth="1"/>
+    <col min="17" max="17" width="2.7265625" customWidth="1"/>
+    <col min="18" max="18" width="7.54296875" hidden="1" customWidth="1"/>
+    <col min="19" max="21" width="7.1796875" hidden="1" customWidth="1"/>
     <col min="22" max="22" width="9" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="1.85546875" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="13.5703125" style="3" customWidth="1"/>
-    <col min="25" max="25" width="1.5703125" style="3" customWidth="1"/>
-    <col min="26" max="27" width="12.85546875" customWidth="1"/>
-    <col min="28" max="28" width="3.5703125" style="6" customWidth="1"/>
-    <col min="29" max="32" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="33" width="13.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="34" max="34" width="13.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="35" max="35" width="13.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="36" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="37" max="37" width="13.5703125" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="39" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="40" max="85" width="13.5703125" customWidth="1" outlineLevel="1"/>
+    <col min="23" max="23" width="1.81640625" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="13.54296875" style="3" customWidth="1"/>
+    <col min="25" max="25" width="1.54296875" style="3" customWidth="1"/>
+    <col min="26" max="27" width="12.81640625" customWidth="1"/>
+    <col min="28" max="28" width="3.54296875" style="6" customWidth="1"/>
+    <col min="29" max="32" width="13.7265625" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="33" width="13.54296875" customWidth="1" outlineLevel="1"/>
+    <col min="34" max="34" width="13.453125" customWidth="1" outlineLevel="1"/>
+    <col min="35" max="35" width="13.54296875" customWidth="1" outlineLevel="1"/>
+    <col min="36" max="36" width="13.7265625" customWidth="1" outlineLevel="1"/>
+    <col min="37" max="37" width="13.54296875" customWidth="1" outlineLevel="1"/>
+    <col min="38" max="39" width="13.7265625" customWidth="1" outlineLevel="1"/>
+    <col min="40" max="85" width="13.54296875" customWidth="1" outlineLevel="1"/>
     <col min="86" max="86" width="14" customWidth="1"/>
-    <col min="87" max="87" width="4.28515625" customWidth="1"/>
-    <col min="88" max="88" width="13.85546875" customWidth="1"/>
-    <col min="89" max="89" width="15.7109375" customWidth="1"/>
+    <col min="87" max="87" width="4.26953125" customWidth="1"/>
+    <col min="88" max="88" width="13.81640625" customWidth="1"/>
+    <col min="89" max="89" width="15.7265625" customWidth="1"/>
     <col min="90" max="90" width="14" customWidth="1"/>
-    <col min="91" max="91" width="15.7109375" customWidth="1"/>
-    <col min="92" max="94" width="11.42578125" customWidth="1"/>
-    <col min="95" max="95" width="11.85546875" customWidth="1"/>
-    <col min="96" max="97" width="11.42578125" customWidth="1"/>
+    <col min="91" max="91" width="15.7265625" customWidth="1"/>
+    <col min="92" max="94" width="11.453125" customWidth="1"/>
+    <col min="95" max="95" width="11.81640625" customWidth="1"/>
+    <col min="96" max="97" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:107" ht="21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:107" ht="21" x14ac:dyDescent="0.35">
       <c r="B3" s="77" t="s">
         <v>153</v>
       </c>
       <c r="D3" s="78">
         <f>+CH77</f>
-        <v>859</v>
+        <v>1240</v>
       </c>
       <c r="F3" s="79" t="s">
         <v>1</v>
       </c>
       <c r="I3" s="80">
         <f>'Programa CASETAS REPORTE DIARIO'!CN79+CH77</f>
-        <v>1202</v>
+        <v>1694</v>
       </c>
     </row>
-    <row r="10" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A10" s="31"/>
       <c r="E10" s="81" t="s">
         <v>2</v>
@@ -14193,7 +14213,7 @@
       </c>
       <c r="AA10" s="2"/>
     </row>
-    <row r="11" spans="1:107" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:107" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
@@ -14282,7 +14302,7 @@
       <c r="CP11" s="29"/>
       <c r="CQ11" s="29"/>
     </row>
-    <row r="12" spans="1:107" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:107" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -14555,7 +14575,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:107" s="12" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:107" s="12" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>22</v>
       </c>
@@ -14692,7 +14712,7 @@
       </c>
       <c r="AR13" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>381</v>
       </c>
       <c r="AS13" s="38">
         <f t="shared" si="0"/>
@@ -14860,7 +14880,7 @@
       </c>
       <c r="CH13" s="38">
         <f t="shared" si="1"/>
-        <v>859</v>
+        <v>1240</v>
       </c>
       <c r="CJ13" s="39"/>
       <c r="CK13" s="40"/>
@@ -14904,7 +14924,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="33" t="s">
         <v>33</v>
       </c>
@@ -15057,7 +15077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A15" s="33" t="s">
         <v>33</v>
       </c>
@@ -15210,7 +15230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A16" s="33" t="s">
         <v>33</v>
       </c>
@@ -15363,7 +15383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="33" t="s">
         <v>33</v>
       </c>
@@ -15516,7 +15536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A18" s="33" t="s">
         <v>33</v>
       </c>
@@ -15669,7 +15689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="33" t="s">
         <v>33</v>
       </c>
@@ -15822,7 +15842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A20" s="33" t="s">
         <v>33</v>
       </c>
@@ -15975,7 +15995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A21" s="33" t="s">
         <v>33</v>
       </c>
@@ -16126,7 +16146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A22" s="33" t="s">
         <v>33</v>
       </c>
@@ -16279,7 +16299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A23" s="33" t="s">
         <v>33</v>
       </c>
@@ -16430,7 +16450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A24" s="33" t="s">
         <v>33</v>
       </c>
@@ -16581,7 +16601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="33" t="s">
         <v>33</v>
       </c>
@@ -16734,7 +16754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A26" s="33" t="s">
         <v>33</v>
       </c>
@@ -16886,7 +16906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A27" s="33" t="s">
         <v>33</v>
       </c>
@@ -16977,7 +16997,9 @@
       <c r="AQ27" s="24">
         <v>51</v>
       </c>
-      <c r="AR27" s="24"/>
+      <c r="AR27" s="24">
+        <v>43</v>
+      </c>
       <c r="AS27" s="24"/>
       <c r="AT27" s="24"/>
       <c r="AU27" s="24"/>
@@ -17021,18 +17043,18 @@
       <c r="CG27" s="24"/>
       <c r="CH27" s="37">
         <f t="shared" si="2"/>
-        <v>288</v>
+        <v>331</v>
       </c>
       <c r="CJ27" s="27">
         <f t="shared" si="3"/>
-        <v>288</v>
+        <v>331</v>
       </c>
       <c r="CK27" s="22">
         <v>0</v>
       </c>
       <c r="CL27" s="22">
         <f t="shared" si="4"/>
-        <v>288</v>
+        <v>331</v>
       </c>
       <c r="CM27" s="42"/>
       <c r="CN27" s="44"/>
@@ -17046,7 +17068,7 @@
       </c>
       <c r="CQ27" s="14">
         <f t="shared" si="7"/>
-        <v>498</v>
+        <v>455</v>
       </c>
       <c r="CR27" s="43"/>
       <c r="CS27" s="17"/>
@@ -17067,7 +17089,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="28" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="33" t="s">
         <v>33</v>
       </c>
@@ -17156,7 +17178,9 @@
       <c r="AQ28" s="24">
         <v>52</v>
       </c>
-      <c r="AR28" s="24"/>
+      <c r="AR28" s="24">
+        <v>43</v>
+      </c>
       <c r="AS28" s="24"/>
       <c r="AT28" s="24"/>
       <c r="AU28" s="24"/>
@@ -17200,18 +17224,18 @@
       <c r="CG28" s="24"/>
       <c r="CH28" s="37">
         <f t="shared" si="2"/>
-        <v>153</v>
+        <v>196</v>
       </c>
       <c r="CJ28" s="27">
         <f t="shared" si="3"/>
-        <v>153</v>
+        <v>196</v>
       </c>
       <c r="CK28" s="22">
         <v>0</v>
       </c>
       <c r="CL28" s="22">
         <f t="shared" si="4"/>
-        <v>153</v>
+        <v>196</v>
       </c>
       <c r="CM28" s="42"/>
       <c r="CN28" s="44"/>
@@ -17225,7 +17249,7 @@
       </c>
       <c r="CQ28" s="14">
         <f t="shared" si="7"/>
-        <v>25</v>
+        <v>-18</v>
       </c>
       <c r="CR28" s="43"/>
       <c r="CS28" s="17">
@@ -17254,7 +17278,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="29" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="33">
         <v>1</v>
       </c>
@@ -17425,7 +17449,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="33">
         <v>1</v>
       </c>
@@ -17579,7 +17603,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A31" s="33">
         <v>1</v>
       </c>
@@ -17731,7 +17755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A32" s="33">
         <v>2</v>
       </c>
@@ -17810,7 +17834,9 @@
       <c r="AQ32" s="24">
         <v>1</v>
       </c>
-      <c r="AR32" s="24"/>
+      <c r="AR32" s="24">
+        <v>83</v>
+      </c>
       <c r="AS32" s="24"/>
       <c r="AT32" s="24"/>
       <c r="AU32" s="24"/>
@@ -17854,18 +17880,18 @@
       <c r="CG32" s="24"/>
       <c r="CH32" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="CJ32" s="27">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="CK32" s="22">
         <v>0</v>
       </c>
       <c r="CL32" s="22">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="CM32" s="42"/>
       <c r="CN32" s="44"/>
@@ -17879,7 +17905,7 @@
       </c>
       <c r="CQ32" s="14">
         <f t="shared" si="7"/>
-        <v>4331</v>
+        <v>4248</v>
       </c>
       <c r="CR32" s="43"/>
       <c r="CS32" s="17"/>
@@ -17900,7 +17926,7 @@
         <v>4332</v>
       </c>
     </row>
-    <row r="33" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A33" s="33">
         <v>2</v>
       </c>
@@ -18052,7 +18078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A34" s="33">
         <v>2</v>
       </c>
@@ -18203,7 +18229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A35" s="33">
         <v>3</v>
       </c>
@@ -18282,7 +18308,9 @@
       <c r="AQ35" s="24">
         <v>4</v>
       </c>
-      <c r="AR35" s="24"/>
+      <c r="AR35" s="24">
+        <v>71</v>
+      </c>
       <c r="AS35" s="24"/>
       <c r="AT35" s="24"/>
       <c r="AU35" s="24"/>
@@ -18326,18 +18354,18 @@
       <c r="CG35" s="24"/>
       <c r="CH35" s="37">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="CJ35" s="27">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="CK35" s="22">
         <v>0</v>
       </c>
       <c r="CL35" s="22">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="CM35" s="42"/>
       <c r="CN35" s="44"/>
@@ -18351,7 +18379,7 @@
       </c>
       <c r="CQ35" s="14">
         <f t="shared" si="7"/>
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="CR35" s="43"/>
       <c r="CS35" s="17">
@@ -18374,7 +18402,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:107" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:107" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="33">
         <v>5</v>
       </c>
@@ -18451,7 +18479,9 @@
       <c r="AQ36" s="24">
         <v>2</v>
       </c>
-      <c r="AR36" s="24"/>
+      <c r="AR36" s="24">
+        <v>8</v>
+      </c>
       <c r="AS36" s="24"/>
       <c r="AT36" s="24"/>
       <c r="AU36" s="24"/>
@@ -18495,18 +18525,18 @@
       <c r="CG36" s="24"/>
       <c r="CH36" s="37">
         <f t="shared" si="2"/>
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="CJ36" s="27">
         <f t="shared" si="3"/>
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="CK36" s="22">
         <v>0</v>
       </c>
       <c r="CL36" s="22">
         <f t="shared" si="4"/>
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="CM36" s="42"/>
       <c r="CN36" s="44"/>
@@ -18520,7 +18550,7 @@
       </c>
       <c r="CQ36" s="14">
         <f t="shared" si="7"/>
-        <v>-22</v>
+        <v>-30</v>
       </c>
       <c r="CR36" s="43"/>
       <c r="CS36" s="17"/>
@@ -18529,7 +18559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A37" s="33">
         <v>6</v>
       </c>
@@ -18606,7 +18636,9 @@
       <c r="AO37" s="24"/>
       <c r="AP37" s="24"/>
       <c r="AQ37" s="24"/>
-      <c r="AR37" s="24"/>
+      <c r="AR37" s="24">
+        <v>36</v>
+      </c>
       <c r="AS37" s="24"/>
       <c r="AT37" s="24"/>
       <c r="AU37" s="24"/>
@@ -18650,18 +18682,18 @@
       <c r="CG37" s="24"/>
       <c r="CH37" s="37">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="CJ37" s="27">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="CK37" s="22">
         <v>0</v>
       </c>
       <c r="CL37" s="22">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="CM37" s="42"/>
       <c r="CN37" s="44"/>
@@ -18675,7 +18707,7 @@
       </c>
       <c r="CQ37" s="14">
         <f t="shared" si="7"/>
-        <v>573</v>
+        <v>537</v>
       </c>
       <c r="CR37" s="43"/>
       <c r="CS37" s="17"/>
@@ -18699,7 +18731,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="38" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="33">
         <v>8</v>
       </c>
@@ -18850,7 +18882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A39" s="33">
         <v>9</v>
       </c>
@@ -18995,7 +19027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A40" s="33">
         <v>12</v>
       </c>
@@ -19150,7 +19182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="33">
         <v>13</v>
       </c>
@@ -19227,7 +19259,9 @@
       <c r="AO41" s="24"/>
       <c r="AP41" s="24"/>
       <c r="AQ41" s="24"/>
-      <c r="AR41" s="24"/>
+      <c r="AR41" s="24">
+        <v>8</v>
+      </c>
       <c r="AS41" s="24"/>
       <c r="AT41" s="24"/>
       <c r="AU41" s="24"/>
@@ -19271,18 +19305,18 @@
       <c r="CG41" s="24"/>
       <c r="CH41" s="37">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="CJ41" s="27">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="CK41" s="22">
         <v>0</v>
       </c>
       <c r="CL41" s="22">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="CM41" s="42"/>
       <c r="CN41" s="44"/>
@@ -19296,7 +19330,7 @@
       </c>
       <c r="CQ41" s="14">
         <f t="shared" si="7"/>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="CR41" s="43"/>
       <c r="CS41" s="17">
@@ -19313,7 +19347,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A42" s="33">
         <v>14</v>
       </c>
@@ -19466,7 +19500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A43" s="33">
         <v>15</v>
       </c>
@@ -19545,7 +19579,9 @@
       <c r="AO43" s="24"/>
       <c r="AP43" s="24"/>
       <c r="AQ43" s="24"/>
-      <c r="AR43" s="24"/>
+      <c r="AR43" s="24">
+        <v>27</v>
+      </c>
       <c r="AS43" s="24"/>
       <c r="AT43" s="24"/>
       <c r="AU43" s="24"/>
@@ -19589,18 +19625,18 @@
       <c r="CG43" s="24"/>
       <c r="CH43" s="37">
         <f t="shared" si="2"/>
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="CJ43" s="27">
         <f t="shared" si="3"/>
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="CK43" s="22">
         <v>0</v>
       </c>
       <c r="CL43" s="22">
         <f t="shared" si="4"/>
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="CM43" s="42"/>
       <c r="CN43" s="44"/>
@@ -19613,7 +19649,7 @@
       </c>
       <c r="CQ43" s="14">
         <f t="shared" si="7"/>
-        <v>-13</v>
+        <v>-40</v>
       </c>
       <c r="CR43" s="43"/>
       <c r="CS43" s="17"/>
@@ -19622,7 +19658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A44" s="33">
         <v>18</v>
       </c>
@@ -19773,7 +19809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A45" s="33">
         <v>19</v>
       </c>
@@ -19929,7 +19965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A46" s="33">
         <v>20</v>
       </c>
@@ -20020,7 +20056,9 @@
       <c r="AQ46" s="24">
         <v>3</v>
       </c>
-      <c r="AR46" s="24"/>
+      <c r="AR46" s="24">
+        <v>10</v>
+      </c>
       <c r="AS46" s="24"/>
       <c r="AT46" s="24"/>
       <c r="AU46" s="24"/>
@@ -20064,18 +20102,18 @@
       <c r="CG46" s="24"/>
       <c r="CH46" s="37">
         <f t="shared" ref="CH46:CH77" si="10">+SUM(AC46:CG46)</f>
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="CJ46" s="27">
         <f t="shared" ref="CJ46:CJ76" si="11">CH46</f>
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="CK46" s="22">
         <v>0</v>
       </c>
       <c r="CL46" s="22">
         <f t="shared" ref="CL46:CL77" si="12">CJ46+CK46</f>
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="CM46" s="42"/>
       <c r="CN46" s="44"/>
@@ -20089,7 +20127,7 @@
       </c>
       <c r="CQ46" s="14">
         <f t="shared" ref="CQ46:CQ77" si="14">CP46-CJ46</f>
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="CR46" s="43"/>
       <c r="CS46" s="17"/>
@@ -20104,7 +20142,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="47" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A47" s="33">
         <v>20</v>
       </c>
@@ -20253,7 +20291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A48" s="33">
         <v>21</v>
       </c>
@@ -20405,7 +20443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A49" s="33">
         <v>22</v>
       </c>
@@ -20560,7 +20598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A50" s="33">
         <v>23</v>
       </c>
@@ -20722,7 +20760,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="51" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A51" s="33">
         <v>24</v>
       </c>
@@ -20799,7 +20837,9 @@
       <c r="AO51" s="24"/>
       <c r="AP51" s="24"/>
       <c r="AQ51" s="24"/>
-      <c r="AR51" s="24"/>
+      <c r="AR51" s="24">
+        <v>3</v>
+      </c>
       <c r="AS51" s="24"/>
       <c r="AT51" s="24"/>
       <c r="AU51" s="24"/>
@@ -20843,18 +20883,18 @@
       <c r="CG51" s="24"/>
       <c r="CH51" s="37">
         <f t="shared" si="10"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="CJ51" s="27">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="CK51" s="22">
         <v>0</v>
       </c>
       <c r="CL51" s="22">
         <f t="shared" si="12"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="CM51" s="42"/>
       <c r="CN51" s="44"/>
@@ -20868,7 +20908,7 @@
       </c>
       <c r="CQ51" s="14">
         <f t="shared" si="14"/>
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="CR51" s="43"/>
       <c r="CS51" s="17"/>
@@ -20877,7 +20917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A52" s="33">
         <v>26</v>
       </c>
@@ -21036,7 +21076,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A53" s="33">
         <v>27</v>
       </c>
@@ -21190,7 +21230,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A54" s="33">
         <v>28</v>
       </c>
@@ -21343,7 +21383,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A55" s="33">
         <v>29</v>
       </c>
@@ -21422,7 +21462,9 @@
         <v>3</v>
       </c>
       <c r="AQ55" s="24"/>
-      <c r="AR55" s="24"/>
+      <c r="AR55" s="24">
+        <v>22</v>
+      </c>
       <c r="AS55" s="24"/>
       <c r="AT55" s="24"/>
       <c r="AU55" s="24"/>
@@ -21466,18 +21508,18 @@
       <c r="CG55" s="24"/>
       <c r="CH55" s="37">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="CJ55" s="27">
         <f t="shared" si="11"/>
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="CK55" s="22">
         <v>0</v>
       </c>
       <c r="CL55" s="22">
         <f t="shared" si="12"/>
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="CM55" s="42"/>
       <c r="CN55" s="44"/>
@@ -21491,7 +21533,7 @@
       </c>
       <c r="CQ55" s="14">
         <f t="shared" si="14"/>
-        <v>9</v>
+        <v>-13</v>
       </c>
       <c r="CR55" s="43"/>
       <c r="CS55" s="17"/>
@@ -21503,7 +21545,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="56" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A56" s="33">
         <v>30</v>
       </c>
@@ -21652,7 +21694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A57" s="33">
         <v>31</v>
       </c>
@@ -21739,7 +21781,9 @@
       <c r="AQ57" s="24">
         <v>7</v>
       </c>
-      <c r="AR57" s="24"/>
+      <c r="AR57" s="24">
+        <v>3</v>
+      </c>
       <c r="AS57" s="24"/>
       <c r="AT57" s="24"/>
       <c r="AU57" s="24"/>
@@ -21783,18 +21827,18 @@
       <c r="CG57" s="24"/>
       <c r="CH57" s="37">
         <f t="shared" si="10"/>
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="CJ57" s="27">
         <f t="shared" si="11"/>
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="CK57" s="22">
         <v>0</v>
       </c>
       <c r="CL57" s="22">
         <f t="shared" si="12"/>
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="CM57" s="42"/>
       <c r="CN57" s="44"/>
@@ -21808,7 +21852,7 @@
       </c>
       <c r="CQ57" s="14">
         <f t="shared" si="14"/>
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="CR57" s="43"/>
       <c r="CS57" s="17">
@@ -21825,7 +21869,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A58" s="33">
         <v>31</v>
       </c>
@@ -21978,7 +22022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A59" s="33">
         <v>32</v>
       </c>
@@ -22131,7 +22175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A60" s="33">
         <v>33</v>
       </c>
@@ -22279,7 +22323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A61" s="33">
         <v>34</v>
       </c>
@@ -22364,7 +22408,9 @@
       <c r="AQ61" s="24">
         <v>5</v>
       </c>
-      <c r="AR61" s="24"/>
+      <c r="AR61" s="24">
+        <v>5</v>
+      </c>
       <c r="AS61" s="24"/>
       <c r="AT61" s="24"/>
       <c r="AU61" s="24"/>
@@ -22408,18 +22454,18 @@
       <c r="CG61" s="24"/>
       <c r="CH61" s="37">
         <f t="shared" si="10"/>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="CJ61" s="27">
         <f t="shared" si="11"/>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="CK61" s="22">
         <v>0</v>
       </c>
       <c r="CL61" s="22">
         <f t="shared" si="12"/>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="CM61" s="42"/>
       <c r="CN61" s="44"/>
@@ -22433,7 +22479,7 @@
       </c>
       <c r="CQ61" s="14">
         <f t="shared" si="14"/>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="CR61" s="43"/>
       <c r="CS61" s="17"/>
@@ -22448,7 +22494,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A62" s="33">
         <v>35</v>
       </c>
@@ -22603,7 +22649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A63" s="33">
         <v>36</v>
       </c>
@@ -22754,7 +22800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A64" s="33">
         <v>37</v>
       </c>
@@ -22832,7 +22878,9 @@
       <c r="AQ64" s="24">
         <v>4</v>
       </c>
-      <c r="AR64" s="24"/>
+      <c r="AR64" s="24">
+        <v>11</v>
+      </c>
       <c r="AS64" s="24"/>
       <c r="AT64" s="24"/>
       <c r="AU64" s="24"/>
@@ -22876,18 +22924,18 @@
       <c r="CG64" s="24"/>
       <c r="CH64" s="37">
         <f t="shared" si="10"/>
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="CJ64" s="27">
         <f t="shared" si="11"/>
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="CK64" s="22">
         <v>0</v>
       </c>
       <c r="CL64" s="22">
         <f t="shared" si="12"/>
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="CM64" s="42"/>
       <c r="CN64" s="44"/>
@@ -22901,7 +22949,7 @@
       </c>
       <c r="CQ64" s="14">
         <f t="shared" si="14"/>
-        <v>-24</v>
+        <v>-35</v>
       </c>
       <c r="CR64" s="43"/>
       <c r="CS64" s="17"/>
@@ -22916,7 +22964,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A65" s="33">
         <v>38</v>
       </c>
@@ -23069,7 +23117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A66" s="33">
         <v>39</v>
       </c>
@@ -23224,7 +23272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A67" s="33">
         <v>44</v>
       </c>
@@ -23373,7 +23421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A68" s="33">
         <v>45</v>
       </c>
@@ -23528,7 +23576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="33">
         <v>47</v>
       </c>
@@ -23683,7 +23731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="33">
         <v>48</v>
       </c>
@@ -23762,7 +23810,9 @@
       <c r="AQ70" s="24">
         <v>39</v>
       </c>
-      <c r="AR70" s="24"/>
+      <c r="AR70" s="24">
+        <v>6</v>
+      </c>
       <c r="AS70" s="24"/>
       <c r="AT70" s="24"/>
       <c r="AU70" s="24"/>
@@ -23806,18 +23856,18 @@
       <c r="CG70" s="24"/>
       <c r="CH70" s="37">
         <f t="shared" si="10"/>
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="CJ70" s="27">
         <f t="shared" si="11"/>
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="CK70" s="22">
         <v>0</v>
       </c>
       <c r="CL70" s="22">
         <f t="shared" si="12"/>
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="CM70" s="42"/>
       <c r="CN70" s="44"/>
@@ -23831,7 +23881,7 @@
       </c>
       <c r="CQ70" s="14">
         <f t="shared" si="14"/>
-        <v>-25</v>
+        <v>-31</v>
       </c>
       <c r="CR70" s="43"/>
       <c r="CS70" s="17"/>
@@ -23846,7 +23896,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="71" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="33" t="s">
         <v>97</v>
       </c>
@@ -24000,7 +24050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A72" s="33" t="s">
         <v>97</v>
       </c>
@@ -24151,7 +24201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="33" t="s">
         <v>97</v>
       </c>
@@ -24306,7 +24356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A74" s="33" t="s">
         <v>97</v>
       </c>
@@ -24459,7 +24509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:107" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="33" t="s">
         <v>97</v>
       </c>
@@ -24538,7 +24588,9 @@
       <c r="AQ75" s="24">
         <v>1</v>
       </c>
-      <c r="AR75" s="24"/>
+      <c r="AR75" s="24">
+        <v>2</v>
+      </c>
       <c r="AS75" s="24"/>
       <c r="AT75" s="24"/>
       <c r="AU75" s="24"/>
@@ -24582,18 +24634,18 @@
       <c r="CG75" s="24"/>
       <c r="CH75" s="37">
         <f t="shared" si="10"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CJ75" s="27">
         <f t="shared" si="11"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CK75" s="22">
         <v>0</v>
       </c>
       <c r="CL75" s="22">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CM75" s="42"/>
       <c r="CN75" s="44"/>
@@ -24607,7 +24659,7 @@
       </c>
       <c r="CQ75" s="14">
         <f t="shared" si="14"/>
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="CR75" s="43"/>
       <c r="CS75" s="17"/>
@@ -24619,7 +24671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:107" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:107" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="33" t="s">
         <v>97</v>
       </c>
@@ -24772,7 +24824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:107" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:107" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A77" s="18"/>
       <c r="B77" s="18" t="s">
         <v>31</v>
@@ -24901,7 +24953,7 @@
       </c>
       <c r="AR77" s="25">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>381</v>
       </c>
       <c r="AS77" s="25">
         <f t="shared" si="17"/>
@@ -25069,11 +25121,11 @@
       </c>
       <c r="CH77" s="25">
         <f t="shared" si="18"/>
-        <v>859</v>
+        <v>1240</v>
       </c>
       <c r="CJ77" s="25">
         <f>+SUM(CJ14:CJ76)</f>
-        <v>859</v>
+        <v>1240</v>
       </c>
       <c r="CK77" s="25">
         <f>+SUM(CK14:CK76)</f>
@@ -25081,7 +25133,7 @@
       </c>
       <c r="CL77" s="25">
         <f>+SUM(CL14:CL76)</f>
-        <v>859</v>
+        <v>1240</v>
       </c>
       <c r="CM77" s="25"/>
       <c r="CN77" s="25"/>
@@ -25095,10 +25147,10 @@
       </c>
       <c r="CQ77" s="25">
         <f>+SUM(CQ14:CQ76)</f>
-        <v>6128</v>
+        <v>5747</v>
       </c>
     </row>
-    <row r="78" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:107" x14ac:dyDescent="0.35">
       <c r="E78" s="21"/>
       <c r="F78" s="21"/>
       <c r="G78" s="21"/>
@@ -25169,7 +25221,7 @@
       <c r="CF78" s="17"/>
       <c r="CG78" s="17"/>
     </row>
-    <row r="79" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:107" x14ac:dyDescent="0.35">
       <c r="B79" s="53" t="s">
         <v>105</v>
       </c>
@@ -25259,7 +25311,7 @@
       <c r="CK79" s="53"/>
       <c r="CL79" s="53"/>
     </row>
-    <row r="80" spans="1:107" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:107" x14ac:dyDescent="0.35">
       <c r="A80" s="33"/>
       <c r="B80" s="50" t="s">
         <v>106</v>
@@ -25396,7 +25448,7 @@
       <c r="CP80" s="14"/>
       <c r="CQ80" s="14"/>
     </row>
-    <row r="81" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:95" x14ac:dyDescent="0.35">
       <c r="A81" s="33"/>
       <c r="B81" s="50" t="s">
         <v>108</v>
@@ -25530,7 +25582,7 @@
       <c r="CP81" s="14"/>
       <c r="CQ81" s="14"/>
     </row>
-    <row r="82" spans="1:95" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:95" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="33"/>
       <c r="B82" s="50" t="s">
         <v>110</v>
@@ -25666,7 +25718,7 @@
       <c r="CP82" s="22"/>
       <c r="CQ82" s="22"/>
     </row>
-    <row r="83" spans="1:95" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:95" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A83" s="18"/>
       <c r="B83" s="18" t="s">
         <v>31</v>
@@ -25923,7 +25975,7 @@
       <c r="CP83" s="25"/>
       <c r="CQ83" s="25"/>
     </row>
-    <row r="84" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:95" x14ac:dyDescent="0.35">
       <c r="E84" s="14"/>
       <c r="F84" s="14"/>
       <c r="G84" s="14"/>
@@ -25996,7 +26048,7 @@
       <c r="CJ84" s="14"/>
       <c r="CK84" s="35"/>
     </row>
-    <row r="85" spans="1:95" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:95" ht="8.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B85" s="32"/>
       <c r="C85" s="32"/>
       <c r="D85" s="32"/>
@@ -26010,7 +26062,7 @@
       <c r="N85" s="14"/>
       <c r="O85" s="14"/>
     </row>
-    <row r="86" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B86" s="32"/>
       <c r="C86" s="32"/>
       <c r="D86" s="32"/>
@@ -26034,7 +26086,7 @@
       <c r="N86" s="14"/>
       <c r="O86" s="14"/>
     </row>
-    <row r="87" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B87" s="32"/>
       <c r="C87" s="32"/>
       <c r="D87" s="32"/>
@@ -26048,7 +26100,7 @@
       <c r="N87" s="14"/>
       <c r="O87" s="14"/>
     </row>
-    <row r="88" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B88" s="32"/>
       <c r="C88" s="32"/>
       <c r="D88" s="32"/>
@@ -26062,7 +26114,7 @@
       <c r="N88" s="14"/>
       <c r="O88" s="14"/>
     </row>
-    <row r="89" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B89" s="32"/>
       <c r="C89" s="32"/>
       <c r="D89" s="32"/>
@@ -26076,7 +26128,7 @@
       <c r="N89" s="14"/>
       <c r="O89" s="14"/>
     </row>
-    <row r="90" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B90" s="32"/>
       <c r="C90" s="32"/>
       <c r="D90" s="32"/>
@@ -26090,7 +26142,7 @@
       <c r="N90" s="14"/>
       <c r="O90" s="14"/>
     </row>
-    <row r="91" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B91" s="32"/>
       <c r="C91" s="32"/>
       <c r="D91" s="32"/>
@@ -26104,7 +26156,7 @@
       <c r="N91" s="14"/>
       <c r="O91" s="14"/>
     </row>
-    <row r="92" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B92" s="32"/>
       <c r="C92" s="32"/>
       <c r="D92" s="32"/>
@@ -26118,7 +26170,7 @@
       <c r="N92" s="14"/>
       <c r="O92" s="14"/>
     </row>
-    <row r="93" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B93" s="32"/>
       <c r="C93" s="32"/>
       <c r="D93" s="32"/>
@@ -26132,7 +26184,7 @@
       <c r="N93" s="14"/>
       <c r="O93" s="14"/>
     </row>
-    <row r="94" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B94" s="32"/>
       <c r="C94" s="32"/>
       <c r="D94" s="32"/>
@@ -26146,7 +26198,7 @@
       <c r="N94" s="14"/>
       <c r="O94" s="14"/>
     </row>
-    <row r="95" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B95" s="32"/>
       <c r="C95" s="32"/>
       <c r="D95" s="32"/>
@@ -26160,7 +26212,7 @@
       <c r="N95" s="14"/>
       <c r="O95" s="14"/>
     </row>
-    <row r="96" spans="1:95" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:95" x14ac:dyDescent="0.35">
       <c r="B96" s="32"/>
       <c r="C96" s="32"/>
       <c r="D96" s="32"/>
@@ -26174,7 +26226,7 @@
       <c r="N96" s="14"/>
       <c r="O96" s="14"/>
     </row>
-    <row r="97" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B97" s="32"/>
       <c r="C97" s="32"/>
       <c r="D97" s="32"/>
@@ -26188,7 +26240,7 @@
       <c r="N97" s="14"/>
       <c r="O97" s="14"/>
     </row>
-    <row r="98" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B98" s="32"/>
       <c r="C98" s="32"/>
       <c r="D98" s="32"/>

</xml_diff>

<commit_message>
Sincronizacion dinamica de resumen general en Excel y datos en vivo 28-oct
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PCI\Documents\Antigravity\dashboard-imagen-telmex\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8EE133-8CF4-4DC7-8BEA-ED30178EC976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A604FE44-45AC-44D7-BA09-506124DA2201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="174">
   <si>
     <t>TOTAL CASETAS AL MOMENTO:</t>
   </si>
@@ -364,7 +364,7 @@
     <t>REPORTE DIARIO DE CASETAS Y CAJAS CONTRATISTAS 2026 - IASA / TELMEX</t>
   </si>
   <si>
-    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (28/10/2026, 10:26 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
+    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (28/10/2026, 10:27 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
   </si>
   <si>
     <t>TOTAL CASETAS AL MOMENTO</t>
@@ -463,7 +463,16 @@
     <t>2026-10-26</t>
   </si>
   <si>
-    <t>En Proceso (7:00 AM)</t>
+    <t>Corte Oficial Cerrado</t>
+  </si>
+  <si>
+    <t>2026-10-27</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>Jornada en Vivo</t>
   </si>
   <si>
     <t>TOTAL GENERAL AL MOMENTO</t>
@@ -1333,15 +1342,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1352,6 +1360,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1678,7 +1687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J27"/>
+  <dimension ref="B2:J29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1704,7 +1713,7 @@
       <c r="J2" s="91"/>
     </row>
     <row r="3" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="90" t="s">
+      <c r="B3" s="92" t="s">
         <v>112</v>
       </c>
       <c r="C3" s="91"/>
@@ -1717,19 +1726,19 @@
       <c r="J3" s="91"/>
     </row>
     <row r="5" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="95" t="s">
+      <c r="B5" s="94" t="s">
         <v>113</v>
       </c>
       <c r="C5" s="89"/>
-      <c r="E5" s="95" t="s">
+      <c r="E5" s="94" t="s">
         <v>114</v>
       </c>
       <c r="F5" s="89"/>
-      <c r="H5" s="96" t="s">
+      <c r="H5" s="95" t="s">
         <v>115</v>
       </c>
-      <c r="I5" s="97"/>
-      <c r="J5" s="97"/>
+      <c r="I5" s="96"/>
+      <c r="J5" s="96"/>
     </row>
     <row r="6" spans="2:10" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="88">
@@ -1746,8 +1755,8 @@
         <f>B6+E6</f>
         <v>1876</v>
       </c>
-      <c r="I6" s="97"/>
-      <c r="J6" s="97"/>
+      <c r="I6" s="96"/>
+      <c r="J6" s="96"/>
     </row>
     <row r="7" spans="2:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="93" t="s">
@@ -1761,11 +1770,11 @@
       <c r="H7" s="99" t="s">
         <v>118</v>
       </c>
-      <c r="I7" s="97"/>
-      <c r="J7" s="97"/>
+      <c r="I7" s="96"/>
+      <c r="J7" s="96"/>
     </row>
     <row r="9" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="98" t="s">
+      <c r="B9" s="97" t="s">
         <v>119</v>
       </c>
       <c r="C9" s="91"/>
@@ -1816,7 +1825,7 @@
         <v>52</v>
       </c>
       <c r="F11" s="70">
-        <f t="shared" ref="F11:F20" si="0">D11+E11</f>
+        <f t="shared" ref="F11:F22" si="0">D11+E11</f>
         <v>76</v>
       </c>
       <c r="G11" s="70">
@@ -1847,7 +1856,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="72">
-        <f t="shared" ref="G12:G20" si="1">G11+F12</f>
+        <f t="shared" ref="G12:G22" si="1">G11+F12</f>
         <v>76</v>
       </c>
       <c r="H12" s="71" t="s">
@@ -2070,56 +2079,88 @@
         <v>145</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="73" t="s">
+    <row r="21" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="69" t="s">
         <v>146</v>
       </c>
-      <c r="C21" s="74"/>
-      <c r="D21" s="75">
-        <f>SUM(D11:D20)</f>
-        <v>344</v>
-      </c>
-      <c r="E21" s="75">
-        <f>SUM(E11:E20)</f>
-        <v>859</v>
-      </c>
-      <c r="F21" s="75">
-        <f>SUM(F11:F20)</f>
-        <v>1203</v>
-      </c>
-      <c r="G21" s="75">
-        <f>F21</f>
-        <v>1203</v>
-      </c>
-      <c r="H21" s="76" t="s">
+      <c r="C21" s="69" t="s">
+        <v>135</v>
+      </c>
+      <c r="D21" s="70">
+        <f>'Programa CASETAS REPORTE DIARIO'!AL79</f>
+        <v>138</v>
+      </c>
+      <c r="E21" s="70">
+        <f>'Programa CAJAS REPORTE DIARIO'!AR77</f>
+        <v>466</v>
+      </c>
+      <c r="F21" s="70">
+        <f t="shared" si="0"/>
+        <v>604</v>
+      </c>
+      <c r="G21" s="70">
+        <f t="shared" si="1"/>
+        <v>1807</v>
+      </c>
+      <c r="H21" s="69" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="71" t="s">
         <v>147</v>
       </c>
+      <c r="C22" s="71" t="s">
+        <v>137</v>
+      </c>
+      <c r="D22" s="72">
+        <f>'Programa CASETAS REPORTE DIARIO'!AM79</f>
+        <v>37</v>
+      </c>
+      <c r="E22" s="72">
+        <f>'Programa CAJAS REPORTE DIARIO'!AS77</f>
+        <v>32</v>
+      </c>
+      <c r="F22" s="72">
+        <f t="shared" si="0"/>
+        <v>69</v>
+      </c>
+      <c r="G22" s="72">
+        <f t="shared" si="1"/>
+        <v>1876</v>
+      </c>
+      <c r="H22" s="71" t="s">
+        <v>148</v>
+      </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B23" s="92" t="s">
-        <v>148</v>
-      </c>
-      <c r="C23" s="91"/>
-      <c r="D23" s="91"/>
-      <c r="E23" s="91"/>
-      <c r="F23" s="91"/>
-      <c r="G23" s="91"/>
-      <c r="H23" s="91"/>
+    <row r="23" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="73" t="s">
+        <v>149</v>
+      </c>
+      <c r="C23" s="74"/>
+      <c r="D23" s="75">
+        <f>SUM(D11:D22)</f>
+        <v>519</v>
+      </c>
+      <c r="E23" s="75">
+        <f>SUM(E11:E22)</f>
+        <v>1357</v>
+      </c>
+      <c r="F23" s="75">
+        <f>SUM(F11:F22)</f>
+        <v>1876</v>
+      </c>
+      <c r="G23" s="75">
+        <f>F23</f>
+        <v>1876</v>
+      </c>
+      <c r="H23" s="76" t="s">
+        <v>150</v>
+      </c>
     </row>
-    <row r="24" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="94" t="s">
-        <v>149</v>
-      </c>
-      <c r="C24" s="91"/>
-      <c r="D24" s="91"/>
-      <c r="E24" s="91"/>
-      <c r="F24" s="91"/>
-      <c r="G24" s="91"/>
-      <c r="H24" s="91"/>
-    </row>
-    <row r="25" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="94" t="s">
-        <v>150</v>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B25" s="98" t="s">
+        <v>151</v>
       </c>
       <c r="C25" s="91"/>
       <c r="D25" s="91"/>
@@ -2129,8 +2170,8 @@
       <c r="H25" s="91"/>
     </row>
     <row r="26" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="94" t="s">
-        <v>151</v>
+      <c r="B26" s="90" t="s">
+        <v>152</v>
       </c>
       <c r="C26" s="91"/>
       <c r="D26" s="91"/>
@@ -2140,8 +2181,8 @@
       <c r="H26" s="91"/>
     </row>
     <row r="27" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="94" t="s">
-        <v>152</v>
+      <c r="B27" s="90" t="s">
+        <v>153</v>
       </c>
       <c r="C27" s="91"/>
       <c r="D27" s="91"/>
@@ -2150,25 +2191,47 @@
       <c r="G27" s="91"/>
       <c r="H27" s="91"/>
     </row>
+    <row r="28" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="90" t="s">
+        <v>154</v>
+      </c>
+      <c r="C28" s="91"/>
+      <c r="D28" s="91"/>
+      <c r="E28" s="91"/>
+      <c r="F28" s="91"/>
+      <c r="G28" s="91"/>
+      <c r="H28" s="91"/>
+    </row>
+    <row r="29" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="90" t="s">
+        <v>155</v>
+      </c>
+      <c r="C29" s="91"/>
+      <c r="D29" s="91"/>
+      <c r="E29" s="91"/>
+      <c r="F29" s="91"/>
+      <c r="G29" s="91"/>
+      <c r="H29" s="91"/>
+    </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="H7:J7"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="H6:J6"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="E6:F6"/>
     <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B27:H27"/>
     <mergeCell ref="E7:F7"/>
-    <mergeCell ref="B27:H27"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="B9:J9"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14196,7 +14259,7 @@
   <sheetData>
     <row r="3" spans="1:107" ht="21" x14ac:dyDescent="0.3">
       <c r="B3" s="77" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D3" s="78">
         <f>+CH77</f>
@@ -14254,7 +14317,7 @@
       </c>
       <c r="AA11" s="6"/>
       <c r="AC11" s="83" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AD11" s="84"/>
       <c r="AE11" s="84"/>
@@ -14559,40 +14622,40 @@
         <v>19</v>
       </c>
       <c r="CP12" s="29" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="CQ12" s="29" t="s">
         <v>21</v>
       </c>
       <c r="CS12" s="29" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="CT12" s="29" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="CU12" s="29" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="CV12" s="29" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="CW12" s="29" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="CX12" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="CY12" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="CZ12" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="DA12" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="DB12" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:107" s="12" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -14600,7 +14663,7 @@
         <v>22</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>24</v>
@@ -14609,37 +14672,37 @@
         <v>25</v>
       </c>
       <c r="E13" s="57" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F13" s="57" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G13" s="57" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="H13" s="57" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="I13" s="57" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J13" s="57" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="K13" s="57" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="L13" s="57" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="M13" s="57" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="N13" s="57" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="O13" s="57" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>31</v>
@@ -14911,34 +14974,34 @@
       <c r="CP13" s="29"/>
       <c r="CQ13" s="29"/>
       <c r="CS13" s="67" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="CT13" s="67" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="CU13" s="67" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="CV13" s="67" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="CW13" s="67" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CX13" s="67" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="CY13" s="67" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="CZ13" s="67" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="DA13" s="67" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="DB13" s="67" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="DC13" s="66" t="s">
         <v>32</v>
@@ -20000,7 +20063,7 @@
         <v>20</v>
       </c>
       <c r="B46" s="58" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C46" s="56" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
Conciliacion estricta 100% con Excel oficial en todas las areas y cache buster v10
</commit_message>
<xml_diff>
--- a/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
+++ b/data/Reporte_Diario_Casetas_y_Cajas_Contratistas_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PCI\Documents\Antigravity\dashboard-imagen-telmex\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C38B4CE6-0CB3-4CB9-801B-E1B4BB647CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82868B7-4B9B-49AD-B83A-F1977A53E5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -364,7 +364,7 @@
     <t>REPORTE DIARIO DE CASETAS Y CAJAS CONTRATISTAS 2026 - IASA / TELMEX</t>
   </si>
   <si>
-    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (28/10/2026, 13:30 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
+    <t>RESUMEN EJECUTIVO CONSOLIDADO AL MOMENTO • Jornada en vivo activa (28/10/2026, 13:34 hrs). Próximo corte oficial hoy a las 10:00 PM.</t>
   </si>
   <si>
     <t>TOTAL CASETAS AL MOMENTO</t>

</xml_diff>